<commit_message>
Actualización automática hashcode vie dic  3 01:11:46 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>59de551a125521c3444790c0661399ae</t>
+    <t>995de0bc8306506ed8cdcf73eb865701</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -536,7 +536,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>dd075c32b83f804ad858b81f767d7141</t>
+    <t>0d6bbaa365734d7d08bb53dde72a97e7</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -593,7 +593,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>c4164dd3c88981d8c135bbe7faeaf0cf</t>
+    <t>3eacd8ac4affa03def23897d1967d1fe</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -839,7 +839,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>501ff54fe1ec0eb156cb3055e62653e8</t>
+    <t>fbe3026801a8a05318e9c6829a33b3fe</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -869,7 +869,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>8f027885c173037131b7c503d2368195</t>
+    <t>f015e1989be6e67e45c04c94b576fb9e</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1505,7 +1505,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>eaa9458a605631a1d065a462c5e5c008</t>
+    <t>fd8005b6571364ab4b65a08e537c60fe</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2453,7 +2453,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>5854519ef399046ca625a71dce515635</t>
+    <t>05328b24a644a1049fed817cced6f182</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2864,7 +2864,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>524aacb4580b4166773e582cb0808dbc</t>
+    <t>97ba8ad7cc67f10abfc35190f825f784</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -2969,7 +2969,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>9908ed097b4574baad512db74f20ff68</t>
+    <t>81fd5b487f4d88146969e31b77720ea2</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3476,7 +3476,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>5b29ef0d3bf73f26c0132e79d57393cb</t>
+    <t>6a39e9e0e0e4c706466d9494df93f046</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3503,7 +3503,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>0dc6f178beadd0b262ab340291e84963</t>
+    <t>d71eea22d9ef4530e74a218236b9560f</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4076,7 +4076,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>84cab191ff25374b88bc173f93d60944</t>
+    <t>e35f2df1dba2149950a3d249f81c0c9a</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4292,7 +4292,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ee1c195c1c2e0f45c3609111d1ac2f34</t>
+    <t>41406fff296e05546707e701b6ddac72</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4307,7 +4307,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>1e2f02d90578b126e9ea63ac2cfcf96b</t>
+    <t>c9c1543a01a0133f5c015bce7e063c68</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb dic  4 01:18:21 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -107,7 +107,7 @@
     <t>915-150012A</t>
   </si>
   <si>
-    <t>09d75f98149a07c4a0583ae9ca10de4d</t>
+    <t>bfb0112f2ae2b24a73ae93e45822355d</t>
   </si>
   <si>
     <t>05-050305TP</t>
@@ -203,7 +203,7 @@
     <t>915-150011A</t>
   </si>
   <si>
-    <t>378ab1f948c4e84c7e2344d013d62a55</t>
+    <t>f63c24810903ed27a1016d346032b0bf</t>
   </si>
   <si>
     <t>05-050316TP</t>
@@ -215,7 +215,7 @@
     <t>915-150018TP</t>
   </si>
   <si>
-    <t>62e8009b0bb43fe17664e9f2373a6c8c</t>
+    <t>cd1debdf85aeee32daf52b7e8ee8951c</t>
   </si>
   <si>
     <t>03-02010301-030102A</t>
@@ -224,7 +224,7 @@
     <t>915-150018TM</t>
   </si>
   <si>
-    <t>39b20a4d3a33d1313cc52833ba6c0bca</t>
+    <t>913e6e600601d0a735fb2df5380c46f9</t>
   </si>
   <si>
     <t>01-010057A</t>
@@ -281,7 +281,7 @@
     <t>915-150018TC</t>
   </si>
   <si>
-    <t>6a8ff615cdb00a46b4e5c0f541ed124b</t>
+    <t>cdb2cc7e869e527db05d1c5b92a430fd</t>
   </si>
   <si>
     <t>915-150007TP</t>
@@ -509,7 +509,7 @@
     <t>01-010076TP</t>
   </si>
   <si>
-    <t>b7d78c63edeadaad65afa9377b208b16</t>
+    <t>8229bda3ea93d7d664acda70705cebcc</t>
   </si>
   <si>
     <t>01-010077A</t>
@@ -1547,7 +1547,7 @@
     <t>915-150011TP</t>
   </si>
   <si>
-    <t>0c26fd91b9125946602969e60614ecb8</t>
+    <t>fa65464b122a0725cddec1011c954d24</t>
   </si>
   <si>
     <t>01-010014TP</t>
@@ -1607,7 +1607,7 @@
     <t>915-150011TC</t>
   </si>
   <si>
-    <t>856b6031b20a0979bfaf8d26d1b23bbe</t>
+    <t>8a65e828cb381b54a5edcc6e8ea43741</t>
   </si>
   <si>
     <t>03-030008TP</t>
@@ -1622,7 +1622,7 @@
     <t>915-150011TM</t>
   </si>
   <si>
-    <t>903bb20630a8ace4e47ca2fd1a725f41</t>
+    <t>763a7db0b0f369a1366432a59e569fca</t>
   </si>
   <si>
     <t>03-030072TP</t>
@@ -2237,7 +2237,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2408,13 +2408,13 @@
     <t>915-150017TP</t>
   </si>
   <si>
-    <t>2882a2cb40dba8d87f6ef93f3dc9b3b3</t>
+    <t>560fdf01660589f6ad7e3fde4430ca1e</t>
   </si>
   <si>
     <t>915-150017TM</t>
   </si>
   <si>
-    <t>ec21d5055c8849c0238a64995935b9ac</t>
+    <t>3abdaa922666a297ebf7f75f6d60bdb3</t>
   </si>
   <si>
     <t>01-010023A</t>
@@ -2477,7 +2477,7 @@
     <t>915-150017TC</t>
   </si>
   <si>
-    <t>466d1df6ad4f7853fa33b6bca722803d</t>
+    <t>d6456b075642a1dc34af12955193ff3d</t>
   </si>
   <si>
     <t>01-010009TC</t>
@@ -3791,7 +3791,7 @@
     <t>915-150002A</t>
   </si>
   <si>
-    <t>74bc5bcce3784988c2080f7367ac96d1</t>
+    <t>69c6545ab4d92f46e37d4e023afa1840</t>
   </si>
   <si>
     <t>03-030054TC</t>
@@ -3935,7 +3935,7 @@
     <t>915-150001A</t>
   </si>
   <si>
-    <t>bbb159c371c7188bcb1da38b8b6d591f</t>
+    <t>88d6ebe35b1aa7b128eb941cd64552e7</t>
   </si>
   <si>
     <t>03-030065TC</t>
@@ -4448,7 +4448,7 @@
     <t>915-150001TP</t>
   </si>
   <si>
-    <t>fb8bdd52c88c645604e93c2f67b8f429</t>
+    <t>65dc4b7cbb93fd4db67f3c1e6e81f370</t>
   </si>
   <si>
     <t>01-010004TP</t>
@@ -4487,7 +4487,7 @@
     <t>915-150001TC</t>
   </si>
   <si>
-    <t>3c8fe25a6d9290e0a1321791ef223075</t>
+    <t>6af94def5a35dca980861eab6a633b73</t>
   </si>
   <si>
     <t>03-02010301-030091A</t>
@@ -4496,7 +4496,7 @@
     <t>915-150001TM</t>
   </si>
   <si>
-    <t>767187267aeb43374fa487d09b04d827</t>
+    <t>00f64d53bb3ffb0cc9a45cfaee7c7c5a</t>
   </si>
   <si>
     <t>03-02010301-030092TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom dic  5 02:44:08 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -659,7 +659,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>8d829c4616cf4b96cdcf731bac392921</t>
+    <t>ac0cc02dfc6891eb373beb0faed137fa</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -1205,7 +1205,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>9b9c5ad6d08999ce87b5a3fb29e233e1</t>
+    <t>029c9af3443af6e2d7b03f1eaac767fa</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1223,7 +1223,7 @@
     <t>05-050009TM</t>
   </si>
   <si>
-    <t>a8a5934b9fbb7f8a3af7943abe7151a7</t>
+    <t>2f64b098590bfe1300dc64b9e618c809</t>
   </si>
   <si>
     <t>03-030077TP</t>
@@ -1235,7 +1235,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>47a95099f630a3c583fbf39b74203835</t>
+    <t>36766d04da50158cf874fadd8ab3c9cf</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1247,7 +1247,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>b49f57b75c313ea891009b54356d4dc7</t>
+    <t>84b310221ab7f505f23bb53c9125572c</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1265,7 +1265,7 @@
     <t>05-050205TC</t>
   </si>
   <si>
-    <t>6ddc9e616f4e07a473378ab68070f8b6</t>
+    <t>70301e041001ac2e12e1e994654fc837</t>
   </si>
   <si>
     <t>04-040014TM</t>
@@ -2546,7 +2546,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>1fae6ea99358972b39c639786ee95090</t>
+    <t>1135cc67d0febc300cf8fe6408c56075</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2771,7 +2771,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>23d15f1cb493200890169d571862b78c</t>
+    <t>7c025acfe1aff88ebe97d77ea60404cf</t>
   </si>
   <si>
     <t>05-050203A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar dic  7 05:20:21 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -65,7 +65,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>c53aca77dd2eb05472af945ce1fab4a0</t>
+    <t>ae2edb3973cf1e6843759d18a536b07b</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -101,7 +101,7 @@
     <t>05-050207TP</t>
   </si>
   <si>
-    <t>be277a350cb68cb239874586d866832c</t>
+    <t>5b6958217855583dcefa6fbb8a5d1dea</t>
   </si>
   <si>
     <t>915-150012A</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>3016d42d9958a4430e511833cbad6fdb</t>
+    <t>bfb30c49ca64e8c049bab0d17d74ed6e</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -152,7 +152,7 @@
     <t>05-050316TC</t>
   </si>
   <si>
-    <t>7174e6b3cf9fa37bacae7ad6c81246c8</t>
+    <t>fa0f5f18dba910c89d0b80fb5803d332</t>
   </si>
   <si>
     <t>03-030059TP</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>cfaa5bf0423f64320f9a9d42bd4cf449</t>
+    <t>2eeb1223d24bfe7bb9567b266512faa3</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -674,7 +674,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>cd850b29b88b6ee555efda7d2e1ed0d8</t>
+    <t>8dae893c68130b652e2fc4451589127b</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -692,7 +692,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>e9e3a3273eaea7f1621c414b75cd8e62</t>
+    <t>6bfd220036718cca09bbde192dc8027e</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -728,7 +728,7 @@
     <t>05-050312TP</t>
   </si>
   <si>
-    <t>0b699f43ea4ee38a8ef5af2190d978db</t>
+    <t>24679fb2e7eecc6f2f6746b4bd2c273f</t>
   </si>
   <si>
     <t>05-0709-070954TC</t>
@@ -743,7 +743,7 @@
     <t>05-050312TC</t>
   </si>
   <si>
-    <t>7cda573046364bdfef778b607b1de319</t>
+    <t>2adcf87b53a93ee95cb2f18d2755a04e</t>
   </si>
   <si>
     <t>03-030055TP</t>
@@ -863,7 +863,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>ec793cf2baa9c1e8e7a640296dc50ce5</t>
+    <t>e746861ff212b1e8c3879cb24487fd1b</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -878,7 +878,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>5296f8a14708031cbb4605357cefad3c</t>
+    <t>ff277090015ad8af73ffc9beed6eb567</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -920,7 +920,7 @@
     <t>05-050203TC</t>
   </si>
   <si>
-    <t>1c233742bac1e1822da8175ed997895e</t>
+    <t>bbbf5898859c5e0f48f9fa4509036ea2</t>
   </si>
   <si>
     <t>01-110304-11030404A</t>
@@ -950,7 +950,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>dab12adcd4ed49832c26769dfc184eee</t>
+    <t>86197b455d35819ac5c2f09ee65e972b</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -977,7 +977,7 @@
     <t>05-050303TC</t>
   </si>
   <si>
-    <t>c8c118d80a2faed223eb06df3af69849</t>
+    <t>a8b9a721c201009e666772885f301378</t>
   </si>
   <si>
     <t>01-010010TP</t>
@@ -995,7 +995,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>bbf014442ec7342f24a53f458de5ad7e</t>
+    <t>33ea6ae7b8c1441462b131b48546db98</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1040,7 +1040,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>2da1fe0de84631b48d3a06e374457a98</t>
+    <t>7405552b523806afe408832fe47359a7</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1082,7 +1082,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>41f45a9006ca64465dcc261596a96597</t>
+    <t>fdf56fc6bec6919ffb9f725b4c26f5cc</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1091,7 +1091,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>99e3a3c99b1a18803949cf311cddee9b</t>
+    <t>a834d057aa9d2ee6297b8ddcd96202f1</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1160,7 +1160,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>3d71c1a01703991aa2e798cd69cc83fd</t>
+    <t>8ed6aa9fa259a9bf72570962dde0a890</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1241,7 +1241,7 @@
     <t>05-050304A</t>
   </si>
   <si>
-    <t>298f515debba9a5401523ba659a476b7</t>
+    <t>67c6bc83096cd2a0d9f9f7b82b142cfe</t>
   </si>
   <si>
     <t>05-050009TP</t>
@@ -1334,7 +1334,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>ea63104c284ba92d83bc28f5d4b4d0fa</t>
+    <t>00dbc0c5da2736bf8c051586c0fe8408</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1493,7 +1493,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>dec5f47ae10b79faf1426a61aa8f8f71</t>
+    <t>fee0bd24848f1864adf96a077414f34b</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1523,7 +1523,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>1ff49cc2cabbac71112c2dd8e1e07df9</t>
+    <t>07c73de9ea680fc89f096e05a99bf931</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1592,7 +1592,7 @@
     <t>05-050310TC</t>
   </si>
   <si>
-    <t>c805972242716513bfadad06ca579d42</t>
+    <t>517085c5ea7869c6e1dab326614576b8</t>
   </si>
   <si>
     <t>04-040004A</t>
@@ -1640,7 +1640,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>e8a4f4a4c128ff1c4f80285ebd76cd83</t>
+    <t>fd94ce3f0d5e7b15293824db7a3fbe97</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1775,7 +1775,7 @@
     <t>05-050005TC</t>
   </si>
   <si>
-    <t>07e7ff1786a3adbf9c279a7e4fbc6815</t>
+    <t>e1c2e69bef2789905ede0dc08a1fbe17</t>
   </si>
   <si>
     <t>04-040018TP</t>
@@ -1796,7 +1796,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>88c2c435c6884dbc5cd8eee399a772bd</t>
+    <t>b5b829b21e375b316eef6c5bc90ee664</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -1820,7 +1820,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>ba89fa237d3c1de83be112506073ffef</t>
+    <t>4fc8fbf16953b0efa4ea25bb66ea5bdd</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2192,7 +2192,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>71eb7d279df1c426c1fd315939e79c4c</t>
+    <t>61fabb2935866b4386bfed27ee03ab1b</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2375,7 +2375,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>6b59dffa6a9d25921f97bf229d443f9f</t>
+    <t>ca492b1cda4660b3f72cbea7e453c4d7</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2447,7 +2447,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>a59190224bf106fc2b4489a4cecd3308</t>
+    <t>a3991196151fb54048cf1a486a90a147</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2558,7 +2558,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>268ccf6c135c07df6ef7a32de07d76ac</t>
+    <t>43f528e33d5498f08856ffb76022adeb</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2639,7 +2639,7 @@
     <t>05-050208TC</t>
   </si>
   <si>
-    <t>40dbccc2a205d1183f72c8ebda232d7f</t>
+    <t>22bb79bb3d1de0fb1737d38153e69a10</t>
   </si>
   <si>
     <t>03-030039A</t>
@@ -2690,7 +2690,7 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>8167a2ba8c125857267cd07e5e751176</t>
+    <t>9394663868f8e4fba4fbb312ddbc5a49</t>
   </si>
   <si>
     <t>05-050208TP</t>
@@ -2720,7 +2720,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>3fb67e4334b5f14ec0e6abda6406aea5</t>
+    <t>13e33513b3bf551b8041b9d1cd22a530</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -2759,13 +2759,13 @@
     <t>05-050317TC</t>
   </si>
   <si>
-    <t>247d2893ef57beb94920af4c3a13268b</t>
+    <t>e128fdd8b36b46efd7e1b8109394f646</t>
   </si>
   <si>
     <t>05-050312A</t>
   </si>
   <si>
-    <t>6838da6c280e0c020cdff659201a38a8</t>
+    <t>fe3ae52593d0a90d67fca0a000914ea8</t>
   </si>
   <si>
     <t>05-050009A</t>
@@ -2777,7 +2777,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>d0635cb66a53dc8f3f496b0b48204ebb</t>
+    <t>820a15d54fea3b90a8778a3bdc8611cc</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>6db229385d7a332619d838a619ce1f0e</t>
+    <t>b1ad9c7d5212e549ae0d6fa675bc7c3b</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -2933,7 +2933,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>d68016c2360cfba9cc7bb1fa05b2fcc8</t>
+    <t>db4211ced69c5787de629a92fa1f3235</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -2951,7 +2951,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>6951d41d22924c7ab8b3bf00c598385c</t>
+    <t>32a933ba7dfc37dbfabe2d0bb333c7e0</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3026,7 +3026,7 @@
     <t>05-050308TC</t>
   </si>
   <si>
-    <t>dcfb9e42e10397fd09d545a4970f1e03</t>
+    <t>1b59b2b46ff8e870b91b0ae1d72250e5</t>
   </si>
   <si>
     <t>02-020002TC</t>
@@ -3044,7 +3044,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>39034531c7e1e066474fb27a4e884d31</t>
+    <t>93f4560ab13a71e4d0fc5fa0131d8372</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3080,7 +3080,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>b7ba5a35fae68f25ce43ece6d5c66757</t>
+    <t>aebd89586fddd665f26812b9ec893442</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3152,7 +3152,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>c6e78183b43f39189efec6685703a997</t>
+    <t>1e3c1e7b10d80841d2d58486399c7acc</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3311,7 +3311,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>273130e8155c20a2a805533d4dc27d6c</t>
+    <t>bbf4e4348b601b8009d0c2a3debb3faa</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3365,7 +3365,7 @@
     <t>05-050204TC</t>
   </si>
   <si>
-    <t>4b37fefbeb61c67215325e4cb59935e5</t>
+    <t>6b6b003fd755901683f7b260cb8bc2b4</t>
   </si>
   <si>
     <t>04-040015TM</t>
@@ -3401,7 +3401,7 @@
     <t>05-050302TC</t>
   </si>
   <si>
-    <t>d7b63d0c5ead8ea370338c4af7bf8d19</t>
+    <t>11c68947622c6f4bbd5c18f2e9b4ffc5</t>
   </si>
   <si>
     <t>01-110304-11030403TP</t>
@@ -3554,7 +3554,7 @@
     <t>05-050317A</t>
   </si>
   <si>
-    <t>60ada143f9042a8d096218e39f0248a2</t>
+    <t>70196355d92fbfc751aa5dd3f011d399</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3620,7 +3620,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>5c55b7bf12ff4456e1b8aedb2f4c8985</t>
+    <t>1153daedcd5e5c64779b88c8be3f1afc</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -3644,7 +3644,7 @@
     <t>05-050206TC</t>
   </si>
   <si>
-    <t>fe3f06501ddafceab9b092665cc20436</t>
+    <t>3f2cac5dbfb4fa7f19e9439cdde0808b</t>
   </si>
   <si>
     <t>04-040013TM</t>
@@ -3728,7 +3728,7 @@
     <t>05-050304TC</t>
   </si>
   <si>
-    <t>22c2b281c13284cc6f284ed199446070</t>
+    <t>890fb26b55b52aab5a33ca149e901aa2</t>
   </si>
   <si>
     <t>03-030043TP</t>
@@ -3740,13 +3740,13 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>46ec2f9ea6517760035a3563ebcad0a2</t>
+    <t>5935597efea1987d25d02cc314439dbc</t>
   </si>
   <si>
     <t>05-050315A</t>
   </si>
   <si>
-    <t>dd9e1c5e0bd7764c6d92dab6d071c342</t>
+    <t>5aa9b78825fa0c958d2e88ab7d76aa0e</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -3809,7 +3809,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>7646562564e2afd2dc47e0c7fdbb92f2</t>
+    <t>f72234d98e438af80575f3814b7c682c</t>
   </si>
   <si>
     <t>04-040002TP</t>
@@ -3857,7 +3857,7 @@
     <t>05-050315TC</t>
   </si>
   <si>
-    <t>5be32278080156c5a60a9623e20d69bc</t>
+    <t>d0bf09101ff51459fcbe3b2e6a964173</t>
   </si>
   <si>
     <t>01-010046TM</t>
@@ -3872,7 +3872,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>cd44ce05963049fb11b16ca8c418e68f</t>
+    <t>7a055ebe965a2a3ebf3e539cf6338802</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -3896,7 +3896,7 @@
     <t>05-050207A</t>
   </si>
   <si>
-    <t>8e89956ea9346583179bddb29fe7a67c</t>
+    <t>9b98347fb1e7fa936f636dae9efd7d48</t>
   </si>
   <si>
     <t>02-020006TM</t>
@@ -3947,7 +3947,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>d47eca90d0b1c581bd5adaebabed648f</t>
+    <t>70c0e3a7a6d3ffa9b39dcb5a65021677</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4019,7 +4019,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>dccb20dfef28d5ed895d63f8f7e04400</t>
+    <t>acaa1861da533e8084aa344c913fb7c6</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4040,7 +4040,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>f18f536e3de80068df632cfe33f3bb03</t>
+    <t>e05063681e631fb6d0a40f56f9c163f9</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4169,7 +4169,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>8a04a9aa62ef3df9bf6a9a7eb767d24e</t>
+    <t>8895992525783d140cb900bc9364090f</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4379,7 +4379,7 @@
     <t>05-050202TC</t>
   </si>
   <si>
-    <t>f9c83da9342f98d4e01c32045e4cd7a5</t>
+    <t>e91e3d6a19f82e1e1f582604d574a0e3</t>
   </si>
   <si>
     <t>03-030062TP</t>
@@ -4397,7 +4397,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>95934d6fd05c3c25aef4d88585311d0c</t>
+    <t>f104ae1611e11d28dbbefdb022ed8f6f</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4424,7 +4424,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>94f8b627ca292ce8f5f6a87cdbae9a88</t>
+    <t>ae8dda6189446dd143ff6f086a604f80</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4523,13 +4523,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>33d9ff0211090157d1fe1c44163c8c81</t>
+    <t>36a3da17cbf41f9a65d168244a1a5d4d</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>97a4b71c619267fbc7a432e40b572498</t>
+    <t>48258eeb88d959a6023137d5ca1859ad</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4559,7 +4559,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>dc081dbe79b68938b1d983e668aeb2a0</t>
+    <t>be40249076493727988f4b67030a2d61</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -4586,7 +4586,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>ca5323dc83c80c367335e59fb001f277</t>
+    <t>2e490268958580f06eeb5e6a1f195d87</t>
   </si>
   <si>
     <t>01-080101-010083A</t>
@@ -4790,7 +4790,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>41db3c4839784cf4d3b168511e209381</t>
+    <t>1d55494e82195a412d2e94419238b09b</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -4925,7 +4925,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>3e9e213a9d032a3e59a0992b563250a8</t>
+    <t>9dadb540c101298c1a677b3e3af4fbfc</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue dic  9 05:34:46 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -182,7 +182,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>9768a0c89cf9a4d0e4eb049cf1e10e50</t>
+    <t>bc193c8dc1cbf7c6c8d3d83225e3f7ad</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -2237,7 +2237,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bf3569543f5afe0bd329968445d710df</t>
+    <t>930e9bd628ccd09c643cd2b4a4b8cfad</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2684,7 +2684,7 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>1f1fee98b33e14a4c767eea7088d4d1a</t>
+    <t>d88a7f73c2a61f13b6f3517661e4d81c</t>
   </si>
   <si>
     <t>05-050311A</t>
@@ -2696,7 +2696,7 @@
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>efbd23f4219cad75c5dcd48237a79503</t>
+    <t>b55dc58d7c18bcb943f97a7db1ea2a2d</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -3374,7 +3374,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>f91da0bd70bc4b36583b401d3391f1a5</t>
+    <t>b7b349184963fec33f5a912c4b687d14</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3548,7 +3548,7 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>03b7accc98cca16374adda1ddc340b24</t>
+    <t>04b228f927f18e2b4a05749735980018</t>
   </si>
   <si>
     <t>05-050317A</t>
@@ -4331,7 +4331,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>8ca78fda18656c861cebf50c49ec0829</t>
+    <t>57bdac694891537d4636637ed2628eee</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue dic 23 04:00:57 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1010,7 +1010,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>7405552b523806afe408832fe47359a7</t>
+    <t>5ea7d2bab0ba454a4e18381dd16bf397</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -2483,7 +2483,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>43f528e33d5498f08856ffb76022adeb</t>
+    <t>a0431bcb4ea3d541395b3dea947b7996</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -4487,7 +4487,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie dic 24 05:50:25 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1010,7 +1010,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>5ea7d2bab0ba454a4e18381dd16bf397</t>
+    <t>7405552b523806afe408832fe47359a7</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -2483,7 +2483,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>a0431bcb4ea3d541395b3dea947b7996</t>
+    <t>43f528e33d5498f08856ffb76022adeb</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -4487,7 +4487,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb dic 25 04:38:09 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1010,7 +1010,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>7405552b523806afe408832fe47359a7</t>
+    <t>5ea7d2bab0ba454a4e18381dd16bf397</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -2168,7 +2168,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>0841f66eec1f7caf51680bed6f5054c6</t>
+    <t>bf3569543f5afe0bd329968445d710df</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2483,7 +2483,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>43f528e33d5498f08856ffb76022adeb</t>
+    <t>a0431bcb4ea3d541395b3dea947b7996</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -4487,7 +4487,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode lun dic 27 05:47:43 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1010,7 +1010,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>5ea7d2bab0ba454a4e18381dd16bf397</t>
+    <t>7405552b523806afe408832fe47359a7</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -2483,7 +2483,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>a0431bcb4ea3d541395b3dea947b7996</t>
+    <t>43f528e33d5498f08856ffb76022adeb</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -4487,7 +4487,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>d878f735a89572d2273c1e98708e28dd</t>
+    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar dic 28 05:51:44 CET 2021
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1010,7 +1010,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>7405552b523806afe408832fe47359a7</t>
+    <t>5ea7d2bab0ba454a4e18381dd16bf397</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -2483,7 +2483,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>43f528e33d5498f08856ffb76022adeb</t>
+    <t>a0431bcb4ea3d541395b3dea947b7996</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -4487,7 +4487,7 @@
     <t>03-030032A</t>
   </si>
   <si>
-    <t>c9c849f03081bb7a17b5eba5feebb7ea</t>
+    <t>d878f735a89572d2273c1e98708e28dd</t>
   </si>
   <si>
     <t>03-030060TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ene  5 00:43:47 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>995de0bc8306506ed8cdcf73eb865701</t>
+    <t>cd53cfda870d675a46aabb75dabac73a</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>3d9668f76ab02d8653e771c2bd737343</t>
+    <t>670ca03d45ae4deda6759bd69228f3b3</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -257,7 +257,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>edda8808bba8e01d90bf48cc890a10be</t>
+    <t>350695fbc57b4bf9ac73e53d7a194efb</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -512,7 +512,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>ffe325fb0a0ee1475fb57fd474a12779</t>
+    <t>f98d3adbdb8efe4d62c7e451ac498e86</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -569,7 +569,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>0d6bbaa365734d7d08bb53dde72a97e7</t>
+    <t>a4b297bff48ec3af836197508aa01004</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -629,7 +629,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>3eacd8ac4affa03def23897d1967d1fe</t>
+    <t>dcae650ff0198395db522f5051a0284b</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -695,7 +695,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>ac0cc02dfc6891eb373beb0faed137fa</t>
+    <t>71a1f5c9a268dd4b1a78437b5f3f1529</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -710,7 +710,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>8dae893c68130b652e2fc4451589127b</t>
+    <t>e1a60b47eb63df3e46d47eb115527ddf</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -875,7 +875,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>fbe3026801a8a05318e9c6829a33b3fe</t>
+    <t>98b160b051be064e950e52b80e8dc6b3</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -905,13 +905,13 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>f015e1989be6e67e45c04c94b576fb9e</t>
+    <t>61f17683d4c301c375f58e5378f7b14b</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>572fc15cff189afe97fe8de246984e47</t>
+    <t>b4d1d6178ed057f8704efcc925066d96</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -959,7 +959,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>6adcfd9be178806ed34169491b6d435a</t>
+    <t>3d76bb078691f3f726ac08246a586095</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1559,7 +1559,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>fd8005b6571364ab4b65a08e537c60fe</t>
+    <t>25e1d7e4e8683c11ece1258ab20b16cf</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2597,7 +2597,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>05328b24a644a1049fed817cced6f182</t>
+    <t>685f55b15b443677a46e3f69c9ba39e9</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2996,7 +2996,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>57ed2a7a3239d7fc1bc06d16e7e25fac</t>
+    <t>fe906ff07e924136c15856e381920b5d</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3095,7 +3095,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>81fd5b487f4d88146969e31b77720ea2</t>
+    <t>f705fc37721472d6922066ff097ddc0f</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3518,7 +3518,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>ad51d2c54edaaf35938b2e40b60f64bb</t>
+    <t>a2b130461b47507481be660abd69a562</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3623,7 +3623,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>6a39e9e0e0e4c706466d9494df93f046</t>
+    <t>c08eadd331bc741a5bfd021e85679e74</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3659,7 +3659,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>d71eea22d9ef4530e74a218236b9560f</t>
+    <t>5772807470bdf084e92a5abdcb5d8620</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4271,7 +4271,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>e35f2df1dba2149950a3d249f81c0c9a</t>
+    <t>48cb46d049a291907c4ab613e1a8486b</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4538,7 +4538,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>c9c1543a01a0133f5c015bce7e063c68</t>
+    <t>24277b83c8f1dd7c586e267ca7294b09</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4547,7 +4547,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>984c72c7a220374fb50717d7e0ff435c</t>
+    <t>4b454b3abd94b34d6df03880c46c21d6</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4610,7 +4610,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>be294fd3215f7afe40acfee87d69d3bd</t>
+    <t>30723e4128085a331f4b551db59153a0</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4808,7 +4808,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>be40249076493727988f4b67030a2d61</t>
+    <t>7cdbf5f1d177f00789b80583f45d2eb4</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie ene  7 00:38:07 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="1790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="1791">
   <si>
     <t>05-050305TM</t>
   </si>
@@ -5312,6 +5312,9 @@
     <t>03-030016TC</t>
   </si>
   <si>
+    <t>25186f157230b906b841ea45772fc542</t>
+  </si>
+  <si>
     <t>915-150005TM</t>
   </si>
   <si>
@@ -5345,7 +5348,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>
@@ -13338,103 +13341,103 @@
         <v>1765</v>
       </c>
       <c r="B990" t="s">
-        <v>1</v>
+        <v>1766</v>
       </c>
     </row>
     <row r="991">
       <c r="A991" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="B991" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
     </row>
     <row r="992">
       <c r="A992" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="B992" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
     </row>
     <row r="993">
       <c r="A993" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="B993" t="s">
-        <v>1771</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="B994" t="s">
-        <v>1773</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="995">
       <c r="A995" t="s">
-        <v>1774</v>
+        <v>1775</v>
       </c>
       <c r="B995" t="s">
-        <v>1775</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="996">
       <c r="A996" t="s">
-        <v>1776</v>
+        <v>1777</v>
       </c>
       <c r="B996" t="s">
-        <v>1777</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="997">
       <c r="A997" t="s">
-        <v>1778</v>
+        <v>1779</v>
       </c>
       <c r="B997" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="998">
       <c r="A998" t="s">
-        <v>1780</v>
+        <v>1781</v>
       </c>
       <c r="B998" t="s">
-        <v>1781</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="999">
       <c r="A999" t="s">
-        <v>1782</v>
+        <v>1783</v>
       </c>
       <c r="B999" t="s">
-        <v>1783</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="1000">
       <c r="A1000" t="s">
-        <v>1784</v>
+        <v>1785</v>
       </c>
       <c r="B1000" t="s">
-        <v>1785</v>
+        <v>1786</v>
       </c>
     </row>
     <row r="1001">
       <c r="A1001" t="s">
-        <v>1786</v>
+        <v>1787</v>
       </c>
       <c r="B1001" t="s">
-        <v>1787</v>
+        <v>1788</v>
       </c>
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>1788</v>
+        <v>1789</v>
       </c>
       <c r="B1002" t="s">
-        <v>1789</v>
+        <v>1790</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática hashcode jue ene 13 00:40:20 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -329,7 +329,7 @@
     <t>05-0709-070908TM</t>
   </si>
   <si>
-    <t>67b7c9f494638cfa165a2cb3d182fc27</t>
+    <t>c53912c4f70059faec7c26b975513572</t>
   </si>
   <si>
     <t>03-030026A</t>
@@ -413,7 +413,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -443,7 +443,7 @@
     <t>03-030001A</t>
   </si>
   <si>
-    <t>e9080851709b95373d75ab3d52b1eed3</t>
+    <t>2aa1d70e294d3f855869abded550101b</t>
   </si>
   <si>
     <t>05-050307TP</t>
@@ -1112,7 +1112,7 @@
     <t>05-0709-070910TM</t>
   </si>
   <si>
-    <t>c7b13c896d79f110af279a23b4fc0266</t>
+    <t>37918519eb60a7bf23f132633a7d14a4</t>
   </si>
   <si>
     <t>01-010045TP</t>
@@ -1988,7 +1988,7 @@
     <t>02-020001TC</t>
   </si>
   <si>
-    <t>4636fa3c864dee87fac88ac66181bc59</t>
+    <t>c09f637a916343cbf944a5182b0ea660</t>
   </si>
   <si>
     <t>01-010016TP</t>
@@ -2018,7 +2018,7 @@
     <t>05-0709-070906ATM</t>
   </si>
   <si>
-    <t>c28618037e25e3704c441d1b6fd012db</t>
+    <t>2d369adbe7742a8e45f327b8cad9e929</t>
   </si>
   <si>
     <t>03-030070TC</t>
@@ -2111,7 +2111,7 @@
     <t>02-020001TM</t>
   </si>
   <si>
-    <t>89657a663624e3a569608d88c8a300b4</t>
+    <t>da5b87f6d7969e339097a5ee6c3c04ad</t>
   </si>
   <si>
     <t>01-080101-010084TP</t>
@@ -2141,7 +2141,7 @@
     <t>02-020001TP</t>
   </si>
   <si>
-    <t>1d2a0fad47aed368e039d0d34410fcec</t>
+    <t>1df16c9e277baf30a157cee4dca37275</t>
   </si>
   <si>
     <t>03-02010301-030091TC</t>
@@ -2207,7 +2207,7 @@
     <t>05-0709-070904TM</t>
   </si>
   <si>
-    <t>70f3101ce53b40825777f574a3f672eb</t>
+    <t>6c323504e32ff72973787c25c3d37b39</t>
   </si>
   <si>
     <t>01-010029TP</t>
@@ -2759,7 +2759,7 @@
     <t>03-030001TC</t>
   </si>
   <si>
-    <t>ac5faa7b24db5e3a4281517c9b86466e</t>
+    <t>d1020ec2c5dafea497bf49ab17c149e7</t>
   </si>
   <si>
     <t>03-030047TC</t>
@@ -3197,7 +3197,7 @@
     <t>03-030001TM</t>
   </si>
   <si>
-    <t>2f7eb22ff6ad0ca3d69e86974d03036b</t>
+    <t>040783e3155e41ea714a9b89a3277a28</t>
   </si>
   <si>
     <t>05-050308TC</t>
@@ -3224,7 +3224,7 @@
     <t>03-030001TP</t>
   </si>
   <si>
-    <t>ce67bdb572db24e4f6a2a30199fbe017</t>
+    <t>7aa025559d8c2585f33a4b2adc895bc1</t>
   </si>
   <si>
     <t>03-030047TM</t>
@@ -4631,7 +4631,7 @@
     <t>05-0709-070903TM</t>
   </si>
   <si>
-    <t>b4e3ba5466c57f698549f42028666b21</t>
+    <t>28b70e4534ed83807931652c2220affe</t>
   </si>
   <si>
     <t>03-02010301-030093A</t>
@@ -5021,7 +5021,7 @@
     <t>05-0709-070906BTM</t>
   </si>
   <si>
-    <t>f3901ef3ea3a05be9304ed56a37b3c83</t>
+    <t>6aa92ec1cba9be4e7479307cf069897a</t>
   </si>
   <si>
     <t>03-030071TC</t>
@@ -5426,7 +5426,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb ene 15 00:38:31 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -413,7 +413,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5438,7 +5438,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ene 19 00:41:50 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -278,7 +278,7 @@
     <t>915-150007TP</t>
   </si>
   <si>
-    <t>5cc5588682a773ee40685b0368545bba</t>
+    <t>c00525d91f07419c652b72675aa7c2e3</t>
   </si>
   <si>
     <t>01-010063TP</t>
@@ -296,7 +296,7 @@
     <t>915-150007TM</t>
   </si>
   <si>
-    <t>65727ea8774885793521081e4dc28868</t>
+    <t>b5c92b099200035da492990e7bac5b2e</t>
   </si>
   <si>
     <t>01-010063TM</t>
@@ -359,7 +359,7 @@
     <t>915-150007TC</t>
   </si>
   <si>
-    <t>14e93851982552fbf4a080c740dbc08b</t>
+    <t>2f5ab210326d83638a983c45e222f843</t>
   </si>
   <si>
     <t>04-040012TP</t>
@@ -608,7 +608,7 @@
     <t>915-150009TM</t>
   </si>
   <si>
-    <t>2e8e66efc2c79c1af81ca0fd730f6485</t>
+    <t>f54b3893d0b6eb7a20cbd10b9c5398e7</t>
   </si>
   <si>
     <t>01-010065TM</t>
@@ -635,7 +635,7 @@
     <t>915-150009TP</t>
   </si>
   <si>
-    <t>b66a4c66387af9396b42655b20102187</t>
+    <t>fbc4e65c774b910b62ca8c9bcb59fa62</t>
   </si>
   <si>
     <t>04-040021TC</t>
@@ -665,7 +665,7 @@
     <t>915-150009TC</t>
   </si>
   <si>
-    <t>b1f662bbaef438759549555e3b484cf1</t>
+    <t>791cd19d5aedf64fc7036d9072e3e054</t>
   </si>
   <si>
     <t>04-040010TP</t>
@@ -3020,7 +3020,7 @@
     <t>915-150008TM</t>
   </si>
   <si>
-    <t>21c05167a0b2146c2f55c788698399b7</t>
+    <t>ea1d674cd8ce2353be0588c06ebde8ed</t>
   </si>
   <si>
     <t>01-010064TM</t>
@@ -3065,7 +3065,7 @@
     <t>915-150008TP</t>
   </si>
   <si>
-    <t>2525de1c783d8988b4f38769345fd54f</t>
+    <t>13b9c404af9d3d1ec3e888d8d0c85ba8</t>
   </si>
   <si>
     <t>01-010075TC</t>
@@ -3101,7 +3101,7 @@
     <t>915-150008TC</t>
   </si>
   <si>
-    <t>348c9ced201772447720ae14cce4865c</t>
+    <t>96c1ef81f682e441cd5ea225800b4153</t>
   </si>
   <si>
     <t>03-02010301-030100TC</t>
@@ -3419,7 +3419,7 @@
     <t>915-150007A</t>
   </si>
   <si>
-    <t>8bf4d4b70def7c3e1618c64e37847534</t>
+    <t>ffa1e7c8a9a56ee682110383762fcbb8</t>
   </si>
   <si>
     <t>05-050204TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom ene 23 00:43:46 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="1782">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="1783">
   <si>
     <t>05-050305TM</t>
   </si>
@@ -3183,6 +3183,9 @@
   </si>
   <si>
     <t>05-050308TP</t>
+  </si>
+  <si>
+    <t>7ec0dab31e5ce420d67791fb1c92097a</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -10186,44 +10189,44 @@
         <v>1056</v>
       </c>
       <c r="B599" t="s">
-        <v>1</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="600">
       <c r="A600" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B600" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="B601" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="602">
       <c r="A602" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="B602" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="603">
       <c r="A603" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="B603" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="604">
       <c r="A604" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="B604" t="s">
         <v>1</v>
@@ -10231,31 +10234,31 @@
     </row>
     <row r="605">
       <c r="A605" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="B605" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="B606" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="B607" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="608">
       <c r="A608" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="B608" t="s">
         <v>1</v>
@@ -10263,23 +10266,23 @@
     </row>
     <row r="609">
       <c r="A609" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="B609" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="B610" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="B611" t="s">
         <v>1</v>
@@ -10287,87 +10290,87 @@
     </row>
     <row r="612">
       <c r="A612" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="B612" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="613">
       <c r="A613" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="B613" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B614" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="615">
       <c r="A615" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="B615" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="616">
       <c r="A616" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B616" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="617">
       <c r="A617" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="B617" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="618">
       <c r="A618" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="B618" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="B619" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="620">
       <c r="A620" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="B620" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="B621" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="B622" t="s">
         <v>1</v>
@@ -10375,103 +10378,103 @@
     </row>
     <row r="623">
       <c r="A623" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="B623" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="B624" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="B625" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="626">
       <c r="A626" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="B626" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="627">
       <c r="A627" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B627" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B628" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="629">
       <c r="A629" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="B629" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="B630" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="631">
       <c r="A631" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="B631" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="632">
       <c r="A632" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B632" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="633">
       <c r="A633" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="B633" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="B634" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="B635" t="s">
         <v>1</v>
@@ -10479,31 +10482,31 @@
     </row>
     <row r="636">
       <c r="A636" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B636" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="B637" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="B638" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="B639" t="s">
         <v>1</v>
@@ -10511,23 +10514,23 @@
     </row>
     <row r="640">
       <c r="A640" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="B640" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="B641" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="B642" t="s">
         <v>1</v>
@@ -10535,7 +10538,7 @@
     </row>
     <row r="643">
       <c r="A643" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B643" t="s">
         <v>1</v>
@@ -10543,15 +10546,15 @@
     </row>
     <row r="644">
       <c r="A644" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="B644" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B645" t="s">
         <v>1</v>
@@ -10559,39 +10562,39 @@
     </row>
     <row r="646">
       <c r="A646" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="B646" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B647" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="B648" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="B649" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="650">
       <c r="A650" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="B650" t="s">
         <v>1</v>
@@ -10599,39 +10602,39 @@
     </row>
     <row r="651">
       <c r="A651" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="B651" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="B652" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B653" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="654">
       <c r="A654" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="B654" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="655">
       <c r="A655" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="B655" t="s">
         <v>1</v>
@@ -10639,39 +10642,39 @@
     </row>
     <row r="656">
       <c r="A656" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="B656" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="657">
       <c r="A657" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="B657" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="B658" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="659">
       <c r="A659" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="B659" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="660">
       <c r="A660" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="B660" t="s">
         <v>1</v>
@@ -10679,23 +10682,23 @@
     </row>
     <row r="661">
       <c r="A661" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="B661" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="662">
       <c r="A662" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="B662" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="663">
       <c r="A663" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="B663" t="s">
         <v>1</v>
@@ -10703,7 +10706,7 @@
     </row>
     <row r="664">
       <c r="A664" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="B664" t="s">
         <v>1</v>
@@ -10711,31 +10714,31 @@
     </row>
     <row r="665">
       <c r="A665" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="B665" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="666">
       <c r="A666" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="B666" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="667">
       <c r="A667" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="B667" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="668">
       <c r="A668" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="B668" t="s">
         <v>1</v>
@@ -10743,31 +10746,31 @@
     </row>
     <row r="669">
       <c r="A669" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B669" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="670">
       <c r="A670" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="B670" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="671">
       <c r="A671" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="B671" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="672">
       <c r="A672" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="B672" t="s">
         <v>1</v>
@@ -10775,103 +10778,103 @@
     </row>
     <row r="673">
       <c r="A673" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="B673" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="674">
       <c r="A674" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="B674" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="675">
       <c r="A675" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="B675" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="676">
       <c r="A676" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="B676" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="677">
       <c r="A677" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="B677" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="678">
       <c r="A678" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="B678" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="679">
       <c r="A679" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="B679" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="680">
       <c r="A680" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="B680" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="681">
       <c r="A681" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="B681" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="682">
       <c r="A682" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="B682" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="683">
       <c r="A683" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="B683" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="684">
       <c r="A684" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="B684" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="685">
       <c r="A685" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="B685" t="s">
         <v>1</v>
@@ -10879,39 +10882,39 @@
     </row>
     <row r="686">
       <c r="A686" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="B686" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="687">
       <c r="A687" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="B687" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="688">
       <c r="A688" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="B688" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="689">
       <c r="A689" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="B689" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="690">
       <c r="A690" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="B690" t="s">
         <v>1</v>
@@ -10919,23 +10922,23 @@
     </row>
     <row r="691">
       <c r="A691" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="B691" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="692">
       <c r="A692" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="B692" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="693">
       <c r="A693" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="B693" t="s">
         <v>1</v>
@@ -10943,7 +10946,7 @@
     </row>
     <row r="694">
       <c r="A694" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="B694" t="s">
         <v>1</v>
@@ -10951,111 +10954,111 @@
     </row>
     <row r="695">
       <c r="A695" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="B695" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="696">
       <c r="A696" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="B696" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="697">
       <c r="A697" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="B697" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="698">
       <c r="A698" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="B698" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="699">
       <c r="A699" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="B699" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="700">
       <c r="A700" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="B700" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="701">
       <c r="A701" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="B701" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="702">
       <c r="A702" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="B702" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="703">
       <c r="A703" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="B703" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="704">
       <c r="A704" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="B704" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="705">
       <c r="A705" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="B705" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="706">
       <c r="A706" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="B706" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="707">
       <c r="A707" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="B707" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="708">
       <c r="A708" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="B708" t="s">
         <v>1</v>
@@ -11063,31 +11066,31 @@
     </row>
     <row r="709">
       <c r="A709" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="B709" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="710">
       <c r="A710" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="B710" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="711">
       <c r="A711" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="B711" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="712">
       <c r="A712" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="B712" t="s">
         <v>1</v>
@@ -11095,15 +11098,15 @@
     </row>
     <row r="713">
       <c r="A713" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="B713" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="714">
       <c r="A714" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="B714" t="s">
         <v>1</v>
@@ -11111,47 +11114,47 @@
     </row>
     <row r="715">
       <c r="A715" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="B715" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="716">
       <c r="A716" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="B716" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="717">
       <c r="A717" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="B717" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="718">
       <c r="A718" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="B718" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="719">
       <c r="A719" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="B719" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="720">
       <c r="A720" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="B720" t="s">
         <v>1</v>
@@ -11159,7 +11162,7 @@
     </row>
     <row r="721">
       <c r="A721" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="B721" t="s">
         <v>1</v>
@@ -11167,31 +11170,31 @@
     </row>
     <row r="722">
       <c r="A722" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="B722" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="723">
       <c r="A723" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="B723" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="724">
       <c r="A724" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="B724" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="725">
       <c r="A725" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="B725" t="s">
         <v>1</v>
@@ -11199,39 +11202,39 @@
     </row>
     <row r="726">
       <c r="A726" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="B726" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="727">
       <c r="A727" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="B727" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="728">
       <c r="A728" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="B728" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="729">
       <c r="A729" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="B729" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="730">
       <c r="A730" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="B730" t="s">
         <v>1</v>
@@ -11239,23 +11242,23 @@
     </row>
     <row r="731">
       <c r="A731" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="B731" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="732">
       <c r="A732" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="B732" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="733">
       <c r="A733" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="B733" t="s">
         <v>1</v>
@@ -11263,7 +11266,7 @@
     </row>
     <row r="734">
       <c r="A734" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="B734" t="s">
         <v>1</v>
@@ -11271,7 +11274,7 @@
     </row>
     <row r="735">
       <c r="A735" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="B735" t="s">
         <v>1</v>
@@ -11279,47 +11282,47 @@
     </row>
     <row r="736">
       <c r="A736" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="B736" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="737">
       <c r="A737" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="B737" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="738">
       <c r="A738" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="B738" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="739">
       <c r="A739" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="B739" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="740">
       <c r="A740" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="B740" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="741">
       <c r="A741" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="B741" t="s">
         <v>1</v>
@@ -11327,31 +11330,31 @@
     </row>
     <row r="742">
       <c r="A742" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B742" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="743">
       <c r="A743" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="B743" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="744">
       <c r="A744" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="B744" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="745">
       <c r="A745" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="B745" t="s">
         <v>1</v>
@@ -11359,7 +11362,7 @@
     </row>
     <row r="746">
       <c r="A746" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="B746" t="s">
         <v>1</v>
@@ -11367,55 +11370,55 @@
     </row>
     <row r="747">
       <c r="A747" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="B747" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="748">
       <c r="A748" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="B748" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="749">
       <c r="A749" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="B749" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="750">
       <c r="A750" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="B750" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="751">
       <c r="A751" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="B751" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="752">
       <c r="A752" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="B752" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="753">
       <c r="A753" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="B753" t="s">
         <v>1</v>
@@ -11423,23 +11426,23 @@
     </row>
     <row r="754">
       <c r="A754" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="B754" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="755">
       <c r="A755" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="B755" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="756">
       <c r="A756" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="B756" t="s">
         <v>1</v>
@@ -11447,23 +11450,23 @@
     </row>
     <row r="757">
       <c r="A757" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="B757" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="758">
       <c r="A758" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="B758" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="759">
       <c r="A759" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="B759" t="s">
         <v>1</v>
@@ -11471,7 +11474,7 @@
     </row>
     <row r="760">
       <c r="A760" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B760" t="s">
         <v>1</v>
@@ -11479,23 +11482,23 @@
     </row>
     <row r="761">
       <c r="A761" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="B761" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="762">
       <c r="A762" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="B762" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="763">
       <c r="A763" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B763" t="s">
         <v>1</v>
@@ -11503,15 +11506,15 @@
     </row>
     <row r="764">
       <c r="A764" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="B764" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="765">
       <c r="A765" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="B765" t="s">
         <v>1</v>
@@ -11519,55 +11522,55 @@
     </row>
     <row r="766">
       <c r="A766" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="B766" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="767">
       <c r="A767" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="B767" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="768">
       <c r="A768" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="B768" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="769">
       <c r="A769" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="B769" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="770">
       <c r="A770" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="B770" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="771">
       <c r="A771" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="B771" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="772">
       <c r="A772" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="B772" t="s">
         <v>1</v>
@@ -11575,55 +11578,55 @@
     </row>
     <row r="773">
       <c r="A773" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="B773" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="774">
       <c r="A774" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="B774" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="775">
       <c r="A775" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="B775" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="776">
       <c r="A776" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="B776" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="777">
       <c r="A777" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="B777" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="778">
       <c r="A778" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="B778" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="779">
       <c r="A779" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="B779" t="s">
         <v>1</v>
@@ -11631,55 +11634,55 @@
     </row>
     <row r="780">
       <c r="A780" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="B780" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="781">
       <c r="A781" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="B781" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="782">
       <c r="A782" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="B782" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="783">
       <c r="A783" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="B783" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="784">
       <c r="A784" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="B784" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="785">
       <c r="A785" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
       <c r="B785" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="786">
       <c r="A786" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="B786" t="s">
         <v>1</v>
@@ -11687,15 +11690,15 @@
     </row>
     <row r="787">
       <c r="A787" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="B787" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="788">
       <c r="A788" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="B788" t="s">
         <v>1</v>
@@ -11703,31 +11706,31 @@
     </row>
     <row r="789">
       <c r="A789" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
       <c r="B789" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="790">
       <c r="A790" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="B790" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="791">
       <c r="A791" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="B791" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="792">
       <c r="A792" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="B792" t="s">
         <v>1</v>
@@ -11735,7 +11738,7 @@
     </row>
     <row r="793">
       <c r="A793" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="B793" t="s">
         <v>1</v>
@@ -11743,191 +11746,191 @@
     </row>
     <row r="794">
       <c r="A794" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="B794" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="795">
       <c r="A795" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="B795" t="s">
-        <v>1403</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="796">
       <c r="A796" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="B796" t="s">
-        <v>1405</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="797">
       <c r="A797" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="B797" t="s">
-        <v>1407</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="798">
       <c r="A798" t="s">
-        <v>1408</v>
+        <v>1409</v>
       </c>
       <c r="B798" t="s">
-        <v>1409</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="799">
       <c r="A799" t="s">
-        <v>1410</v>
+        <v>1411</v>
       </c>
       <c r="B799" t="s">
-        <v>1411</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="800">
       <c r="A800" t="s">
-        <v>1412</v>
+        <v>1413</v>
       </c>
       <c r="B800" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="801">
       <c r="A801" t="s">
-        <v>1414</v>
+        <v>1415</v>
       </c>
       <c r="B801" t="s">
-        <v>1415</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="802">
       <c r="A802" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
       <c r="B802" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="803">
       <c r="A803" t="s">
-        <v>1418</v>
+        <v>1419</v>
       </c>
       <c r="B803" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="804">
       <c r="A804" t="s">
-        <v>1420</v>
+        <v>1421</v>
       </c>
       <c r="B804" t="s">
-        <v>1421</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="805">
       <c r="A805" t="s">
-        <v>1422</v>
+        <v>1423</v>
       </c>
       <c r="B805" t="s">
-        <v>1423</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="806">
       <c r="A806" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="B806" t="s">
-        <v>1425</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="807">
       <c r="A807" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B807" t="s">
-        <v>1427</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="808">
       <c r="A808" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="B808" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="809">
       <c r="A809" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="B809" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="810">
       <c r="A810" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="B810" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="811">
       <c r="A811" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
       <c r="B811" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="812">
       <c r="A812" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="B812" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
     </row>
     <row r="813">
       <c r="A813" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="B813" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="814">
       <c r="A814" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
       <c r="B814" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="815">
       <c r="A815" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="B815" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="816">
       <c r="A816" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="B816" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="817">
       <c r="A817" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="B817" t="s">
         <v>1</v>
@@ -11935,135 +11938,135 @@
     </row>
     <row r="818">
       <c r="A818" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="B818" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="B819" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="820">
       <c r="A820" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="B820" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="821">
       <c r="A821" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="B821" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="822">
       <c r="A822" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="B822" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="823">
       <c r="A823" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="B823" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="824">
       <c r="A824" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
       <c r="B824" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
     </row>
     <row r="825">
       <c r="A825" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
       <c r="B825" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="826">
       <c r="A826" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="B826" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="827">
       <c r="A827" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="B827" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="828">
       <c r="A828" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="B828" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="829">
       <c r="A829" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
       <c r="B829" t="s">
-        <v>1470</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="830">
       <c r="A830" t="s">
-        <v>1471</v>
+        <v>1472</v>
       </c>
       <c r="B830" t="s">
-        <v>1472</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="831">
       <c r="A831" t="s">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="B831" t="s">
-        <v>1474</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="s">
-        <v>1475</v>
+        <v>1476</v>
       </c>
       <c r="B832" t="s">
-        <v>1476</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="833">
       <c r="A833" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="B833" t="s">
-        <v>1478</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="834">
       <c r="A834" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="B834" t="s">
         <v>1</v>
@@ -12071,15 +12074,15 @@
     </row>
     <row r="835">
       <c r="A835" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
       <c r="B835" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="836">
       <c r="A836" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="B836" t="s">
         <v>1</v>
@@ -12087,15 +12090,15 @@
     </row>
     <row r="837">
       <c r="A837" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
       <c r="B837" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
     </row>
     <row r="838">
       <c r="A838" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="B838" t="s">
         <v>1</v>
@@ -12103,7 +12106,7 @@
     </row>
     <row r="839">
       <c r="A839" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="B839" t="s">
         <v>1</v>
@@ -12111,23 +12114,23 @@
     </row>
     <row r="840">
       <c r="A840" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
       <c r="B840" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="841">
       <c r="A841" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
       <c r="B841" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="842">
       <c r="A842" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
       <c r="B842" t="s">
         <v>1</v>
@@ -12135,39 +12138,39 @@
     </row>
     <row r="843">
       <c r="A843" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
       <c r="B843" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="844">
       <c r="A844" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
       <c r="B844" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="845">
       <c r="A845" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
       <c r="B845" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="846">
       <c r="A846" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
       <c r="B846" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="847">
       <c r="A847" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="B847" t="s">
         <v>1</v>
@@ -12175,31 +12178,31 @@
     </row>
     <row r="848">
       <c r="A848" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
       <c r="B848" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="849">
       <c r="A849" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="B849" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="850">
       <c r="A850" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
       <c r="B850" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="851">
       <c r="A851" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
       <c r="B851" t="s">
         <v>1</v>
@@ -12207,23 +12210,23 @@
     </row>
     <row r="852">
       <c r="A852" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="B852" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="853">
       <c r="A853" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="B853" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="854">
       <c r="A854" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="B854" t="s">
         <v>1</v>
@@ -12231,31 +12234,31 @@
     </row>
     <row r="855">
       <c r="A855" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="B855" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="856">
       <c r="A856" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="B856" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
     </row>
     <row r="857">
       <c r="A857" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="B857" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="858">
       <c r="A858" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="B858" t="s">
         <v>1</v>
@@ -12263,23 +12266,23 @@
     </row>
     <row r="859">
       <c r="A859" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="B859" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="B860" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="861">
       <c r="A861" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="B861" t="s">
         <v>1</v>
@@ -12287,23 +12290,23 @@
     </row>
     <row r="862">
       <c r="A862" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
       <c r="B862" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="B863" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="B864" t="s">
         <v>1</v>
@@ -12311,39 +12314,39 @@
     </row>
     <row r="865">
       <c r="A865" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
       <c r="B865" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="866">
       <c r="A866" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="B866" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="867">
       <c r="A867" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
       <c r="B867" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="868">
       <c r="A868" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
       <c r="B868" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="869">
       <c r="A869" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
       <c r="B869" t="s">
         <v>1</v>
@@ -12351,127 +12354,127 @@
     </row>
     <row r="870">
       <c r="A870" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="B870" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="871">
       <c r="A871" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="B871" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="872">
       <c r="A872" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="B872" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="873">
       <c r="A873" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="B873" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="874">
       <c r="A874" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="B874" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="875">
       <c r="A875" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="B875" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="876">
       <c r="A876" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="B876" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="877">
       <c r="A877" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="B877" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="878">
       <c r="A878" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="B878" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="879">
       <c r="A879" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="B879" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="880">
       <c r="A880" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="B880" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="881">
       <c r="A881" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="B881" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="882">
       <c r="A882" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="B882" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="883">
       <c r="A883" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="B883" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="884">
       <c r="A884" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="B884" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="B885" t="s">
         <v>1</v>
@@ -12479,23 +12482,23 @@
     </row>
     <row r="886">
       <c r="A886" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="B886" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="887">
       <c r="A887" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="B887" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="888">
       <c r="A888" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="B888" t="s">
         <v>1</v>
@@ -12503,7 +12506,7 @@
     </row>
     <row r="889">
       <c r="A889" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="B889" t="s">
         <v>1</v>
@@ -12511,63 +12514,63 @@
     </row>
     <row r="890">
       <c r="A890" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
       <c r="B890" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
     </row>
     <row r="891">
       <c r="A891" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="B891" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="892">
       <c r="A892" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="B892" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="893">
       <c r="A893" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="B893" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="894">
       <c r="A894" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="B894" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
     </row>
     <row r="895">
       <c r="A895" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="B895" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="896">
       <c r="A896" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="B896" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="897">
       <c r="A897" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="B897" t="s">
         <v>1</v>
@@ -12575,47 +12578,47 @@
     </row>
     <row r="898">
       <c r="A898" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="B898" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="899">
       <c r="A899" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="B899" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="900">
       <c r="A900" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="B900" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="901">
       <c r="A901" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="B901" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="902">
       <c r="A902" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="B902" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="903">
       <c r="A903" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="B903" t="s">
         <v>1</v>
@@ -12623,79 +12626,79 @@
     </row>
     <row r="904">
       <c r="A904" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="B904" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="905">
       <c r="A905" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="B905" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
     </row>
     <row r="906">
       <c r="A906" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="B906" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="907">
       <c r="A907" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="B907" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="908">
       <c r="A908" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="B908" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
     </row>
     <row r="909">
       <c r="A909" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="B909" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
     </row>
     <row r="910">
       <c r="A910" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="B910" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="911">
       <c r="A911" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="B911" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
     </row>
     <row r="912">
       <c r="A912" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="B912" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="913">
       <c r="A913" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="B913" t="s">
         <v>1</v>
@@ -12703,23 +12706,23 @@
     </row>
     <row r="914">
       <c r="A914" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="B914" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="915">
       <c r="A915" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="B915" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="916">
       <c r="A916" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="B916" t="s">
         <v>1</v>
@@ -12727,23 +12730,23 @@
     </row>
     <row r="917">
       <c r="A917" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="B917" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="918">
       <c r="A918" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="B918" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="919">
       <c r="A919" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="B919" t="s">
         <v>1</v>
@@ -12751,31 +12754,31 @@
     </row>
     <row r="920">
       <c r="A920" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
       <c r="B920" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="921">
       <c r="A921" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
       <c r="B921" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="922">
       <c r="A922" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="B922" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
     </row>
     <row r="923">
       <c r="A923" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="B923" t="s">
         <v>1</v>
@@ -12783,15 +12786,15 @@
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="B924" t="s">
-        <v>1639</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="925">
       <c r="A925" t="s">
-        <v>1640</v>
+        <v>1641</v>
       </c>
       <c r="B925" t="s">
         <v>1</v>
@@ -12799,15 +12802,15 @@
     </row>
     <row r="926">
       <c r="A926" t="s">
-        <v>1641</v>
+        <v>1642</v>
       </c>
       <c r="B926" t="s">
-        <v>1642</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="927">
       <c r="A927" t="s">
-        <v>1643</v>
+        <v>1644</v>
       </c>
       <c r="B927" t="s">
         <v>1</v>
@@ -12815,23 +12818,23 @@
     </row>
     <row r="928">
       <c r="A928" t="s">
-        <v>1644</v>
+        <v>1645</v>
       </c>
       <c r="B928" t="s">
-        <v>1645</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="929">
       <c r="A929" t="s">
-        <v>1646</v>
+        <v>1647</v>
       </c>
       <c r="B929" t="s">
-        <v>1647</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="930">
       <c r="A930" t="s">
-        <v>1648</v>
+        <v>1649</v>
       </c>
       <c r="B930" t="s">
         <v>1</v>
@@ -12839,71 +12842,71 @@
     </row>
     <row r="931">
       <c r="A931" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="B931" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="932">
       <c r="A932" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="B932" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="933">
       <c r="A933" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="B933" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="934">
       <c r="A934" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="B934" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="935">
       <c r="A935" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="B935" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="936">
       <c r="A936" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="B936" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="937">
       <c r="A937" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
       <c r="B937" t="s">
-        <v>1662</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="938">
       <c r="A938" t="s">
-        <v>1663</v>
+        <v>1664</v>
       </c>
       <c r="B938" t="s">
-        <v>1664</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="939">
       <c r="A939" t="s">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="B939" t="s">
         <v>1</v>
@@ -12911,191 +12914,191 @@
     </row>
     <row r="940">
       <c r="A940" t="s">
-        <v>1666</v>
+        <v>1667</v>
       </c>
       <c r="B940" t="s">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="941">
       <c r="A941" t="s">
-        <v>1668</v>
+        <v>1669</v>
       </c>
       <c r="B941" t="s">
-        <v>1669</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="942">
       <c r="A942" t="s">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="B942" t="s">
-        <v>1671</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="943">
       <c r="A943" t="s">
-        <v>1672</v>
+        <v>1673</v>
       </c>
       <c r="B943" t="s">
-        <v>1673</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="944">
       <c r="A944" t="s">
-        <v>1674</v>
+        <v>1675</v>
       </c>
       <c r="B944" t="s">
-        <v>1675</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="945">
       <c r="A945" t="s">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="B945" t="s">
-        <v>1677</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="946">
       <c r="A946" t="s">
-        <v>1678</v>
+        <v>1679</v>
       </c>
       <c r="B946" t="s">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="947">
       <c r="A947" t="s">
-        <v>1680</v>
+        <v>1681</v>
       </c>
       <c r="B947" t="s">
-        <v>1681</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="948">
       <c r="A948" t="s">
-        <v>1682</v>
+        <v>1683</v>
       </c>
       <c r="B948" t="s">
-        <v>1683</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="949">
       <c r="A949" t="s">
-        <v>1684</v>
+        <v>1685</v>
       </c>
       <c r="B949" t="s">
-        <v>1685</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="950">
       <c r="A950" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="B950" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="951">
       <c r="A951" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="B951" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="952">
       <c r="A952" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="B952" t="s">
-        <v>1691</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="953">
       <c r="A953" t="s">
-        <v>1692</v>
+        <v>1693</v>
       </c>
       <c r="B953" t="s">
-        <v>1693</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="954">
       <c r="A954" t="s">
-        <v>1694</v>
+        <v>1695</v>
       </c>
       <c r="B954" t="s">
-        <v>1695</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="955">
       <c r="A955" t="s">
-        <v>1696</v>
+        <v>1697</v>
       </c>
       <c r="B955" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="956">
       <c r="A956" t="s">
-        <v>1698</v>
+        <v>1699</v>
       </c>
       <c r="B956" t="s">
-        <v>1699</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="957">
       <c r="A957" t="s">
-        <v>1700</v>
+        <v>1701</v>
       </c>
       <c r="B957" t="s">
-        <v>1701</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="958">
       <c r="A958" t="s">
-        <v>1702</v>
+        <v>1703</v>
       </c>
       <c r="B958" t="s">
-        <v>1703</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="959">
       <c r="A959" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="B959" t="s">
-        <v>1705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="960">
       <c r="A960" t="s">
-        <v>1706</v>
+        <v>1707</v>
       </c>
       <c r="B960" t="s">
-        <v>1707</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="961">
       <c r="A961" t="s">
-        <v>1708</v>
+        <v>1709</v>
       </c>
       <c r="B961" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="962">
       <c r="A962" t="s">
-        <v>1710</v>
+        <v>1711</v>
       </c>
       <c r="B962" t="s">
-        <v>1711</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="963">
       <c r="A963" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="B963" t="s">
         <v>1</v>
@@ -13103,7 +13106,7 @@
     </row>
     <row r="964">
       <c r="A964" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
       <c r="B964" t="s">
         <v>1</v>
@@ -13111,7 +13114,7 @@
     </row>
     <row r="965">
       <c r="A965" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="B965" t="s">
         <v>1</v>
@@ -13119,7 +13122,7 @@
     </row>
     <row r="966">
       <c r="A966" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
       <c r="B966" t="s">
         <v>1</v>
@@ -13127,7 +13130,7 @@
     </row>
     <row r="967">
       <c r="A967" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="B967" t="s">
         <v>1</v>
@@ -13135,63 +13138,63 @@
     </row>
     <row r="968">
       <c r="A968" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
       <c r="B968" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="969">
       <c r="A969" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
       <c r="B969" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="970">
       <c r="A970" t="s">
-        <v>1721</v>
+        <v>1722</v>
       </c>
       <c r="B970" t="s">
-        <v>1722</v>
+        <v>1723</v>
       </c>
     </row>
     <row r="971">
       <c r="A971" t="s">
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="B971" t="s">
-        <v>1724</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="972">
       <c r="A972" t="s">
-        <v>1725</v>
+        <v>1726</v>
       </c>
       <c r="B972" t="s">
-        <v>1726</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="973">
       <c r="A973" t="s">
-        <v>1727</v>
+        <v>1728</v>
       </c>
       <c r="B973" t="s">
-        <v>1728</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="974">
       <c r="A974" t="s">
-        <v>1729</v>
+        <v>1730</v>
       </c>
       <c r="B974" t="s">
-        <v>1730</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="975">
       <c r="A975" t="s">
-        <v>1731</v>
+        <v>1732</v>
       </c>
       <c r="B975" t="s">
         <v>1</v>
@@ -13199,15 +13202,15 @@
     </row>
     <row r="976">
       <c r="A976" t="s">
-        <v>1732</v>
+        <v>1733</v>
       </c>
       <c r="B976" t="s">
-        <v>1733</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="977">
       <c r="A977" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="B977" t="s">
         <v>1</v>
@@ -13215,7 +13218,7 @@
     </row>
     <row r="978">
       <c r="A978" t="s">
-        <v>1735</v>
+        <v>1736</v>
       </c>
       <c r="B978" t="s">
         <v>1</v>
@@ -13223,23 +13226,23 @@
     </row>
     <row r="979">
       <c r="A979" t="s">
-        <v>1736</v>
+        <v>1737</v>
       </c>
       <c r="B979" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="980">
       <c r="A980" t="s">
-        <v>1738</v>
+        <v>1739</v>
       </c>
       <c r="B980" t="s">
-        <v>1739</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="981">
       <c r="A981" t="s">
-        <v>1740</v>
+        <v>1741</v>
       </c>
       <c r="B981" t="s">
         <v>1</v>
@@ -13247,170 +13250,170 @@
     </row>
     <row r="982">
       <c r="A982" t="s">
-        <v>1741</v>
+        <v>1742</v>
       </c>
       <c r="B982" t="s">
-        <v>1742</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="983">
       <c r="A983" t="s">
-        <v>1743</v>
+        <v>1744</v>
       </c>
       <c r="B983" t="s">
-        <v>1744</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="984">
       <c r="A984" t="s">
-        <v>1745</v>
+        <v>1746</v>
       </c>
       <c r="B984" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="985">
       <c r="A985" t="s">
-        <v>1746</v>
+        <v>1747</v>
       </c>
       <c r="B985" t="s">
-        <v>1747</v>
+        <v>1748</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" t="s">
-        <v>1748</v>
+        <v>1749</v>
       </c>
       <c r="B986" t="s">
-        <v>1749</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="987">
       <c r="A987" t="s">
-        <v>1750</v>
+        <v>1751</v>
       </c>
       <c r="B987" t="s">
-        <v>1751</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="988">
       <c r="A988" t="s">
-        <v>1752</v>
+        <v>1753</v>
       </c>
       <c r="B988" t="s">
-        <v>1753</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="989">
       <c r="A989" t="s">
-        <v>1754</v>
+        <v>1755</v>
       </c>
       <c r="B989" t="s">
-        <v>1755</v>
+        <v>1756</v>
       </c>
     </row>
     <row r="990">
       <c r="A990" t="s">
-        <v>1756</v>
+        <v>1757</v>
       </c>
       <c r="B990" t="s">
-        <v>1757</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="991">
       <c r="A991" t="s">
-        <v>1758</v>
+        <v>1759</v>
       </c>
       <c r="B991" t="s">
-        <v>1759</v>
+        <v>1760</v>
       </c>
     </row>
     <row r="992">
       <c r="A992" t="s">
-        <v>1760</v>
+        <v>1761</v>
       </c>
       <c r="B992" t="s">
-        <v>1761</v>
+        <v>1762</v>
       </c>
     </row>
     <row r="993">
       <c r="A993" t="s">
-        <v>1762</v>
+        <v>1763</v>
       </c>
       <c r="B993" t="s">
-        <v>1763</v>
+        <v>1764</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" t="s">
-        <v>1764</v>
+        <v>1765</v>
       </c>
       <c r="B994" t="s">
-        <v>1765</v>
+        <v>1766</v>
       </c>
     </row>
     <row r="995">
       <c r="A995" t="s">
-        <v>1766</v>
+        <v>1767</v>
       </c>
       <c r="B995" t="s">
-        <v>1767</v>
+        <v>1768</v>
       </c>
     </row>
     <row r="996">
       <c r="A996" t="s">
-        <v>1768</v>
+        <v>1769</v>
       </c>
       <c r="B996" t="s">
-        <v>1769</v>
+        <v>1770</v>
       </c>
     </row>
     <row r="997">
       <c r="A997" t="s">
-        <v>1770</v>
+        <v>1771</v>
       </c>
       <c r="B997" t="s">
-        <v>1771</v>
+        <v>1772</v>
       </c>
     </row>
     <row r="998">
       <c r="A998" t="s">
-        <v>1772</v>
+        <v>1773</v>
       </c>
       <c r="B998" t="s">
-        <v>1773</v>
+        <v>1774</v>
       </c>
     </row>
     <row r="999">
       <c r="A999" t="s">
-        <v>1774</v>
+        <v>1775</v>
       </c>
       <c r="B999" t="s">
-        <v>1775</v>
+        <v>1776</v>
       </c>
     </row>
     <row r="1000">
       <c r="A1000" t="s">
-        <v>1776</v>
+        <v>1777</v>
       </c>
       <c r="B1000" t="s">
-        <v>1777</v>
+        <v>1778</v>
       </c>
     </row>
     <row r="1001">
       <c r="A1001" t="s">
-        <v>1778</v>
+        <v>1779</v>
       </c>
       <c r="B1001" t="s">
-        <v>1779</v>
+        <v>1780</v>
       </c>
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>1780</v>
+        <v>1781</v>
       </c>
       <c r="B1002" t="s">
-        <v>1781</v>
+        <v>1782</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática hashcode dom ene 30 00:51:40 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -416,7 +416,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -863,7 +863,7 @@
     <t>01-010017A</t>
   </si>
   <si>
-    <t>94e3bdce9575af42f713c012e310963c</t>
+    <t>8c426e7290c4d1f01eeb3fbf2ba62f3e</t>
   </si>
   <si>
     <t>03-030033TC</t>
@@ -2543,7 +2543,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>132cb2ce7322a45f69527701ed8a4d23</t>
+    <t>6f604c66bf55c7354d0b02b41b484b06</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -2999,7 +2999,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>379d4952f7b707ba2ab09e2a82834f06</t>
+    <t>ee0661f8b517fbfeb3f1c9c39b3afbbb</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -5381,7 +5381,7 @@
     <t>02-020004A</t>
   </si>
   <si>
-    <t>81016273d6b4ba3f8e0fca8df6f28510</t>
+    <t>2358690801cdba3cc8571a3232208510</t>
   </si>
   <si>
     <t>01-010019TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié feb  2 00:52:37 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -62,7 +62,7 @@
     <t>03-030005A</t>
   </si>
   <si>
-    <t>b9894e60fbfa01ea11b5198f1b3e6816</t>
+    <t>0169e37e3988212261d59205cf57eaf4</t>
   </si>
   <si>
     <t>05-050305TC</t>
@@ -182,7 +182,7 @@
     <t>02-020005TC</t>
   </si>
   <si>
-    <t>2d603006f9044dd5ba838871fd6ca17f</t>
+    <t>e8db67910fb1f6d3504293c333c436bc</t>
   </si>
   <si>
     <t>05-0709-070921BTC</t>
@@ -194,7 +194,7 @@
     <t>03-030004A</t>
   </si>
   <si>
-    <t>275517544ea9c4a5c08f3e12dd907d64</t>
+    <t>5edbfa08927dfe7c01263719cfb649d7</t>
   </si>
   <si>
     <t>915-150011A</t>
@@ -1271,7 +1271,7 @@
     <t>03-030006A</t>
   </si>
   <si>
-    <t>31a1f5f2035dc54ba81e7354575f6b98</t>
+    <t>fbdbd89fe4c8a3e0b5263adc22dcecda</t>
   </si>
   <si>
     <t>05-050009TM</t>
@@ -2006,7 +2006,7 @@
     <t>03-030006TC</t>
   </si>
   <si>
-    <t>1a32d413d8e585b9ec898238a0f8b4cb</t>
+    <t>78de7d0156a844a2f8b0f8580cf6bf5a</t>
   </si>
   <si>
     <t>03-030006TM</t>
@@ -2027,7 +2027,7 @@
     <t>03-030006TP</t>
   </si>
   <si>
-    <t>83edd588031ac62cdc12c22965a4b3b9</t>
+    <t>c688fd3d455afcb71bdad83bdd5dccd8</t>
   </si>
   <si>
     <t>01-010016TM</t>
@@ -2102,7 +2102,7 @@
     <t>03-030070TP</t>
   </si>
   <si>
-    <t>b144c9348c1ba9f4281b4caf0324bbcf</t>
+    <t>03dec063dded497e23888fd1023a6ec0</t>
   </si>
   <si>
     <t>01-080101-010084TC</t>
@@ -2276,7 +2276,7 @@
     <t>03-030004TC</t>
   </si>
   <si>
-    <t>ab039e8b28b07cb439eb3fe7f2a6baee</t>
+    <t>85d73053d6bd2ddfbfe94826f269c34f</t>
   </si>
   <si>
     <t>01-010018TC</t>
@@ -2309,7 +2309,7 @@
     <t>03-030004TP</t>
   </si>
   <si>
-    <t>84a1a9aff333a40f7b93ff13f396825b</t>
+    <t>6ba5cbfe528424fdaa8ce50b3ac4c668</t>
   </si>
   <si>
     <t>03-030004TM</t>
@@ -2918,7 +2918,7 @@
     <t>03-030014TC</t>
   </si>
   <si>
-    <t>2effef6c964dcb44f3b44ffedd192277</t>
+    <t>eefff1636a79415d3da7ef860713c062</t>
   </si>
   <si>
     <t>05-0709-070904A</t>
@@ -2969,7 +2969,7 @@
     <t>03-030014TP</t>
   </si>
   <si>
-    <t>0f6a021fc3f90e64cb2240f676c06a7a</t>
+    <t>524de80c25f6a950f1045cc594eee0e7</t>
   </si>
   <si>
     <t>05-050317TC</t>
@@ -2999,7 +2999,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>ee0661f8b517fbfeb3f1c9c39b3afbbb</t>
+    <t>8057717257aa10a5aefef8701e479f97</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -3014,7 +3014,7 @@
     <t>03-030014A</t>
   </si>
   <si>
-    <t>9eb4c66d0f55cbf4bada3d8e5d1c7d14</t>
+    <t>0f7ee37177b494487dc85696289c131e</t>
   </si>
   <si>
     <t>03-030025TC</t>
@@ -4190,7 +4190,7 @@
     <t>02-020006TC</t>
   </si>
   <si>
-    <t>2802ab1063279d54146223f696f20eb3</t>
+    <t>179f3f0ad5983380b4d715dcc58e6ed8</t>
   </si>
   <si>
     <t>05-0709-070921ATC</t>
@@ -4208,7 +4208,7 @@
     <t>02-020006TM</t>
   </si>
   <si>
-    <t>fb6579275369feca2249f6a62946d497</t>
+    <t>85327766952c59c3a659c3f442d5bcba</t>
   </si>
   <si>
     <t>902-0204-02040101BTM</t>
@@ -4235,7 +4235,7 @@
     <t>02-020006TP</t>
   </si>
   <si>
-    <t>45cce2fdc22e2cfd7fa5302a2e549dab</t>
+    <t>16d862b5b45348824aa3b9f98f2217b8</t>
   </si>
   <si>
     <t>915-150001A</t>
@@ -4484,7 +4484,7 @@
     <t>03-030071A</t>
   </si>
   <si>
-    <t>bc215835c85ba728793c88004710b458</t>
+    <t>d6d0b2f8c75f698ee3d8d03972bdc7f0</t>
   </si>
   <si>
     <t>915-150010TP</t>
@@ -4565,7 +4565,7 @@
     <t>03-030070A</t>
   </si>
   <si>
-    <t>2ef08e05d9da3935517d358309018e8d</t>
+    <t>d8b1b0cf52780635fe09bb6c9e56df53</t>
   </si>
   <si>
     <t>03-02010301-030083TM</t>
@@ -5147,7 +5147,7 @@
     <t>03-030071TP</t>
   </si>
   <si>
-    <t>1ce9255c51d6bdec0678e73941c7577d</t>
+    <t>34f140734844fb61a075d45ac239509f</t>
   </si>
   <si>
     <t>915-150003TP</t>
@@ -5327,7 +5327,7 @@
     <t>02-020006A</t>
   </si>
   <si>
-    <t>0739e4252751d56b83824b70b671b54d</t>
+    <t>34ed1d8adeba8de35d50444181be245d</t>
   </si>
   <si>
     <t>03-030053A</t>
@@ -5375,13 +5375,13 @@
     <t>02-020005A</t>
   </si>
   <si>
-    <t>1a8e5457a3bd9250cc7c67eafb8d7f7a</t>
+    <t>6ae2c5c35eb4f600baf3c2fffc6ade50</t>
   </si>
   <si>
     <t>02-020004A</t>
   </si>
   <si>
-    <t>2358690801cdba3cc8571a3232208510</t>
+    <t>d235dc46db8c4188419edce01ac8d842</t>
   </si>
   <si>
     <t>01-010019TC</t>
@@ -5504,7 +5504,7 @@
     <t>03-030016TP</t>
   </si>
   <si>
-    <t>796573ddf36d26f56dec96dabdc96555</t>
+    <t>fee48c7deafa82713e9c9af486c3842b</t>
   </si>
   <si>
     <t>01-010080A</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue feb  3 00:49:04 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>cd53cfda870d675a46aabb75dabac73a</t>
+    <t>126cbfa771e07125e4b2588cb088a4f4</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>670ca03d45ae4deda6759bd69228f3b3</t>
+    <t>3b0fbddf9266f96c15f95f1cb78bd03e</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -257,7 +257,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>350695fbc57b4bf9ac73e53d7a194efb</t>
+    <t>bf86e0fcb1789146d8535d534852e2af</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -515,7 +515,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>f98d3adbdb8efe4d62c7e451ac498e86</t>
+    <t>cb708a4a797a3cd0f1914adf72b7a468</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -572,7 +572,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>a4b297bff48ec3af836197508aa01004</t>
+    <t>9e224f966054136359fa28a688aa0d21</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -632,7 +632,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>dcae650ff0198395db522f5051a0284b</t>
+    <t>b9a93d673458a0ca78015973f44cc41c</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -698,7 +698,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>71a1f5c9a268dd4b1a78437b5f3f1529</t>
+    <t>6eab34aa1446a6aee47e1b409eec906e</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -881,7 +881,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>98b160b051be064e950e52b80e8dc6b3</t>
+    <t>873b191962817aeaf6117898dd6bb831</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -914,13 +914,13 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>61f17683d4c301c375f58e5378f7b14b</t>
+    <t>48efd80717af1a8e5381b3a703081903</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>b4d1d6178ed057f8704efcc925066d96</t>
+    <t>477d93f0becca0e82152fc1649b52818</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -971,7 +971,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>3d76bb078691f3f726ac08246a586095</t>
+    <t>c5aebb6a943c2402c01201f18880780f</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1601,7 +1601,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>25e1d7e4e8683c11ece1258ab20b16cf</t>
+    <t>e2c9b0035f9c35f9936f140eecfb6ef6</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2663,7 +2663,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>685f55b15b443677a46e3f69c9ba39e9</t>
+    <t>f4ae1c33a5619a407c116f29b554953f</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3089,7 +3089,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>fe906ff07e924136c15856e381920b5d</t>
+    <t>2cc1855530e6c6092b359bf260a7fadd</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3194,7 +3194,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>f705fc37721472d6922066ff097ddc0f</t>
+    <t>549616537b4b413b4adf7188898abf39</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3629,7 +3629,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>a2b130461b47507481be660abd69a562</t>
+    <t>6e267de39856e55e5cb006860a4a9396</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3734,7 +3734,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>c08eadd331bc741a5bfd021e85679e74</t>
+    <t>ba871e7f461443cf68031fa50e3d2136</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3770,7 +3770,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>5772807470bdf084e92a5abdcb5d8620</t>
+    <t>0c79e5c6e1b3262747b018da6bb8637c</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4406,7 +4406,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>48cb46d049a291907c4ab613e1a8486b</t>
+    <t>92fa48fd25f7c71c8e69186732251937</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4670,7 +4670,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>24277b83c8f1dd7c586e267ca7294b09</t>
+    <t>ea04e986719044dacb28812c1fed4cef</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4679,7 +4679,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>4b454b3abd94b34d6df03880c46c21d6</t>
+    <t>633237cb971ea411cffa912a712f0e59</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4748,7 +4748,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>30723e4128085a331f4b551db59153a0</t>
+    <t>dbb72e87d18491c0aef0ea2199e21686</t>
   </si>
   <si>
     <t>05-050202TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie feb  4 00:43:55 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -110,7 +110,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>d4439f2b3e758b77cc649f1c996c2927</t>
+    <t>bde706590a3e736e4fe844136b815a85</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -4955,7 +4955,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>7cdbf5f1d177f00789b80583f45d2eb4</t>
+    <t>8349317b919c3bc475f817f4f4f67934</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb feb  5 00:49:37 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -713,7 +713,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>e1a60b47eb63df3e46d47eb115527ddf</t>
+    <t>c0ba50cafa6f8aa8dce5a5ad71c9dc11</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -728,7 +728,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>c5af9b683434da0d29df101587b4e8e2</t>
+    <t>9b0ffb71cffe94c202cfd850de163fe3</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -2729,7 +2729,7 @@
     <t>03-030016A</t>
   </si>
   <si>
-    <t>7e42d9e06c095ae413cd9106ea846901</t>
+    <t>02f2bd6e6d934cb7f2dec0a74c8feaa1</t>
   </si>
   <si>
     <t>03-030036TP</t>
@@ -5480,7 +5480,7 @@
     <t>03-030016TC</t>
   </si>
   <si>
-    <t>25186f157230b906b841ea45772fc542</t>
+    <t>cfd3dbf8f62cde614784deec086088dd</t>
   </si>
   <si>
     <t>915-150005TM</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié feb  9 00:39:55 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -3305,7 +3305,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>7ec0dab31e5ce420d67791fb1c92097a</t>
+    <t>d5535c875849057eeb461761b14a9610</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -5369,7 +5369,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
+    <t>49e6a091e08e2fc592046231facaf4a0</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue feb 10 00:24:11 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -908,7 +908,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>8227c75a000ca3ee33cd55a4260dfa13</t>
+    <t>f63c3e94a0bfb57878e76a5916e73977</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -1052,7 +1052,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>a99579acd27f9a5c815f23c37c4d6d09</t>
+    <t>e0e32f798bc918b54a9cefad21440407</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1139,7 +1139,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>3b7df35e6918b7366869a13856537bea</t>
+    <t>7c399ad9dd9e28c31a3fea1a3c291cd3</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1406,7 +1406,7 @@
     <t>05-050003TC</t>
   </si>
   <si>
-    <t>f931bbdaee592cd41b631d93ed47b49d</t>
+    <t>f08d623b4999e85c79a472cb17a8ea55</t>
   </si>
   <si>
     <t>03-030074TC</t>
@@ -1592,7 +1592,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>d0b9a813c810b9ce4d34f30cd6cc03b8</t>
+    <t>2431588cf19a84402c1ba2a8c76015e8</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1616,7 +1616,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>5987238f976ccd46dfa3db4de38d424a</t>
+    <t>4cb5c0718ec9fd482082874d301d566a</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1943,7 +1943,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>d2d95f832564b4407c329db49ccb0485</t>
+    <t>c61035de8b6147d7b10f7138b92bc4e7</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2573,7 +2573,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>18f3d1cf970697586af4ea8623a585de</t>
+    <t>2b296e12d0eec4bfc102c0563d5021cf</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2657,7 +2657,7 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>cd3665b58fbeaa58a957ffb8ec951beb</t>
+    <t>0545be46131de673c87e73d0dffe5aa2</t>
   </si>
   <si>
     <t>05-050313A</t>
@@ -2891,7 +2891,7 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>ef333b99210b49e5b1f5e82c75cfd2af</t>
+    <t>e0c657cf0a953344b52b67e6fce99458</t>
   </si>
   <si>
     <t>05-050311A</t>
@@ -2987,7 +2987,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>4d50a04fa20e22a3a287690c6f029d08</t>
+    <t>c1d306f9e2ba80920002b67c69cc0dc3</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -3554,7 +3554,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>b8d0e6287ef2d0179cae3a707bb020c2</t>
+    <t>7866d99db7a250464efab0abc15676b2</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -4331,7 +4331,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>4e077e8e7f470e510df8ed140e2a0be7</t>
+    <t>5f917ca17136ea08a2eae9703618a5b1</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4697,7 +4697,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>4f27c67acc81ee2525ce43b0ef23edd1</t>
+    <t>36ad985b6771b250d4bf63a975aefb82</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -5195,7 +5195,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>0cad4e262ba9a9a8d782ac9750965db2</t>
+    <t>12616f808cf635546ba0456a5d08c2fb</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -5339,7 +5339,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>be930e48d944e7f21f0e7d532b20aefb</t>
+    <t>a7f79e681597ac75b0080e7bfe77616e</t>
   </si>
   <si>
     <t>05-050002TM</t>
@@ -5369,7 +5369,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>49e6a091e08e2fc592046231facaf4a0</t>
+    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie feb 11 00:41:55 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -926,7 +926,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>e4eeed5217a92eeb68f69ee5784a4667</t>
+    <t>26b6388fc9538f693d1873579c77a281</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -1208,7 +1208,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>617ba96103c96c19149cd84cb1b8f02b</t>
+    <t>dc38857b873391537f19bac4ce575a3f</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -3560,7 +3560,7 @@
     <t>915-150007A</t>
   </si>
   <si>
-    <t>ffa1e7c8a9a56ee682110383762fcbb8</t>
+    <t>aafc841008ee60932cb171d145b4731f</t>
   </si>
   <si>
     <t>05-050204TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb feb 12 00:36:36 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -3179,7 +3179,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>1a04453f06db3fd36f54fec63082ea9a</t>
+    <t>cf3b48b676eef0643cac9a9258603993</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -5369,7 +5369,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
+    <t>49e6a091e08e2fc592046231facaf4a0</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié feb 16 00:30:50 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1103,7 +1103,7 @@
     <t>03-030008A</t>
   </si>
   <si>
-    <t>7cd6cd009cd0d26730b7d958f6e267ec</t>
+    <t>d08173185aa878798c80e1af79d01b17</t>
   </si>
   <si>
     <t>01-010014A</t>
@@ -1703,7 +1703,7 @@
     <t>03-030008TP</t>
   </si>
   <si>
-    <t>245144099cfad5d5c42d95bfa67945b0</t>
+    <t>c2b0ffd73d8f0e650ecb9479fc19bdc3</t>
   </si>
   <si>
     <t>01-010025TC</t>
@@ -1721,7 +1721,7 @@
     <t>03-030072TP</t>
   </si>
   <si>
-    <t>350988c015adaef798f9ca27e0db87e2</t>
+    <t>7e401525bef9802cbb1fb418d783a0c8</t>
   </si>
   <si>
     <t>01-080101-010082TC</t>
@@ -3212,7 +3212,7 @@
     <t>03-030012A</t>
   </si>
   <si>
-    <t>56c8d45a7d37b859645830d7ec698895</t>
+    <t>81af3bb337018d506e033f52f46e6229</t>
   </si>
   <si>
     <t>03-030045TC</t>
@@ -3287,7 +3287,7 @@
     <t>03-030012TC</t>
   </si>
   <si>
-    <t>eb90b19323a5859efa320578d58c13a6</t>
+    <t>c343b8af9730d9b0f2a1bda9812cad00</t>
   </si>
   <si>
     <t>03-030058TC</t>
@@ -3356,7 +3356,7 @@
     <t>03-030012TP</t>
   </si>
   <si>
-    <t>68cebef0e28dc8122bf6c530043b3209</t>
+    <t>ed5e5f90f4c12819871f5a7a639f3949</t>
   </si>
   <si>
     <t>03-030058TM</t>
@@ -4370,7 +4370,7 @@
     <t>03-030072A</t>
   </si>
   <si>
-    <t>fdcf1341c4940500bc3314e7d423c93f</t>
+    <t>cdc7797eb778eee8606b68e60f838635</t>
   </si>
   <si>
     <t>04-040019TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue feb 24 00:11:33 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -416,7 +416,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -1298,7 +1298,7 @@
     <t>05-050304A</t>
   </si>
   <si>
-    <t>99bc21ac42831f39bff659f8935330aa</t>
+    <t>fc8314de0008fc3294259c300333bcb5</t>
   </si>
   <si>
     <t>05-050009TP</t>
@@ -1733,7 +1733,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>9bfa2c0e7b53970858e269693029892d</t>
+    <t>c50399213199c10c9914952386204901</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -2354,7 +2354,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>0813cb845249c5451c8c01e79a519d76</t>
+    <t>83fa94b167cf58ad538c1b2b673197a3</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2897,7 +2897,7 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>efcd984cd91f208d2786d2d0969ff65a</t>
+    <t>4e02ae31e23bee984efec83658109f77</t>
   </si>
   <si>
     <t>05-050208TP</t>
@@ -3269,7 +3269,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>602e933d6d2aaeedd0b651a0e938944a</t>
+    <t>59e4bd4bb983798f5b5cc8cf58f31e43</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -4364,7 +4364,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>d1de03b9ac0400e9a34a7742526d3648</t>
+    <t>21645fb60f3090798330aaa1686e95ff</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4796,7 +4796,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>48b00896a9bde1b8e88944f68154ec90</t>
+    <t>abae9ca1c4ec548868a7cb0eb4be78a5</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4913,7 +4913,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>26e121910b71722f8e1c89ac50bb5a85</t>
+    <t>152445d28cf7d5a12d36b78d856d69aa</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -4994,7 +4994,7 @@
     <t>05-050003A</t>
   </si>
   <si>
-    <t>9c7541186009e0dc7ec43f55f2c7ec54</t>
+    <t>19d056e962c12a8561b6842187745c0e</t>
   </si>
   <si>
     <t>01-080101-010083A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar mar  1 00:00:43 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -266,7 +266,7 @@
     <t>03-030003A</t>
   </si>
   <si>
-    <t>ad0c0adeb810057d23e0313eea661020</t>
+    <t>c2509abefb4d160861c68976c38e0e4b</t>
   </si>
   <si>
     <t>915-150010A</t>
@@ -416,7 +416,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -2543,7 +2543,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>6f604c66bf55c7354d0b02b41b484b06</t>
+    <t>132cb2ce7322a45f69527701ed8a4d23</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -2870,7 +2870,7 @@
     <t>03-030003TP</t>
   </si>
   <si>
-    <t>a2236fa3a4e98225b0c3ca7cfa341108</t>
+    <t>4885538d2619b692ce63f642a9459cd6</t>
   </si>
   <si>
     <t>03-030049TP</t>
@@ -3161,7 +3161,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>cca1be701c5cbe681e1d2bf165590201</t>
+    <t>5dbec04815ce7ea72c19a98f9398c43e</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -5054,7 +5054,7 @@
     <t>03-030007TC</t>
   </si>
   <si>
-    <t>e957554b2c2c2b4c5ea763398deaa68f</t>
+    <t>69824790963390cecea97dd6ecd10bbd</t>
   </si>
   <si>
     <t>03-030060TM</t>
@@ -5126,7 +5126,7 @@
     <t>03-030007TP</t>
   </si>
   <si>
-    <t>ab60911b3a8c2def46c039a7ea38212a</t>
+    <t>69260edc45399a9e74fcd2b59b20a84b</t>
   </si>
   <si>
     <t>03-030055A</t>
@@ -5399,7 +5399,7 @@
     <t>03-030005TC</t>
   </si>
   <si>
-    <t>23d5a9f0ba40e9adc3292c76b87a5959</t>
+    <t>51bf60829c0e2a7b1e95dd5a446cc284</t>
   </si>
   <si>
     <t>915-150016TM</t>
@@ -5414,7 +5414,7 @@
     <t>03-030005TP</t>
   </si>
   <si>
-    <t>ea3d017c4918ce58e9ce802125274a83</t>
+    <t>af22f4a95f974c28e1577a463bb81f43</t>
   </si>
   <si>
     <t>01-010019TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar mar  1 23:52:32 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1262,7 +1262,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>69d4284d376990d418085daf75abd481</t>
+    <t>1b6422d083b2736d97d2b9b7461f2802</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1292,7 +1292,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>64afa6d2e791b9f6112ce49e177e285f</t>
+    <t>1a0ac85e8a8a563d5ed0f5cbad9040b2</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1304,7 +1304,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>dc751a302537469092198eaa8285e97f</t>
+    <t>d4e333626b97ce3d58f09b8b4a1a58e9</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1919,7 +1919,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>e1ded442d1e8b35961ea5da13b709e9f</t>
+    <t>edf4628911742339a6b3b5b7ad85ad2c</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2543,7 +2543,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>132cb2ce7322a45f69527701ed8a4d23</t>
+    <t>6f604c66bf55c7354d0b02b41b484b06</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -2762,7 +2762,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>7d4b45c186c577912f797b2cc368a27c</t>
+    <t>213b69a41b27dcea9947180af8c436be</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2903,7 +2903,7 @@
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>3b669c1005e4e0cbc720ec9ef5b123c6</t>
+    <t>da95f2992e5284998eb24e64fa5bc489</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2981,7 +2981,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>2743ed8a2ebf5ec609b103b49756d68b</t>
+    <t>0075cf71783d7d39531805a72161090f</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3374,7 +3374,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>59de58cbc09f296acee2a2ed29ba0d71</t>
+    <t>0cb3442e2f127197a4d44d538f9b37d7</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3824,7 +3824,7 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>19cdfee959ea099af41c01352a9630e0</t>
+    <t>564212c83d13024501f17513481bdfb2</t>
   </si>
   <si>
     <t>05-050317A</t>
@@ -3914,7 +3914,7 @@
     <t>05-050206TP</t>
   </si>
   <si>
-    <t>c0726107eb2f5f3f5c1b59e88cb28e2c</t>
+    <t>240833e01f8f202f7a40501e4baedccc</t>
   </si>
   <si>
     <t>01-010068TM</t>
@@ -4046,7 +4046,7 @@
     <t>05-050206A</t>
   </si>
   <si>
-    <t>2ec2b7e9549493900095ad760ffcff0e</t>
+    <t>a3bd54880573955dfb86226aa96ee80f</t>
   </si>
   <si>
     <t>05-050315A</t>
@@ -4109,7 +4109,7 @@
     <t>05-050304TP</t>
   </si>
   <si>
-    <t>765f11d2c1e45c2867103a0f0e8a03b0</t>
+    <t>601e1ff34b27c3e943372011c5d9533c</t>
   </si>
   <si>
     <t>04-040002TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue mar  3 00:48:56 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>126cbfa771e07125e4b2588cb088a4f4</t>
+    <t>31ac26a5582dbdf7f3d145f0fbfb00f4</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>3b0fbddf9266f96c15f95f1cb78bd03e</t>
+    <t>236c0c4eeb0730eb9a945b2f5570a182</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -416,7 +416,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -698,7 +698,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>6eab34aa1446a6aee47e1b409eec906e</t>
+    <t>6c01875b8a5e0aaaed5f0b29c620f4aa</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -728,7 +728,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>9b0ffb71cffe94c202cfd850de163fe3</t>
+    <t>ebd70716affc8c5c74c881671968808b</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -2663,7 +2663,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>f4ae1c33a5619a407c116f29b554953f</t>
+    <t>48106b354b6ec496451425876ca97f5a</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2999,7 +2999,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>8057717257aa10a5aefef8701e479f97</t>
+    <t>cbce97f245d8a2439b22aba0cbdff288</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -3629,7 +3629,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>6e267de39856e55e5cb006860a4a9396</t>
+    <t>bea992ccc75a691253ebffdb64fa1849</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3734,7 +3734,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>ba871e7f461443cf68031fa50e3d2136</t>
+    <t>c0da705ab138b6a2046866db350a13b2</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3770,7 +3770,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>0c79e5c6e1b3262747b018da6bb8637c</t>
+    <t>59f9b30e514380adfb3524daa64bb81c</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4955,7 +4955,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>8349317b919c3bc475f817f4f4f67934</t>
+    <t>bd19c62d4edcca4faa353a2dcfd9a6e4</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5381,7 +5381,7 @@
     <t>02-020004A</t>
   </si>
   <si>
-    <t>d235dc46db8c4188419edce01ac8d842</t>
+    <t>1e40f44430b614f8e24ae4d804cc0702</t>
   </si>
   <si>
     <t>01-010019TC</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie mar  4 00:44:02 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -257,7 +257,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>bf86e0fcb1789146d8535d534852e2af</t>
+    <t>c44ecad3aacc07617ba359234e6fafaa</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -515,7 +515,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>cb708a4a797a3cd0f1914adf72b7a468</t>
+    <t>a58ffda7d2e30f995ac0ff47632581c9</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -572,7 +572,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>9e224f966054136359fa28a688aa0d21</t>
+    <t>113715e6a0cbe9fe60c06aed9de89d72</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -632,7 +632,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>b9a93d673458a0ca78015973f44cc41c</t>
+    <t>f557dbd1c5e704a570470b4d580ab972</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -920,7 +920,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>477d93f0becca0e82152fc1649b52818</t>
+    <t>00610d373843ccb616240d7f737630e9</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -971,7 +971,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>c5aebb6a943c2402c01201f18880780f</t>
+    <t>47367f68d2bcfd0f3a6cb6810f7e2fa6</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1601,7 +1601,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>e2c9b0035f9c35f9936f140eecfb6ef6</t>
+    <t>6c10b3f3f86b5a994011bed91360a467</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -4406,7 +4406,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>92fa48fd25f7c71c8e69186732251937</t>
+    <t>09f66485e748018ab15bdd291c0e2129</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4679,7 +4679,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>633237cb971ea411cffa912a712f0e59</t>
+    <t>7707be0448aa86e220f2dfa55506f83b</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4748,7 +4748,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>dbb72e87d18491c0aef0ea2199e21686</t>
+    <t>78af1f43104c2cc3052b9b8c0306cc2e</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom mar  6 00:53:57 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -881,7 +881,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>873b191962817aeaf6117898dd6bb831</t>
+    <t>f5e43c4dd3dbee113c282c9947202abc</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -914,7 +914,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>48efd80717af1a8e5381b3a703081903</t>
+    <t>12463510cf82fc627510985e62c336bc</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3089,7 +3089,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>2cc1855530e6c6092b359bf260a7fadd</t>
+    <t>a3a57feae52a183feaa00f2cdb002eca</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3194,7 +3194,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>549616537b4b413b4adf7188898abf39</t>
+    <t>c775c56409fe4b9a45738b8812ca0293</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4670,7 +4670,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>ea04e986719044dacb28812c1fed4cef</t>
+    <t>7a2800eba5ffabf27adf1c9ff2e33d00</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar mar  8 00:42:45 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -110,7 +110,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>bde706590a3e736e4fe844136b815a85</t>
+    <t>0f23e8e12cee55cab6263bbe10828794</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -881,7 +881,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>f5e43c4dd3dbee113c282c9947202abc</t>
+    <t>873b191962817aeaf6117898dd6bb831</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -914,7 +914,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>12463510cf82fc627510985e62c336bc</t>
+    <t>48efd80717af1a8e5381b3a703081903</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3089,7 +3089,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>a3a57feae52a183feaa00f2cdb002eca</t>
+    <t>2cc1855530e6c6092b359bf260a7fadd</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3194,7 +3194,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c775c56409fe4b9a45738b8812ca0293</t>
+    <t>549616537b4b413b4adf7188898abf39</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4670,7 +4670,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>7a2800eba5ffabf27adf1c9ff2e33d00</t>
+    <t>ea04e986719044dacb28812c1fed4cef</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié mar  9 00:47:30 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -881,7 +881,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>873b191962817aeaf6117898dd6bb831</t>
+    <t>f5e43c4dd3dbee113c282c9947202abc</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -914,7 +914,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>48efd80717af1a8e5381b3a703081903</t>
+    <t>12463510cf82fc627510985e62c336bc</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -1052,7 +1052,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>e0e32f798bc918b54a9cefad21440407</t>
+    <t>b8ef3fee579fde6d42de5fd7a412c9f9</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1208,7 +1208,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>dc38857b873391537f19bac4ce575a3f</t>
+    <t>329947d03f5fbb4c41b5da2a9a29556a</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -3089,7 +3089,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>2cc1855530e6c6092b359bf260a7fadd</t>
+    <t>a3a57feae52a183feaa00f2cdb002eca</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3194,7 +3194,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>549616537b4b413b4adf7188898abf39</t>
+    <t>c775c56409fe4b9a45738b8812ca0293</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4670,7 +4670,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>ea04e986719044dacb28812c1fed4cef</t>
+    <t>7a2800eba5ffabf27adf1c9ff2e33d00</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue mar 10 00:37:40 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1919,7 +1919,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>edf4628911742339a6b3b5b7ad85ad2c</t>
+    <t>f1acef47e1a6b24d4d82cd2963aecce9</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -3305,7 +3305,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>d5535c875849057eeb461761b14a9610</t>
+    <t>15597e91a9b66aabdb7db7095ebf903a</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3374,7 +3374,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>0cb3442e2f127197a4d44d538f9b37d7</t>
+    <t>8f08d10cf74388becddf1552339983eb</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3629,7 +3629,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>bea992ccc75a691253ebffdb64fa1849</t>
+    <t>abcfbd4a5e0c7fc097ffdd83c6ee3275</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -5369,7 +5369,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
+    <t>49e6a091e08e2fc592046231facaf4a0</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie mar 11 00:09:22 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -926,7 +926,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>26b6388fc9538f693d1873579c77a281</t>
+    <t>1f31b8081129ecf4dd01e6fe1b16a476</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -1007,7 +1007,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>4238da6fb96789bb498971d8e512f54e</t>
+    <t>3c6a5e7496fcbb03cf86179a7d98c29b</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -2384,7 +2384,7 @@
     <t>03-030015TC</t>
   </si>
   <si>
-    <t>83915188c396798e95a3c5d842cea75a</t>
+    <t>b3c4b2fb1f0217bb6b2b3e81e013dcb9</t>
   </si>
   <si>
     <t>01-010007TC</t>
@@ -2420,7 +2420,7 @@
     <t>03-030015TP</t>
   </si>
   <si>
-    <t>abd8e9546a63d64fa7b638163f0d318d</t>
+    <t>6759f7e9b1f1f5c2c479e44ea398f3b1</t>
   </si>
   <si>
     <t>01-080101-010086TM</t>
@@ -2912,7 +2912,7 @@
     <t>03-030015A</t>
   </si>
   <si>
-    <t>19ddbcf717fba0b769c5f1391bea6f6e</t>
+    <t>877e7c3d22c24d7d1914aa2aceb67ec1</t>
   </si>
   <si>
     <t>03-030014TC</t>
@@ -3629,7 +3629,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>abcfbd4a5e0c7fc097ffdd83c6ee3275</t>
+    <t>bea992ccc75a691253ebffdb64fa1849</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -5369,7 +5369,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>49e6a091e08e2fc592046231facaf4a0</t>
+    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue mar 17 00:53:09 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1955,7 +1955,7 @@
     <t>915-150009A</t>
   </si>
   <si>
-    <t>510470d83a4916f17d151f817dbfe2c4</t>
+    <t>b86412fe5fe5c6be104b3ad2a09b253c</t>
   </si>
   <si>
     <t>05-050201TM</t>
@@ -3455,7 +3455,7 @@
     <t>915-150008A</t>
   </si>
   <si>
-    <t>c9fbd1d8b978bfce2d8482188976632d</t>
+    <t>624b35154f98b71b8c80936587e244d8</t>
   </si>
   <si>
     <t>05-0709-070955TP</t>
@@ -5369,7 +5369,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>49e6a091e08e2fc592046231facaf4a0</t>
+    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
   </si>
   <si>
     <t>02-020005A</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom mar 20 00:49:39 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -3089,7 +3089,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>a3a57feae52a183feaa00f2cdb002eca</t>
+    <t>b9238c3d16a8c518a0a90b12bbf6f636</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié mar 23 00:53:59 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -3734,7 +3734,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>c0da705ab138b6a2046866db350a13b2</t>
+    <t>ec4b9c72eadf05b03a44f79b9ba310c6</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie abr  1 00:55:54 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -251,7 +251,7 @@
     <t>05-0709-070908TC</t>
   </si>
   <si>
-    <t>d78990df1862b6dbc3cc8a970f8a3480</t>
+    <t>88ce1735532480c72b32ef51646daa05</t>
   </si>
   <si>
     <t>05-050105A</t>
@@ -332,7 +332,7 @@
     <t>05-0709-070908TM</t>
   </si>
   <si>
-    <t>c53912c4f70059faec7c26b975513572</t>
+    <t>5825b7d3596921e31aca9320332509b2</t>
   </si>
   <si>
     <t>03-030026A</t>
@@ -350,7 +350,7 @@
     <t>05-0709-070908TP</t>
   </si>
   <si>
-    <t>4e05305223e360a8e38718a184190ecd</t>
+    <t>aec1b3939c8038a5e89e2c291a3f4e97</t>
   </si>
   <si>
     <t>03-030002A</t>
@@ -479,7 +479,7 @@
     <t>05-0709-070952TC</t>
   </si>
   <si>
-    <t>9a5db73c9534f604467f508eb15529c7</t>
+    <t>a51f7748889faaecd4eb06c74c666900</t>
   </si>
   <si>
     <t>01-010041TM</t>
@@ -497,7 +497,7 @@
     <t>05-0709-070952TP</t>
   </si>
   <si>
-    <t>6d8341204789516057bbfe961f4c210f</t>
+    <t>96e9549a1a76078106d55f3b6f03ae51</t>
   </si>
   <si>
     <t>03-030057TP</t>
@@ -509,7 +509,7 @@
     <t>05-0709-070952TM</t>
   </si>
   <si>
-    <t>358cdad6f08cddf8823a1319b7362204</t>
+    <t>2e98ae1fbd37482b4bb718204ba65ab6</t>
   </si>
   <si>
     <t>05-050104A</t>
@@ -770,7 +770,7 @@
     <t>05-0709-070954TC</t>
   </si>
   <si>
-    <t>6b2f90f1c4f24cf840931c80057aeb5b</t>
+    <t>95985cb9733b6d87c6293b5eb69488f3</t>
   </si>
   <si>
     <t>04-040003TC</t>
@@ -848,7 +848,7 @@
     <t>05-0709-070954TP</t>
   </si>
   <si>
-    <t>55aa84e32c71003ec1c2da80fa01a948</t>
+    <t>200ccbd2f6a1307fb9201573cfa06429</t>
   </si>
   <si>
     <t>01-080101-010079TM</t>
@@ -1070,7 +1070,7 @@
     <t>05-0709-070906AA</t>
   </si>
   <si>
-    <t>20ad1b50ac69fb61eef5b1ac5bf6b447</t>
+    <t>2036bb49d693ba503f6b90238e04c6e8</t>
   </si>
   <si>
     <t>01-010067TC</t>
@@ -1115,13 +1115,13 @@
     <t>05-0709-070910TC</t>
   </si>
   <si>
-    <t>66af25c41f4beae13518d52d8bf6c7ef</t>
+    <t>1292de644e0e91823db29e72f7a2a593</t>
   </si>
   <si>
     <t>05-0709-070910TM</t>
   </si>
   <si>
-    <t>37918519eb60a7bf23f132633a7d14a4</t>
+    <t>9d53101d83aec8012af958899f8f2dd8</t>
   </si>
   <si>
     <t>01-010045TP</t>
@@ -1214,7 +1214,7 @@
     <t>05-0709-070910TP</t>
   </si>
   <si>
-    <t>bb9ffa8ad25621f081e6aa7a6eb95859</t>
+    <t>25bb6b8922786406c85e7f4e6793f028</t>
   </si>
   <si>
     <t>01-010045TC</t>
@@ -1820,7 +1820,7 @@
     <t>05-0709-070902TC</t>
   </si>
   <si>
-    <t>b40b1af66372a7b4200f93a3b9a705ab</t>
+    <t>e91a8bb3e8e757dd0d222541df0ee727</t>
   </si>
   <si>
     <t>03-02010301-030097TC</t>
@@ -1937,7 +1937,7 @@
     <t>05-0709-070902TP</t>
   </si>
   <si>
-    <t>852dd907a8027478a4daf60cf9088c2c</t>
+    <t>066d89d3f1ea5c31ac232654fdea51a1</t>
   </si>
   <si>
     <t>05-050201TP</t>
@@ -1949,7 +1949,7 @@
     <t>05-0709-070902TM</t>
   </si>
   <si>
-    <t>e3f9086b79cf7fd8be61a08dec119123</t>
+    <t>698ab646403cf6bca4514ee4f655526e</t>
   </si>
   <si>
     <t>915-150009A</t>
@@ -1994,7 +1994,7 @@
     <t>05-0709-070906ATC</t>
   </si>
   <si>
-    <t>da974a67874a2d43bbb8495550ba2bd8</t>
+    <t>3e634d60428857b97f54e37c1e206330</t>
   </si>
   <si>
     <t>915-150013TP</t>
@@ -2045,7 +2045,7 @@
     <t>05-0709-070906ATM</t>
   </si>
   <si>
-    <t>2d369adbe7742a8e45f327b8cad9e929</t>
+    <t>8cc5a4d99bf226aa2995aa0d14699b32</t>
   </si>
   <si>
     <t>03-030070TC</t>
@@ -2054,7 +2054,7 @@
     <t>05-0709-070906ATP</t>
   </si>
   <si>
-    <t>d2366e3876160ff8d83a9104aaef04fe</t>
+    <t>c423b2fd0c22582aa89570a92b795b16</t>
   </si>
   <si>
     <t>915-150013TC</t>
@@ -2084,7 +2084,7 @@
     <t>05-0709-070910A</t>
   </si>
   <si>
-    <t>ca3bc93378cdc336fb1d23bfd0287161</t>
+    <t>95362085d86e2357363fb6a130d4808d</t>
   </si>
   <si>
     <t>01-010074A</t>
@@ -2180,7 +2180,7 @@
     <t>05-0709-070904TC</t>
   </si>
   <si>
-    <t>2ea0d4a0a3b541bbee7a6b692bac4838</t>
+    <t>fe8de9a31d9deb0d2fa9bdd1836c8aa4</t>
   </si>
   <si>
     <t>01-010073A</t>
@@ -2234,7 +2234,7 @@
     <t>05-0709-070904TM</t>
   </si>
   <si>
-    <t>6c323504e32ff72973787c25c3d37b39</t>
+    <t>e9716c23cd2b38929b66696199d804ab</t>
   </si>
   <si>
     <t>01-010029TP</t>
@@ -2246,7 +2246,7 @@
     <t>05-0709-070904TP</t>
   </si>
   <si>
-    <t>263b79777cba372a1ce8952159ab7e5a</t>
+    <t>601d6bc103483850ab7140071515f8da</t>
   </si>
   <si>
     <t>03-030066A</t>
@@ -2264,7 +2264,7 @@
     <t>05-0709-070955A</t>
   </si>
   <si>
-    <t>f104fcc525b46f52197e6fa526a914d9</t>
+    <t>e987cfc30c2fbcd90de9c06292b04601</t>
   </si>
   <si>
     <t>915-150015TP</t>
@@ -2360,7 +2360,7 @@
     <t>05-0709-070954A</t>
   </si>
   <si>
-    <t>3363b4c2e8d7958f3eb77a47037d30e2</t>
+    <t>7d5c7dc8f623aebd7e22b44f194c3b80</t>
   </si>
   <si>
     <t>01-080101-010086TC</t>
@@ -2483,7 +2483,7 @@
     <t>05-0709-070953A</t>
   </si>
   <si>
-    <t>69eaf0d15580db9662dbadd5e7757bf6</t>
+    <t>aeeec4b2d3d6d45258b75168146bf6db</t>
   </si>
   <si>
     <t>03-030064A</t>
@@ -2531,7 +2531,7 @@
     <t>05-0709-070952A</t>
   </si>
   <si>
-    <t>625a89473f71f5ad7c8cf7e7d4c1e5cf</t>
+    <t>a89d4798e177098e2141ef2bcb9c67d7</t>
   </si>
   <si>
     <t>03-02010301-030088A</t>
@@ -2651,7 +2651,7 @@
     <t>05-0709-070909TC</t>
   </si>
   <si>
-    <t>4e57d31c81b8f0b4e80c3d80a51d4c70</t>
+    <t>3a9669a6089f20a9d3c870fbba3cb4cc</t>
   </si>
   <si>
     <t>05-050204A</t>
@@ -2780,7 +2780,7 @@
     <t>05-0709-070909TM</t>
   </si>
   <si>
-    <t>3dcb045817c3098469dbe3b3069eb83d</t>
+    <t>7ec6ac3224d80f978a7da37f3286e688</t>
   </si>
   <si>
     <t>01-010009TP</t>
@@ -2804,7 +2804,7 @@
     <t>05-0709-070909TP</t>
   </si>
   <si>
-    <t>1651e0a559aaee0fdaf68eecd726d95c</t>
+    <t>6efcb93f76d3f7ed23f6a5d4dd2f147c</t>
   </si>
   <si>
     <t>04-040011TP</t>
@@ -2924,7 +2924,7 @@
     <t>05-0709-070904A</t>
   </si>
   <si>
-    <t>198651d299d2370b52a79c886970ff2e</t>
+    <t>c9edcfcb1038e192fb210f9a82a62141</t>
   </si>
   <si>
     <t>05-050306TP</t>
@@ -3026,7 +3026,7 @@
     <t>05-0709-070903A</t>
   </si>
   <si>
-    <t>d9ab9cd344bee97c0795af36b91d8128</t>
+    <t>8eec6ffcef97e4d2bf963b50dc94cfa8</t>
   </si>
   <si>
     <t>05-050317TP</t>
@@ -3107,7 +3107,7 @@
     <t>05-0709-070902A</t>
   </si>
   <si>
-    <t>b28a09c762509387e269714acae243b2</t>
+    <t>58ccb35a244e1d5a7d9583fbcff414b1</t>
   </si>
   <si>
     <t>03-030013A</t>
@@ -3206,7 +3206,7 @@
     <t>05-0709-070901A</t>
   </si>
   <si>
-    <t>e6ece49d19fe9fdfa605f0790e42ec84</t>
+    <t>979f049d9df98d1f708386b326bb16c4</t>
   </si>
   <si>
     <t>03-030012A</t>
@@ -3461,7 +3461,7 @@
     <t>05-0709-070955TP</t>
   </si>
   <si>
-    <t>bb9dff84e3ecb0b4d96379730af7b7c7</t>
+    <t>30072928ba18de42643e147d855869dc</t>
   </si>
   <si>
     <t>03-02010301-030090A</t>
@@ -3752,13 +3752,13 @@
     <t>05-0709-070953TC</t>
   </si>
   <si>
-    <t>61f5ab1a750febd2448d6d4ca0bbfe4e</t>
+    <t>6525697d4f8377e1d8eae6c3a6308700</t>
   </si>
   <si>
     <t>05-0709-070953TP</t>
   </si>
   <si>
-    <t>87d77c62805a11f381beb9c5e15f72ae</t>
+    <t>c3889a0449e0bab2160be2a250d2f6f2</t>
   </si>
   <si>
     <t>03-030056TP</t>
@@ -3932,7 +3932,7 @@
     <t>05-0709-070909A</t>
   </si>
   <si>
-    <t>31cfbe580fe6dfa303d681e53f909b80</t>
+    <t>f64b266e8eaadc4e2e1e01f3f5d9a9e5</t>
   </si>
   <si>
     <t>05-050206TM</t>
@@ -4058,7 +4058,7 @@
     <t>05-0709-070908A</t>
   </si>
   <si>
-    <t>7392593711ab7bb3250d7e56e6dece16</t>
+    <t>60dd4bf4c2a0a853e9ee671012b01132</t>
   </si>
   <si>
     <t>01-010022TC</t>
@@ -4076,7 +4076,7 @@
     <t>05-0709-070905AA</t>
   </si>
   <si>
-    <t>b63bbf7509084a2b7b03ebc9663565f9</t>
+    <t>2499dffb01c68114a99ea19c9dcd1faa</t>
   </si>
   <si>
     <t>01-080101-010110TP</t>
@@ -4118,7 +4118,7 @@
     <t>05-0709-070955TC</t>
   </si>
   <si>
-    <t>5542a8cf58fbce45f1f2e76684655616</t>
+    <t>3cb2a3fe2dbe2798f113a586cc7b1b66</t>
   </si>
   <si>
     <t>03-030054TM</t>
@@ -4130,7 +4130,7 @@
     <t>05-0709-070921ATP</t>
   </si>
   <si>
-    <t>ea3f030a8a490b970f7da01d292fecd4</t>
+    <t>4339094c037786953fa88297fefbed6e</t>
   </si>
   <si>
     <t>01-010024A</t>
@@ -4196,7 +4196,7 @@
     <t>05-0709-070921ATC</t>
   </si>
   <si>
-    <t>f0e5c24140c9cb41727b2a54e3a260c8</t>
+    <t>77d7c1a0f6b4aa4c63452ee3164f851b</t>
   </si>
   <si>
     <t>05-050207A</t>
@@ -4268,7 +4268,7 @@
     <t>05-0709-070901TC</t>
   </si>
   <si>
-    <t>ed8d0f2e534d224e43bcd71563f0f88b</t>
+    <t>c140a13e825c462304778c0dd1cbd5d1</t>
   </si>
   <si>
     <t>03-02010301-030096TC</t>
@@ -4280,7 +4280,7 @@
     <t>05-0709-070901TM</t>
   </si>
   <si>
-    <t>d0a4601da0fc5a5240d54ddfe8dc7a7f</t>
+    <t>ea17c22c4563d2752ae5ddea4add6cb9</t>
   </si>
   <si>
     <t>01-010035TP</t>
@@ -4382,7 +4382,7 @@
     <t>05-0709-070901TP</t>
   </si>
   <si>
-    <t>ba34bad9b6e7c800a1ade4e878ae97ca</t>
+    <t>ec225dcc5f11ea0f240d0239b6d4bc16</t>
   </si>
   <si>
     <t>01-010035TC</t>
@@ -4601,7 +4601,7 @@
     <t>05-0709-070903TC</t>
   </si>
   <si>
-    <t>9015365624e759a6072540b262a12577</t>
+    <t>59dab8a7c07c3f0cee96a36884cdc7d5</t>
   </si>
   <si>
     <t>01-010037TC</t>
@@ -4703,7 +4703,7 @@
     <t>05-0709-070903TM</t>
   </si>
   <si>
-    <t>28b70e4534ed83807931652c2220affe</t>
+    <t>8d80d2d73cc5f33a32758b3a83592ca5</t>
   </si>
   <si>
     <t>03-02010301-030093A</t>
@@ -4724,7 +4724,7 @@
     <t>05-0709-070903TP</t>
   </si>
   <si>
-    <t>92e7cdbfdcec19b5bd7e74db6e8e538e</t>
+    <t>50ed6d92f70752b191f8846ae1fe2cf9</t>
   </si>
   <si>
     <t>04-040017TM</t>
@@ -5165,7 +5165,7 @@
     <t>05-0709-070905ATC</t>
   </si>
   <si>
-    <t>b2f44d3255fdd42d13a8b4353660a499</t>
+    <t>01df1df69a676cb2b68302ebf35e251b</t>
   </si>
   <si>
     <t>01-010006TC</t>
@@ -5243,7 +5243,7 @@
     <t>05-0709-070905ATP</t>
   </si>
   <si>
-    <t>b213c4e2488ad106b7235cb5839dce7a</t>
+    <t>3e858897f1ebce7138cacc3416a4c648</t>
   </si>
   <si>
     <t>03-030018TP</t>
@@ -5297,7 +5297,7 @@
     <t>05-0709-070921AA</t>
   </si>
   <si>
-    <t>95060d6e31bc91f2529e80a514b7f8a5</t>
+    <t>80c0ac0afae53c3b9d33dc6442967c45</t>
   </si>
   <si>
     <t>03-02010301-030094TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar abr  5 00:54:52 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>31ac26a5582dbdf7f3d145f0fbfb00f4</t>
+    <t>7d7c824d13b0edd9eb60004046df9e4c</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -110,7 +110,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>0f23e8e12cee55cab6263bbe10828794</t>
+    <t>e67da1c17f1502730c5ce1b99c683dc2</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>236c0c4eeb0730eb9a945b2f5570a182</t>
+    <t>1dbae929a398c0d7f341b4e0786afce1</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -257,7 +257,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>c44ecad3aacc07617ba359234e6fafaa</t>
+    <t>839afb82a7e9f485e2d2bcb09e1883fe</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -515,7 +515,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>a58ffda7d2e30f995ac0ff47632581c9</t>
+    <t>321a7e2a6fcefc626b64b06976f7c6bf</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -572,7 +572,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>113715e6a0cbe9fe60c06aed9de89d72</t>
+    <t>c1e4405a1645da86a794ce03898a9ef3</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -632,7 +632,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>f557dbd1c5e704a570470b4d580ab972</t>
+    <t>e77e811212818e1fe2da0f0a14ac6a46</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -698,7 +698,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>6c01875b8a5e0aaaed5f0b29c620f4aa</t>
+    <t>3e94cd92713379db1d84781c4fd47745</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -728,7 +728,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>ebd70716affc8c5c74c881671968808b</t>
+    <t>b4a7eca52aa90494d691ed0199186987</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -920,7 +920,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>00610d373843ccb616240d7f737630e9</t>
+    <t>ef95df62684b8387e6b4e1b7d48d62f7</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -971,7 +971,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>47367f68d2bcfd0f3a6cb6810f7e2fa6</t>
+    <t>821b2f0c4dd2dba17d082f9e1f79c783</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1601,7 +1601,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>6c10b3f3f86b5a994011bed91360a467</t>
+    <t>3ce2a2e3a59fdb0bac8e2f4ae25c5bf1</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2663,7 +2663,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>48106b354b6ec496451425876ca97f5a</t>
+    <t>3fefee5266c5808f908928623f67a55a</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3629,7 +3629,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>bea992ccc75a691253ebffdb64fa1849</t>
+    <t>50e430fc6f1e5a0cdf9319926e67599c</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3734,7 +3734,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>ec4b9c72eadf05b03a44f79b9ba310c6</t>
+    <t>3fa36eceba0dfc3928b76a26be3a057d</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3770,7 +3770,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>59f9b30e514380adfb3524daa64bb81c</t>
+    <t>752066aab612d792774f2a2fce61f748</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4406,7 +4406,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>09f66485e748018ab15bdd291c0e2129</t>
+    <t>370dd69d7dfe4dfeb0398252a0a8d6bd</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4679,7 +4679,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>7707be0448aa86e220f2dfa55506f83b</t>
+    <t>39a644bc9f34ccf8a002a473f177d0a4</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4748,7 +4748,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>78af1f43104c2cc3052b9b8c0306cc2e</t>
+    <t>feaf305e644a42347b28f33895da1e24</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4955,7 +4955,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>bd19c62d4edcca4faa353a2dcfd9a6e4</t>
+    <t>8e33ddbb48f509251c5788c3a6fafc4f</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue abr  7 00:48:01 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -881,7 +881,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>f5e43c4dd3dbee113c282c9947202abc</t>
+    <t>30550cba60603b3e82560b2057c0ebd5</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -914,7 +914,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>12463510cf82fc627510985e62c336bc</t>
+    <t>a4e0841b6cc8e8299c956b14c3174793</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3089,7 +3089,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>a3a57feae52a183feaa00f2cdb002eca</t>
+    <t>eef484af3c5b531d7b1bf20097b06551</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3194,7 +3194,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c775c56409fe4b9a45738b8812ca0293</t>
+    <t>fba1c716ba7c767371b3e6a4bf556735</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4670,7 +4670,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>7a2800eba5ffabf27adf1c9ff2e33d00</t>
+    <t>67648602f343be1c049a646dd66e1223</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie abr  8 00:49:11 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -713,7 +713,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>160044f0de910fac8d988d86c4588113</t>
+    <t>176fe717c556419f54307c9901b478e7</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -5516,7 +5516,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb abr 16 00:52:08 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -728,7 +728,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>b4a7eca52aa90494d691ed0199186987</t>
+    <t>56fac8b22afabfadd6421facc15af7fa</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -1052,7 +1052,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>b8ef3fee579fde6d42de5fd7a412c9f9</t>
+    <t>72452e70fc571abe35f60e9417bd4234</t>
   </si>
   <si>
     <t>04-040001TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue abr 21 00:47:44 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1571,7 +1571,7 @@
     <t>01-080101-010112TM</t>
   </si>
   <si>
-    <t>8c6e2b75376b8490b816902250befb49</t>
+    <t>85f7fbd715009cfab666983e3b1e6500</t>
   </si>
   <si>
     <t>01-010025TP</t>
@@ -4796,7 +4796,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>abae9ca1c4ec548868a7cb0eb4be78a5</t>
+    <t>1552a9e70e2088ecb4db5fe271ceca3a</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb abr 23 00:50:53 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="1847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2014" uniqueCount="1853">
   <si>
     <t>05-050305TM</t>
   </si>
@@ -5553,6 +5553,24 @@
   </si>
   <si>
     <t>a97cf78dd347585236b4e5bc9903ed0c</t>
+  </si>
+  <si>
+    <t>915-150002TP</t>
+  </si>
+  <si>
+    <t>915-150002TC</t>
+  </si>
+  <si>
+    <t>915-150002TM</t>
+  </si>
+  <si>
+    <t>915-150012TP</t>
+  </si>
+  <si>
+    <t>915-150012TC</t>
+  </si>
+  <si>
+    <t>915-150012TM</t>
   </si>
 </sst>
 </file>
@@ -13608,6 +13626,54 @@
         <v>1846</v>
       </c>
     </row>
+    <row r="1003">
+      <c r="A1003" t="s">
+        <v>1847</v>
+      </c>
+      <c r="B1003" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="s">
+        <v>1848</v>
+      </c>
+      <c r="B1004" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B1005" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="s">
+        <v>1850</v>
+      </c>
+      <c r="B1006" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="s">
+        <v>1851</v>
+      </c>
+      <c r="B1007" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="s">
+        <v>1852</v>
+      </c>
+      <c r="B1008" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática hashcode dom abr 24 00:56:05 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2014" uniqueCount="1853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2014" uniqueCount="1859">
   <si>
     <t>05-050305TM</t>
   </si>
@@ -2105,6 +2105,12 @@
     <t>03dec063dded497e23888fd1023a6ec0</t>
   </si>
   <si>
+    <t>915-150002TP</t>
+  </si>
+  <si>
+    <t>b6a1722c3cc0f4ac1c97c7d11c079d13</t>
+  </si>
+  <si>
     <t>01-080101-010084TC</t>
   </si>
   <si>
@@ -2135,6 +2141,12 @@
     <t>172db03539e2184365cf33be7505021b</t>
   </si>
   <si>
+    <t>915-150002TC</t>
+  </si>
+  <si>
+    <t>4dd7776ba6aa9646b072298ff0fa82c1</t>
+  </si>
+  <si>
     <t>02-020001TM</t>
   </si>
   <si>
@@ -2153,6 +2165,12 @@
     <t>1cbf49cdf87c5e50867291337099287d</t>
   </si>
   <si>
+    <t>915-150002TM</t>
+  </si>
+  <si>
+    <t>9e81969ae9925e8802c0ee7a5299642c</t>
+  </si>
+  <si>
     <t>03-030068A</t>
   </si>
   <si>
@@ -4766,6 +4784,12 @@
     <t>1e100934088aa191d7842f44a16ab78e</t>
   </si>
   <si>
+    <t>915-150012TP</t>
+  </si>
+  <si>
+    <t>bacaef8f55e0252f60122196f3ddefb5</t>
+  </si>
+  <si>
     <t>05-050311TC</t>
   </si>
   <si>
@@ -4775,12 +4799,24 @@
     <t>3bbeda48cc454f005a899945f7dbc5cd</t>
   </si>
   <si>
+    <t>915-150012TC</t>
+  </si>
+  <si>
+    <t>a3b98661bba10de86905304ca5f76fb3</t>
+  </si>
+  <si>
     <t>03-02010301-030092A</t>
   </si>
   <si>
     <t>c2356f648cfd8d7c6bafa8fa529e2fc9</t>
   </si>
   <si>
+    <t>915-150012TM</t>
+  </si>
+  <si>
+    <t>2b891fbc54698215fedcc1e5175bcb17</t>
+  </si>
+  <si>
     <t>03-030073TC</t>
   </si>
   <si>
@@ -5553,24 +5589,6 @@
   </si>
   <si>
     <t>a97cf78dd347585236b4e5bc9903ed0c</t>
-  </si>
-  <si>
-    <t>915-150002TP</t>
-  </si>
-  <si>
-    <t>915-150002TC</t>
-  </si>
-  <si>
-    <t>915-150002TM</t>
-  </si>
-  <si>
-    <t>915-150012TP</t>
-  </si>
-  <si>
-    <t>915-150012TC</t>
-  </si>
-  <si>
-    <t>915-150012TM</t>
   </si>
 </sst>
 </file>
@@ -8831,28 +8849,28 @@
         <v>733</v>
       </c>
       <c r="B403" t="s">
-        <v>1</v>
+        <v>734</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B404" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B405" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B406" t="s">
         <v>1</v>
@@ -8860,26 +8878,26 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B407" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="B408" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="B409" t="s">
-        <v>744</v>
+        <v>1</v>
       </c>
     </row>
     <row r="410">
@@ -8951,28 +8969,28 @@
         <v>761</v>
       </c>
       <c r="B418" t="s">
-        <v>1</v>
+        <v>762</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="B419" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B420" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B421" t="s">
         <v>1</v>
@@ -8980,26 +8998,26 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B422" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B423" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B424" t="s">
-        <v>772</v>
+        <v>1</v>
       </c>
     </row>
     <row r="425">
@@ -9199,31 +9217,31 @@
         <v>821</v>
       </c>
       <c r="B449" t="s">
-        <v>1</v>
+        <v>822</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B450" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B451" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="B452" t="s">
-        <v>827</v>
+        <v>1</v>
       </c>
     </row>
     <row r="453">
@@ -9367,28 +9385,28 @@
         <v>862</v>
       </c>
       <c r="B470" t="s">
-        <v>1</v>
+        <v>863</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="B471" t="s">
-        <v>1</v>
+        <v>865</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="B472" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="B473" t="s">
         <v>1</v>
@@ -9396,26 +9414,26 @@
     </row>
     <row r="474">
       <c r="A474" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="B474" t="s">
-        <v>868</v>
+        <v>1</v>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B475" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B476" t="s">
-        <v>872</v>
+        <v>1</v>
       </c>
     </row>
     <row r="477">
@@ -9423,31 +9441,31 @@
         <v>873</v>
       </c>
       <c r="B477" t="s">
-        <v>1</v>
+        <v>874</v>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B478" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B479" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B480" t="s">
-        <v>879</v>
+        <v>1</v>
       </c>
     </row>
     <row r="481">
@@ -9471,39 +9489,39 @@
         <v>884</v>
       </c>
       <c r="B483" t="s">
-        <v>1</v>
+        <v>885</v>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="B484" t="s">
-        <v>1</v>
+        <v>887</v>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="B485" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="B486" t="s">
-        <v>889</v>
+        <v>1</v>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B487" t="s">
-        <v>891</v>
+        <v>1</v>
       </c>
     </row>
     <row r="488">
@@ -9599,28 +9617,28 @@
         <v>914</v>
       </c>
       <c r="B499" t="s">
-        <v>1</v>
+        <v>915</v>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="B500" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="B501" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="B502" t="s">
         <v>1</v>
@@ -9628,34 +9646,34 @@
     </row>
     <row r="503">
       <c r="A503" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="B503" t="s">
-        <v>1</v>
+        <v>922</v>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="s">
-        <v>921</v>
+        <v>923</v>
       </c>
       <c r="B504" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="B505" t="s">
-        <v>924</v>
+        <v>1</v>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="B506" t="s">
-        <v>926</v>
+        <v>1</v>
       </c>
     </row>
     <row r="507">
@@ -9735,28 +9753,28 @@
         <v>945</v>
       </c>
       <c r="B516" t="s">
-        <v>1</v>
+        <v>946</v>
       </c>
     </row>
     <row r="517">
       <c r="A517" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="B517" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
     </row>
     <row r="518">
       <c r="A518" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B518" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
     <row r="519">
       <c r="A519" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B519" t="s">
         <v>1</v>
@@ -9764,26 +9782,26 @@
     </row>
     <row r="520">
       <c r="A520" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B520" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
     </row>
     <row r="521">
       <c r="A521" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B521" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
     </row>
     <row r="522">
       <c r="A522" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B522" t="s">
-        <v>956</v>
+        <v>1</v>
       </c>
     </row>
     <row r="523">
@@ -9791,31 +9809,31 @@
         <v>957</v>
       </c>
       <c r="B523" t="s">
-        <v>1</v>
+        <v>958</v>
       </c>
     </row>
     <row r="524">
       <c r="A524" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B524" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
     </row>
     <row r="525">
       <c r="A525" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B525" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B526" t="s">
-        <v>963</v>
+        <v>1</v>
       </c>
     </row>
     <row r="527">
@@ -9823,31 +9841,31 @@
         <v>964</v>
       </c>
       <c r="B527" t="s">
-        <v>1</v>
+        <v>965</v>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B528" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B529" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
     </row>
     <row r="530">
       <c r="A530" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="B530" t="s">
-        <v>970</v>
+        <v>1</v>
       </c>
     </row>
     <row r="531">
@@ -9855,31 +9873,31 @@
         <v>971</v>
       </c>
       <c r="B531" t="s">
-        <v>1</v>
+        <v>972</v>
       </c>
     </row>
     <row r="532">
       <c r="A532" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="B532" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
     </row>
     <row r="533">
       <c r="A533" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="B533" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
     </row>
     <row r="534">
       <c r="A534" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="B534" t="s">
-        <v>977</v>
+        <v>1</v>
       </c>
     </row>
     <row r="535">
@@ -9919,39 +9937,39 @@
         <v>986</v>
       </c>
       <c r="B539" t="s">
-        <v>1</v>
+        <v>987</v>
       </c>
     </row>
     <row r="540">
       <c r="A540" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="B540" t="s">
-        <v>1</v>
+        <v>989</v>
       </c>
     </row>
     <row r="541">
       <c r="A541" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="B541" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
     </row>
     <row r="542">
       <c r="A542" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="B542" t="s">
-        <v>991</v>
+        <v>1</v>
       </c>
     </row>
     <row r="543">
       <c r="A543" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="B543" t="s">
-        <v>993</v>
+        <v>1</v>
       </c>
     </row>
     <row r="544">
@@ -9967,31 +9985,31 @@
         <v>996</v>
       </c>
       <c r="B545" t="s">
-        <v>1</v>
+        <v>997</v>
       </c>
     </row>
     <row r="546">
       <c r="A546" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="B546" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
     </row>
     <row r="547">
       <c r="A547" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="B547" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="548">
       <c r="A548" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="B548" t="s">
-        <v>1002</v>
+        <v>1</v>
       </c>
     </row>
     <row r="549">
@@ -10031,31 +10049,31 @@
         <v>1011</v>
       </c>
       <c r="B553" t="s">
-        <v>1</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="554">
       <c r="A554" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B554" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="555">
       <c r="A555" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="B555" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="556">
       <c r="A556" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B556" t="s">
-        <v>1017</v>
+        <v>1</v>
       </c>
     </row>
     <row r="557">
@@ -10119,28 +10137,28 @@
         <v>1032</v>
       </c>
       <c r="B564" t="s">
-        <v>1</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="565">
       <c r="A565" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="B565" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="566">
       <c r="A566" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="B566" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="567">
       <c r="A567" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="B567" t="s">
         <v>1</v>
@@ -10148,34 +10166,34 @@
     </row>
     <row r="568">
       <c r="A568" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="B568" t="s">
-        <v>1</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="569">
       <c r="A569" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="B569" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="570">
       <c r="A570" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
       <c r="B570" t="s">
-        <v>1042</v>
+        <v>1</v>
       </c>
     </row>
     <row r="571">
       <c r="A571" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="B571" t="s">
-        <v>1044</v>
+        <v>1</v>
       </c>
     </row>
     <row r="572">
@@ -10183,31 +10201,31 @@
         <v>1045</v>
       </c>
       <c r="B572" t="s">
-        <v>1</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="573">
       <c r="A573" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="B573" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="574">
       <c r="A574" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B574" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="575">
       <c r="A575" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="B575" t="s">
-        <v>1051</v>
+        <v>1</v>
       </c>
     </row>
     <row r="576">
@@ -10239,31 +10257,31 @@
         <v>1058</v>
       </c>
       <c r="B579" t="s">
-        <v>1</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="580">
       <c r="A580" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="B580" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="581">
       <c r="A581" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="B581" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="582">
       <c r="A582" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="B582" t="s">
-        <v>1064</v>
+        <v>1</v>
       </c>
     </row>
     <row r="583">
@@ -10327,31 +10345,31 @@
         <v>1079</v>
       </c>
       <c r="B590" t="s">
-        <v>1</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="591">
       <c r="A591" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="B591" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="592">
       <c r="A592" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B592" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="593">
       <c r="A593" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="B593" t="s">
-        <v>1085</v>
+        <v>1</v>
       </c>
     </row>
     <row r="594">
@@ -10439,31 +10457,31 @@
         <v>1106</v>
       </c>
       <c r="B604" t="s">
-        <v>1</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B605" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B606" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="B607" t="s">
-        <v>1112</v>
+        <v>1</v>
       </c>
     </row>
     <row r="608">
@@ -10583,31 +10601,31 @@
         <v>1141</v>
       </c>
       <c r="B622" t="s">
-        <v>1</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="623">
       <c r="A623" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B623" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="624">
       <c r="A624" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="B624" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="B625" t="s">
-        <v>1147</v>
+        <v>1</v>
       </c>
     </row>
     <row r="626">
@@ -10687,31 +10705,31 @@
         <v>1166</v>
       </c>
       <c r="B635" t="s">
-        <v>1</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="B636" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="B637" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="B638" t="s">
-        <v>1172</v>
+        <v>1</v>
       </c>
     </row>
     <row r="639">
@@ -10719,28 +10737,28 @@
         <v>1173</v>
       </c>
       <c r="B639" t="s">
-        <v>1</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="640">
       <c r="A640" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="B640" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B641" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="B642" t="s">
         <v>1</v>
@@ -10748,23 +10766,23 @@
     </row>
     <row r="643">
       <c r="A643" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="B643" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="B644" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="B645" t="s">
         <v>1</v>
@@ -10772,26 +10790,26 @@
     </row>
     <row r="646">
       <c r="A646" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="B646" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="B647" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="B648" t="s">
-        <v>1189</v>
+        <v>1</v>
       </c>
     </row>
     <row r="649">
@@ -10807,31 +10825,31 @@
         <v>1192</v>
       </c>
       <c r="B650" t="s">
-        <v>1</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="651">
       <c r="A651" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="B651" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="B652" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="B653" t="s">
-        <v>1198</v>
+        <v>1</v>
       </c>
     </row>
     <row r="654">
@@ -10847,31 +10865,31 @@
         <v>1201</v>
       </c>
       <c r="B655" t="s">
-        <v>1</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="656">
       <c r="A656" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="B656" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="657">
       <c r="A657" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="B657" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="B658" t="s">
-        <v>1207</v>
+        <v>1</v>
       </c>
     </row>
     <row r="659">
@@ -10887,28 +10905,28 @@
         <v>1210</v>
       </c>
       <c r="B660" t="s">
-        <v>1</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="661">
       <c r="A661" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="B661" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="662">
       <c r="A662" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="B662" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="663">
       <c r="A663" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="B663" t="s">
         <v>1</v>
@@ -10916,34 +10934,34 @@
     </row>
     <row r="664">
       <c r="A664" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="B664" t="s">
-        <v>1</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="665">
       <c r="A665" t="s">
-        <v>1217</v>
+        <v>1219</v>
       </c>
       <c r="B665" t="s">
-        <v>1218</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="666">
       <c r="A666" t="s">
-        <v>1219</v>
+        <v>1221</v>
       </c>
       <c r="B666" t="s">
-        <v>1220</v>
+        <v>1</v>
       </c>
     </row>
     <row r="667">
       <c r="A667" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="B667" t="s">
-        <v>1222</v>
+        <v>1</v>
       </c>
     </row>
     <row r="668">
@@ -10951,31 +10969,31 @@
         <v>1223</v>
       </c>
       <c r="B668" t="s">
-        <v>1</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="669">
       <c r="A669" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="B669" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="670">
       <c r="A670" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="B670" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="671">
       <c r="A671" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="B671" t="s">
-        <v>1229</v>
+        <v>1</v>
       </c>
     </row>
     <row r="672">
@@ -10983,31 +11001,31 @@
         <v>1230</v>
       </c>
       <c r="B672" t="s">
-        <v>1</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="673">
       <c r="A673" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="B673" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="674">
       <c r="A674" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="B674" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="675">
       <c r="A675" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="B675" t="s">
-        <v>1236</v>
+        <v>1</v>
       </c>
     </row>
     <row r="676">
@@ -11087,31 +11105,31 @@
         <v>1255</v>
       </c>
       <c r="B685" t="s">
-        <v>1</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="686">
       <c r="A686" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="B686" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="687">
       <c r="A687" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="B687" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="688">
       <c r="A688" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="B688" t="s">
-        <v>1261</v>
+        <v>1</v>
       </c>
     </row>
     <row r="689">
@@ -11127,31 +11145,31 @@
         <v>1264</v>
       </c>
       <c r="B690" t="s">
-        <v>1</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="691">
       <c r="A691" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="B691" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="692">
       <c r="A692" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="B692" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="693">
       <c r="A693" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="B693" t="s">
-        <v>1270</v>
+        <v>1</v>
       </c>
     </row>
     <row r="694">
@@ -11303,47 +11321,47 @@
         <v>1307</v>
       </c>
       <c r="B712" t="s">
-        <v>1</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="713">
       <c r="A713" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="B713" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="714">
       <c r="A714" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="B714" t="s">
-        <v>1</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="715">
       <c r="A715" t="s">
-        <v>1311</v>
+        <v>1313</v>
       </c>
       <c r="B715" t="s">
-        <v>1312</v>
+        <v>1</v>
       </c>
     </row>
     <row r="716">
       <c r="A716" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="B716" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="717">
       <c r="A717" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="B717" t="s">
-        <v>1316</v>
+        <v>1</v>
       </c>
     </row>
     <row r="718">
@@ -11367,39 +11385,39 @@
         <v>1321</v>
       </c>
       <c r="B720" t="s">
-        <v>1</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="721">
       <c r="A721" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="B721" t="s">
-        <v>1</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="722">
       <c r="A722" t="s">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="B722" t="s">
-        <v>1324</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="723">
       <c r="A723" t="s">
-        <v>1325</v>
+        <v>1327</v>
       </c>
       <c r="B723" t="s">
-        <v>1326</v>
+        <v>1</v>
       </c>
     </row>
     <row r="724">
       <c r="A724" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="B724" t="s">
-        <v>1328</v>
+        <v>1</v>
       </c>
     </row>
     <row r="725">
@@ -11407,31 +11425,31 @@
         <v>1329</v>
       </c>
       <c r="B725" t="s">
-        <v>1</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="726">
       <c r="A726" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="B726" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="727">
       <c r="A727" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="B727" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="728">
       <c r="A728" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B728" t="s">
-        <v>1335</v>
+        <v>1</v>
       </c>
     </row>
     <row r="729">
@@ -11447,31 +11465,31 @@
         <v>1338</v>
       </c>
       <c r="B730" t="s">
-        <v>1</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="731">
       <c r="A731" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="B731" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="732">
       <c r="A732" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="B732" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="733">
       <c r="A733" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="B733" t="s">
-        <v>1344</v>
+        <v>1</v>
       </c>
     </row>
     <row r="734">
@@ -11479,39 +11497,39 @@
         <v>1345</v>
       </c>
       <c r="B734" t="s">
-        <v>1</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="735">
       <c r="A735" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="B735" t="s">
-        <v>1</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="736">
       <c r="A736" t="s">
-        <v>1347</v>
+        <v>1349</v>
       </c>
       <c r="B736" t="s">
-        <v>1348</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="737">
       <c r="A737" t="s">
-        <v>1349</v>
+        <v>1351</v>
       </c>
       <c r="B737" t="s">
-        <v>1350</v>
+        <v>1</v>
       </c>
     </row>
     <row r="738">
       <c r="A738" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="B738" t="s">
-        <v>1352</v>
+        <v>1</v>
       </c>
     </row>
     <row r="739">
@@ -11535,31 +11553,31 @@
         <v>1357</v>
       </c>
       <c r="B741" t="s">
-        <v>1</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="742">
       <c r="A742" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="B742" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="743">
       <c r="A743" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="B743" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="744">
       <c r="A744" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="B744" t="s">
-        <v>1363</v>
+        <v>1</v>
       </c>
     </row>
     <row r="745">
@@ -11575,31 +11593,31 @@
         <v>1366</v>
       </c>
       <c r="B746" t="s">
-        <v>1</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="747">
       <c r="A747" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="B747" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="748">
       <c r="A748" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="B748" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="749">
       <c r="A749" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="B749" t="s">
-        <v>1372</v>
+        <v>1</v>
       </c>
     </row>
     <row r="750">
@@ -11631,28 +11649,28 @@
         <v>1379</v>
       </c>
       <c r="B753" t="s">
-        <v>1</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="754">
       <c r="A754" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="B754" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="755">
       <c r="A755" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="B755" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="756">
       <c r="A756" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="B756" t="s">
         <v>1</v>
@@ -11660,23 +11678,23 @@
     </row>
     <row r="757">
       <c r="A757" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="B757" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="758">
       <c r="A758" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="B758" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="759">
       <c r="A759" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="B759" t="s">
         <v>1</v>
@@ -11684,34 +11702,34 @@
     </row>
     <row r="760">
       <c r="A760" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
       <c r="B760" t="s">
-        <v>1</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="761">
       <c r="A761" t="s">
-        <v>1391</v>
+        <v>1393</v>
       </c>
       <c r="B761" t="s">
-        <v>1392</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="762">
       <c r="A762" t="s">
-        <v>1393</v>
+        <v>1395</v>
       </c>
       <c r="B762" t="s">
-        <v>1394</v>
+        <v>1</v>
       </c>
     </row>
     <row r="763">
       <c r="A763" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="B763" t="s">
-        <v>1396</v>
+        <v>1</v>
       </c>
     </row>
     <row r="764">
@@ -11727,31 +11745,31 @@
         <v>1399</v>
       </c>
       <c r="B765" t="s">
-        <v>1</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="766">
       <c r="A766" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="B766" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="767">
       <c r="A767" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="B767" t="s">
-        <v>1403</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="768">
       <c r="A768" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="B768" t="s">
-        <v>1405</v>
+        <v>1</v>
       </c>
     </row>
     <row r="769">
@@ -11783,31 +11801,31 @@
         <v>1412</v>
       </c>
       <c r="B772" t="s">
-        <v>1</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="773">
       <c r="A773" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="B773" t="s">
-        <v>1414</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="774">
       <c r="A774" t="s">
-        <v>1415</v>
+        <v>1416</v>
       </c>
       <c r="B774" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
     </row>
     <row r="775">
       <c r="A775" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="B775" t="s">
-        <v>1418</v>
+        <v>1</v>
       </c>
     </row>
     <row r="776">
@@ -11839,31 +11857,31 @@
         <v>1425</v>
       </c>
       <c r="B779" t="s">
-        <v>1</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="780">
       <c r="A780" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="B780" t="s">
-        <v>1427</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="781">
       <c r="A781" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="B781" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
     </row>
     <row r="782">
       <c r="A782" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="B782" t="s">
-        <v>1431</v>
+        <v>1</v>
       </c>
     </row>
     <row r="783">
@@ -11911,31 +11929,31 @@
         <v>1442</v>
       </c>
       <c r="B788" t="s">
-        <v>1</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="789">
       <c r="A789" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
       <c r="B789" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="790">
       <c r="A790" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="B790" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="791">
       <c r="A791" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="B791" t="s">
-        <v>1448</v>
+        <v>1</v>
       </c>
     </row>
     <row r="792">
@@ -12143,31 +12161,31 @@
         <v>1499</v>
       </c>
       <c r="B817" t="s">
-        <v>1</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="818">
       <c r="A818" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="B818" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="B819" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="820">
       <c r="A820" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
       <c r="B820" t="s">
-        <v>1505</v>
+        <v>1</v>
       </c>
     </row>
     <row r="821">
@@ -12279,44 +12297,44 @@
         <v>1532</v>
       </c>
       <c r="B834" t="s">
-        <v>1</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="835">
       <c r="A835" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="B835" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="836">
       <c r="A836" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="B836" t="s">
-        <v>1</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="837">
       <c r="A837" t="s">
-        <v>1536</v>
+        <v>1538</v>
       </c>
       <c r="B837" t="s">
-        <v>1537</v>
+        <v>1</v>
       </c>
     </row>
     <row r="838">
       <c r="A838" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
       <c r="B838" t="s">
-        <v>1</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="839">
       <c r="A839" t="s">
-        <v>1539</v>
+        <v>1541</v>
       </c>
       <c r="B839" t="s">
         <v>1</v>
@@ -12324,23 +12342,23 @@
     </row>
     <row r="840">
       <c r="A840" t="s">
-        <v>1540</v>
+        <v>1542</v>
       </c>
       <c r="B840" t="s">
-        <v>1541</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="841">
       <c r="A841" t="s">
-        <v>1542</v>
+        <v>1544</v>
       </c>
       <c r="B841" t="s">
-        <v>1543</v>
+        <v>1</v>
       </c>
     </row>
     <row r="842">
       <c r="A842" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="B842" t="s">
         <v>1</v>
@@ -12348,26 +12366,26 @@
     </row>
     <row r="843">
       <c r="A843" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="B843" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
     </row>
     <row r="844">
       <c r="A844" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="B844" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="845">
       <c r="A845" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="B845" t="s">
-        <v>1550</v>
+        <v>1</v>
       </c>
     </row>
     <row r="846">
@@ -12383,31 +12401,31 @@
         <v>1553</v>
       </c>
       <c r="B847" t="s">
-        <v>1</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="848">
       <c r="A848" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="B848" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="849">
       <c r="A849" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="B849" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="850">
       <c r="A850" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="B850" t="s">
-        <v>1559</v>
+        <v>1</v>
       </c>
     </row>
     <row r="851">
@@ -12439,31 +12457,31 @@
         <v>1566</v>
       </c>
       <c r="B854" t="s">
-        <v>1</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="855">
       <c r="A855" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="B855" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="856">
       <c r="A856" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="B856" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="857">
       <c r="A857" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="B857" t="s">
-        <v>1572</v>
+        <v>1</v>
       </c>
     </row>
     <row r="858">
@@ -12495,28 +12513,28 @@
         <v>1579</v>
       </c>
       <c r="B861" t="s">
-        <v>1</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="862">
       <c r="A862" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="B862" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="B863" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="B864" t="s">
         <v>1</v>
@@ -12524,34 +12542,34 @@
     </row>
     <row r="865">
       <c r="A865" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="B865" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="866">
       <c r="A866" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="B866" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="867">
       <c r="A867" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="B867" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="868">
       <c r="A868" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="B868" t="s">
-        <v>1592</v>
+        <v>1</v>
       </c>
     </row>
     <row r="869">
@@ -12687,55 +12705,55 @@
         <v>1625</v>
       </c>
       <c r="B885" t="s">
-        <v>1</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="886">
       <c r="A886" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="B886" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="887">
       <c r="A887" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="B887" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="888">
       <c r="A888" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="B888" t="s">
-        <v>1631</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="889">
       <c r="A889" t="s">
-        <v>1632</v>
+        <v>1633</v>
       </c>
       <c r="B889" t="s">
-        <v>1633</v>
+        <v>1634</v>
       </c>
     </row>
     <row r="890">
       <c r="A890" t="s">
-        <v>1634</v>
+        <v>1635</v>
       </c>
       <c r="B890" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="891">
       <c r="A891" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="B891" t="s">
-        <v>1637</v>
+        <v>1</v>
       </c>
     </row>
     <row r="892">
@@ -12783,55 +12801,55 @@
         <v>1648</v>
       </c>
       <c r="B897" t="s">
-        <v>1</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="898">
       <c r="A898" t="s">
-        <v>1649</v>
+        <v>1650</v>
       </c>
       <c r="B898" t="s">
-        <v>1650</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="899">
       <c r="A899" t="s">
-        <v>1651</v>
+        <v>1652</v>
       </c>
       <c r="B899" t="s">
-        <v>1652</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="900">
       <c r="A900" t="s">
-        <v>1653</v>
+        <v>1654</v>
       </c>
       <c r="B900" t="s">
-        <v>1654</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="901">
       <c r="A901" t="s">
-        <v>1655</v>
+        <v>1656</v>
       </c>
       <c r="B901" t="s">
-        <v>1656</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="902">
       <c r="A902" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="B902" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="903">
       <c r="A903" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="B903" t="s">
-        <v>1660</v>
+        <v>1</v>
       </c>
     </row>
     <row r="904">
@@ -12935,76 +12953,76 @@
         <v>1685</v>
       </c>
       <c r="B916" t="s">
-        <v>1</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="917">
       <c r="A917" t="s">
-        <v>1686</v>
+        <v>1687</v>
       </c>
       <c r="B917" t="s">
-        <v>1687</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="918">
       <c r="A918" t="s">
-        <v>1688</v>
+        <v>1689</v>
       </c>
       <c r="B918" t="s">
-        <v>1689</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="919">
       <c r="A919" t="s">
-        <v>1690</v>
+        <v>1691</v>
       </c>
       <c r="B919" t="s">
-        <v>1</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="920">
       <c r="A920" t="s">
-        <v>1691</v>
+        <v>1693</v>
       </c>
       <c r="B920" t="s">
-        <v>1692</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="921">
       <c r="A921" t="s">
-        <v>1693</v>
+        <v>1695</v>
       </c>
       <c r="B921" t="s">
-        <v>1694</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="922">
       <c r="A922" t="s">
-        <v>1695</v>
+        <v>1697</v>
       </c>
       <c r="B922" t="s">
-        <v>1696</v>
+        <v>1</v>
       </c>
     </row>
     <row r="923">
       <c r="A923" t="s">
-        <v>1697</v>
+        <v>1698</v>
       </c>
       <c r="B923" t="s">
-        <v>1</v>
+        <v>1699</v>
       </c>
     </row>
     <row r="924">
       <c r="A924" t="s">
-        <v>1698</v>
+        <v>1700</v>
       </c>
       <c r="B924" t="s">
-        <v>1699</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="925">
       <c r="A925" t="s">
-        <v>1700</v>
+        <v>1702</v>
       </c>
       <c r="B925" t="s">
         <v>1</v>
@@ -13012,90 +13030,90 @@
     </row>
     <row r="926">
       <c r="A926" t="s">
-        <v>1701</v>
+        <v>1703</v>
       </c>
       <c r="B926" t="s">
-        <v>1702</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="927">
       <c r="A927" t="s">
-        <v>1703</v>
+        <v>1705</v>
       </c>
       <c r="B927" t="s">
-        <v>1704</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="928">
       <c r="A928" t="s">
-        <v>1705</v>
+        <v>1707</v>
       </c>
       <c r="B928" t="s">
-        <v>1706</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="929">
       <c r="A929" t="s">
-        <v>1707</v>
+        <v>1709</v>
       </c>
       <c r="B929" t="s">
-        <v>1708</v>
+        <v>1</v>
       </c>
     </row>
     <row r="930">
       <c r="A930" t="s">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="B930" t="s">
-        <v>1</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="931">
       <c r="A931" t="s">
-        <v>1710</v>
+        <v>1712</v>
       </c>
       <c r="B931" t="s">
-        <v>1711</v>
+        <v>1</v>
       </c>
     </row>
     <row r="932">
       <c r="A932" t="s">
-        <v>1712</v>
+        <v>1713</v>
       </c>
       <c r="B932" t="s">
-        <v>1713</v>
+        <v>1714</v>
       </c>
     </row>
     <row r="933">
       <c r="A933" t="s">
-        <v>1714</v>
+        <v>1715</v>
       </c>
       <c r="B933" t="s">
-        <v>1715</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="934">
       <c r="A934" t="s">
-        <v>1716</v>
+        <v>1717</v>
       </c>
       <c r="B934" t="s">
-        <v>1717</v>
+        <v>1718</v>
       </c>
     </row>
     <row r="935">
       <c r="A935" t="s">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="B935" t="s">
-        <v>1719</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="936">
       <c r="A936" t="s">
-        <v>1720</v>
+        <v>1721</v>
       </c>
       <c r="B936" t="s">
-        <v>1721</v>
+        <v>1</v>
       </c>
     </row>
     <row r="937">
@@ -13319,79 +13337,79 @@
         <v>1776</v>
       </c>
       <c r="B964" t="s">
-        <v>1</v>
+        <v>1777</v>
       </c>
     </row>
     <row r="965">
       <c r="A965" t="s">
-        <v>1777</v>
+        <v>1778</v>
       </c>
       <c r="B965" t="s">
-        <v>1</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="966">
       <c r="A966" t="s">
-        <v>1778</v>
+        <v>1780</v>
       </c>
       <c r="B966" t="s">
-        <v>1</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="967">
       <c r="A967" t="s">
-        <v>1779</v>
+        <v>1782</v>
       </c>
       <c r="B967" t="s">
-        <v>1</v>
+        <v>1783</v>
       </c>
     </row>
     <row r="968">
       <c r="A968" t="s">
-        <v>1780</v>
+        <v>1784</v>
       </c>
       <c r="B968" t="s">
-        <v>1781</v>
+        <v>1785</v>
       </c>
     </row>
     <row r="969">
       <c r="A969" t="s">
-        <v>1782</v>
+        <v>1786</v>
       </c>
       <c r="B969" t="s">
-        <v>1783</v>
+        <v>1787</v>
       </c>
     </row>
     <row r="970">
       <c r="A970" t="s">
-        <v>1784</v>
+        <v>1788</v>
       </c>
       <c r="B970" t="s">
-        <v>1785</v>
+        <v>1</v>
       </c>
     </row>
     <row r="971">
       <c r="A971" t="s">
-        <v>1786</v>
+        <v>1789</v>
       </c>
       <c r="B971" t="s">
-        <v>1787</v>
+        <v>1</v>
       </c>
     </row>
     <row r="972">
       <c r="A972" t="s">
-        <v>1788</v>
+        <v>1790</v>
       </c>
       <c r="B972" t="s">
-        <v>1789</v>
+        <v>1</v>
       </c>
     </row>
     <row r="973">
       <c r="A973" t="s">
-        <v>1790</v>
+        <v>1791</v>
       </c>
       <c r="B973" t="s">
-        <v>1791</v>
+        <v>1</v>
       </c>
     </row>
     <row r="974">
@@ -13423,111 +13441,111 @@
         <v>1798</v>
       </c>
       <c r="B977" t="s">
-        <v>1</v>
+        <v>1799</v>
       </c>
     </row>
     <row r="978">
       <c r="A978" t="s">
-        <v>1799</v>
+        <v>1800</v>
       </c>
       <c r="B978" t="s">
-        <v>1800</v>
+        <v>1801</v>
       </c>
     </row>
     <row r="979">
       <c r="A979" t="s">
-        <v>1801</v>
+        <v>1802</v>
       </c>
       <c r="B979" t="s">
-        <v>1802</v>
+        <v>1803</v>
       </c>
     </row>
     <row r="980">
       <c r="A980" t="s">
-        <v>1803</v>
+        <v>1804</v>
       </c>
       <c r="B980" t="s">
-        <v>1804</v>
+        <v>1805</v>
       </c>
     </row>
     <row r="981">
       <c r="A981" t="s">
-        <v>1805</v>
+        <v>1806</v>
       </c>
       <c r="B981" t="s">
-        <v>1</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="982">
       <c r="A982" t="s">
-        <v>1806</v>
+        <v>1808</v>
       </c>
       <c r="B982" t="s">
-        <v>1807</v>
+        <v>1809</v>
       </c>
     </row>
     <row r="983">
       <c r="A983" t="s">
-        <v>1808</v>
+        <v>1810</v>
       </c>
       <c r="B983" t="s">
-        <v>1809</v>
+        <v>1</v>
       </c>
     </row>
     <row r="984">
       <c r="A984" t="s">
-        <v>1810</v>
+        <v>1811</v>
       </c>
       <c r="B984" t="s">
-        <v>1501</v>
+        <v>1812</v>
       </c>
     </row>
     <row r="985">
       <c r="A985" t="s">
-        <v>1811</v>
+        <v>1813</v>
       </c>
       <c r="B985" t="s">
-        <v>1812</v>
+        <v>1814</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" t="s">
-        <v>1813</v>
+        <v>1815</v>
       </c>
       <c r="B986" t="s">
-        <v>1814</v>
+        <v>1816</v>
       </c>
     </row>
     <row r="987">
       <c r="A987" t="s">
-        <v>1815</v>
+        <v>1817</v>
       </c>
       <c r="B987" t="s">
-        <v>1816</v>
+        <v>1</v>
       </c>
     </row>
     <row r="988">
       <c r="A988" t="s">
-        <v>1817</v>
+        <v>1818</v>
       </c>
       <c r="B988" t="s">
-        <v>1818</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="989">
       <c r="A989" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="B989" t="s">
-        <v>1820</v>
+        <v>1821</v>
       </c>
     </row>
     <row r="990">
       <c r="A990" t="s">
-        <v>1821</v>
+        <v>1822</v>
       </c>
       <c r="B990" t="s">
-        <v>1822</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="991">
@@ -13631,47 +13649,47 @@
         <v>1847</v>
       </c>
       <c r="B1003" t="s">
-        <v>1</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="1004">
       <c r="A1004" t="s">
-        <v>1848</v>
+        <v>1849</v>
       </c>
       <c r="B1004" t="s">
-        <v>1</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="1005">
       <c r="A1005" t="s">
-        <v>1849</v>
+        <v>1851</v>
       </c>
       <c r="B1005" t="s">
-        <v>1</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="1006">
       <c r="A1006" t="s">
-        <v>1850</v>
+        <v>1853</v>
       </c>
       <c r="B1006" t="s">
-        <v>1</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="1007">
       <c r="A1007" t="s">
-        <v>1851</v>
+        <v>1855</v>
       </c>
       <c r="B1007" t="s">
-        <v>1</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="1008">
       <c r="A1008" t="s">
-        <v>1852</v>
+        <v>1857</v>
       </c>
       <c r="B1008" t="s">
-        <v>1</v>
+        <v>1858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática hashcode mié abr 27 00:40:13 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -3323,7 +3323,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>15597e91a9b66aabdb7db7095ebf903a</t>
+    <t>9a040d0af7c6fe5e46c4ab2869afe01b</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -5552,7 +5552,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue may  5 00:49:42 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>7d7c824d13b0edd9eb60004046df9e4c</t>
+    <t>9a50355f3c5257dc784f15d9dbf1b536</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>1dbae929a398c0d7f341b4e0786afce1</t>
+    <t>de623e32f99f9821edfa782dd5846359</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -257,7 +257,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>839afb82a7e9f485e2d2bcb09e1883fe</t>
+    <t>b80911106de4d46b33958d9beea6a4ec</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -515,7 +515,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>321a7e2a6fcefc626b64b06976f7c6bf</t>
+    <t>44bd868d80778a5842afa4b92b62f266</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -572,7 +572,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>c1e4405a1645da86a794ce03898a9ef3</t>
+    <t>febe3f9aade4dff8d686a3c1fec9f400</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -632,7 +632,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>e77e811212818e1fe2da0f0a14ac6a46</t>
+    <t>eb4da83630f123d409d90e122a18005e</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -698,7 +698,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>3e94cd92713379db1d84781c4fd47745</t>
+    <t>00be445f4366d1a784e9729f473d9782</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -920,7 +920,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>ef95df62684b8387e6b4e1b7d48d62f7</t>
+    <t>72644e5641e091924f187a8a0560c025</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -971,7 +971,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>821b2f0c4dd2dba17d082f9e1f79c783</t>
+    <t>c8037ca7e1a08ae0d6e55fa8941e1e0a</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1601,7 +1601,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>3ce2a2e3a59fdb0bac8e2f4ae25c5bf1</t>
+    <t>33d8871cf069c8e5f3fed801317b1a30</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2681,7 +2681,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>3fefee5266c5808f908928623f67a55a</t>
+    <t>30ac241ca85fdd217430bd9640832c2b</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3647,7 +3647,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>50e430fc6f1e5a0cdf9319926e67599c</t>
+    <t>815b33e2b068336c1d3a7bf4e5e94de3</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3752,7 +3752,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>3fa36eceba0dfc3928b76a26be3a057d</t>
+    <t>5a3792f109cc4f35ab550ef6d177444c</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3788,7 +3788,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>752066aab612d792774f2a2fce61f748</t>
+    <t>96afe18bc6706b2b540d478366283729</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4424,7 +4424,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>370dd69d7dfe4dfeb0398252a0a8d6bd</t>
+    <t>9d7a7b0b6899c1c9b7d740e2e7eb4f94</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4697,7 +4697,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>39a644bc9f34ccf8a002a473f177d0a4</t>
+    <t>66e1064db415704b2a73bddc1543894e</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4766,7 +4766,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>feaf305e644a42347b28f33895da1e24</t>
+    <t>dc0a47dbf8c0035f07c88f781d1c74b8</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4991,7 +4991,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>7195fccf72f102b5b537c8c07ea25f47</t>
+    <t>46499adb5b8dab0bcaa84a1b86463358</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar may 10 00:37:36 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -881,7 +881,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>30550cba60603b3e82560b2057c0ebd5</t>
+    <t>22fae723c38c974e5b34812047b48fcc</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -908,13 +908,13 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>f63c3e94a0bfb57878e76a5916e73977</t>
+    <t>90b6f6bd227e2a29f4ec2b721661da35</t>
   </si>
   <si>
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>a4e0841b6cc8e8299c956b14c3174793</t>
+    <t>2279a0120ec4d25c495708aa908ba46a</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3107,7 +3107,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>eef484af3c5b531d7b1bf20097b06551</t>
+    <t>6695551493219b637185d0a26aef13b6</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3212,7 +3212,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>fba1c716ba7c767371b3e6a4bf556735</t>
+    <t>c569ecf812618847dc13c400ebdd663b</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3323,7 +3323,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>9a040d0af7c6fe5e46c4ab2869afe01b</t>
+    <t>e133255bbe89e6a38fb0e66828566b86</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -4349,7 +4349,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>5f917ca17136ea08a2eae9703618a5b1</t>
+    <t>9dfc0103abf18682e35d3e875c38f69f</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4688,7 +4688,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>67648602f343be1c049a646dd66e1223</t>
+    <t>78f8692a11db6e4a97b200a034ee25b7</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -5552,7 +5552,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue may 12 00:47:34 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -866,7 +866,7 @@
     <t>01-010017A</t>
   </si>
   <si>
-    <t>94e3bdce9575af42f713c012e310963c</t>
+    <t>8c426e7290c4d1f01eeb3fbf2ba62f3e</t>
   </si>
   <si>
     <t>03-030033TC</t>
@@ -1577,7 +1577,7 @@
     <t>01-080101-010112TM</t>
   </si>
   <si>
-    <t>85f7fbd715009cfab666983e3b1e6500</t>
+    <t>8c6e2b75376b8490b816902250befb49</t>
   </si>
   <si>
     <t>01-010025TP</t>
@@ -2567,7 +2567,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>132cb2ce7322a45f69527701ed8a4d23</t>
+    <t>6f604c66bf55c7354d0b02b41b484b06</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -5420,7 +5420,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>49e6a091e08e2fc592046231facaf4a0</t>
+    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
   </si>
   <si>
     <t>02-020005A</t>
@@ -5567,7 +5567,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb may 14 00:54:02 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2014" uniqueCount="1864">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2026" uniqueCount="1870">
   <si>
     <t>05-050305TM</t>
   </si>
@@ -2210,7 +2210,7 @@
     <t>01-010073A</t>
   </si>
   <si>
-    <t>24533b1fe65ce1798cd795859bc88a70</t>
+    <t>b7d115f0e0b938974dcb0716426c2780</t>
   </si>
   <si>
     <t>03-02010301-030091TP</t>
@@ -2669,7 +2669,7 @@
     <t>01-010073TP</t>
   </si>
   <si>
-    <t>47510d93d91e1f97d67c36e1a6125689</t>
+    <t>d12651c4b96f34d9614b9a796149e3b9</t>
   </si>
   <si>
     <t>05-0709-070909TC</t>
@@ -2777,7 +2777,7 @@
     <t>01-010073TC</t>
   </si>
   <si>
-    <t>67788199ba4e2e76136c9ff1c1b35f65</t>
+    <t>ce42756ec01c0727aec21745a7bd1769</t>
   </si>
   <si>
     <t>901-010202-9010102021TM</t>
@@ -5567,7 +5567,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>
@@ -5604,6 +5604,24 @@
   </si>
   <si>
     <t>a97cf78dd347585236b4e5bc9903ed0c</t>
+  </si>
+  <si>
+    <t>01-010273A</t>
+  </si>
+  <si>
+    <t>01-010173TP</t>
+  </si>
+  <si>
+    <t>01-010173TC</t>
+  </si>
+  <si>
+    <t>01-010273TC</t>
+  </si>
+  <si>
+    <t>01-010173A</t>
+  </si>
+  <si>
+    <t>01-010273TP</t>
   </si>
 </sst>
 </file>
@@ -13707,6 +13725,54 @@
         <v>1863</v>
       </c>
     </row>
+    <row r="1009">
+      <c r="A1009" t="s">
+        <v>1864</v>
+      </c>
+      <c r="B1009" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="s">
+        <v>1865</v>
+      </c>
+      <c r="B1010" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="s">
+        <v>1866</v>
+      </c>
+      <c r="B1011" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="s">
+        <v>1867</v>
+      </c>
+      <c r="B1012" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="s">
+        <v>1868</v>
+      </c>
+      <c r="B1013" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="s">
+        <v>1869</v>
+      </c>
+      <c r="B1014" t="s">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualización automática hashcode mié may 18 00:50:50 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2117,7 +2117,7 @@
     <t>03-030070TP</t>
   </si>
   <si>
-    <t>03dec063dded497e23888fd1023a6ec0</t>
+    <t>b924d191aa8e6f2ec0e5b6eb33e53617</t>
   </si>
   <si>
     <t>915-150002TP</t>
@@ -4535,7 +4535,7 @@
     <t>03-030071A</t>
   </si>
   <si>
-    <t>d6d0b2f8c75f698ee3d8d03972bdc7f0</t>
+    <t>d0fbe15fcee421c39a0783645c20ceca</t>
   </si>
   <si>
     <t>915-150010TP</t>
@@ -4616,7 +4616,7 @@
     <t>03-030070A</t>
   </si>
   <si>
-    <t>d8b1b0cf52780635fe09bb6c9e56df53</t>
+    <t>ca364509a9a7c587bb413d6ed0acb7eb</t>
   </si>
   <si>
     <t>03-02010301-030083TM</t>
@@ -5216,7 +5216,7 @@
     <t>03-030071TP</t>
   </si>
   <si>
-    <t>34f140734844fb61a075d45ac239509f</t>
+    <t>c1f338019655564a84aced240d0f078d</t>
   </si>
   <si>
     <t>915-150003TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue may 26 00:50:04 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1235,7 +1235,7 @@
     <t>03-030077TC</t>
   </si>
   <si>
-    <t>4c8664be1392de5ec5727e4fdf20f15c</t>
+    <t>62158517bbca30370868dab96e2b992c</t>
   </si>
   <si>
     <t>03-030031TC</t>
@@ -1247,7 +1247,7 @@
     <t>03-030077TM</t>
   </si>
   <si>
-    <t>32d0365fece4a049d27d8a80f7b1e0c0</t>
+    <t>0e7f38563522c7de665af7e994caed1b</t>
   </si>
   <si>
     <t>01-010023TM</t>
@@ -1289,7 +1289,7 @@
     <t>03-030077TP</t>
   </si>
   <si>
-    <t>ad0ea039ffd7104a57f2a618e4f30a1e</t>
+    <t>1ca3db9d241f5bcccd2f63e40c270371</t>
   </si>
   <si>
     <t>01-010023TP</t>
@@ -3518,7 +3518,7 @@
     <t>03-030078TC</t>
   </si>
   <si>
-    <t>d8ee6fd2518da55303cb22f636c2aba0</t>
+    <t>df6ff6b1695b7eefa42548864db43dd2</t>
   </si>
   <si>
     <t>01-010007A</t>
@@ -3548,7 +3548,7 @@
     <t>03-030078TM</t>
   </si>
   <si>
-    <t>53d7a7f55ee39ab75dcdea97b56f5baa</t>
+    <t>f3f83b5eb6fb296e2766341fbb4c0dbd</t>
   </si>
   <si>
     <t>01-010020TM</t>
@@ -3590,7 +3590,7 @@
     <t>03-030078TP</t>
   </si>
   <si>
-    <t>9050a7fb9f946dd351f41aba575a41ad</t>
+    <t>f36199d34c3f0d11ba28c925d89913d2</t>
   </si>
   <si>
     <t>01-110304-11030401TP</t>
@@ -3905,13 +3905,13 @@
     <t>03-030076TC</t>
   </si>
   <si>
-    <t>3a294ee4aacf630c0fc012cadd14abe7</t>
+    <t>de2e08bac9749604acc11641c8a0b651</t>
   </si>
   <si>
     <t>03-030076TM</t>
   </si>
   <si>
-    <t>945122acd065d03f8d8c37d0ae06971d</t>
+    <t>39de56a13264c369ba3c863ebba30c8e</t>
   </si>
   <si>
     <t>01-010022TM</t>
@@ -3971,7 +3971,7 @@
     <t>03-030076TP</t>
   </si>
   <si>
-    <t>c1777322fd937ab36d399620acb153fa</t>
+    <t>da57af880c80ea3d4159d755efcc4ca8</t>
   </si>
   <si>
     <t>05-0709-070909A</t>
@@ -4559,7 +4559,7 @@
     <t>03-030075TC</t>
   </si>
   <si>
-    <t>1dd2ae8d880542e886ef8a0209785ad8</t>
+    <t>4fb535522848c113e4e3264ba618decc</t>
   </si>
   <si>
     <t>05-050002TC</t>
@@ -4568,7 +4568,7 @@
     <t>03-030075TP</t>
   </si>
   <si>
-    <t>4275c97ed1a790378ff8d6467314d457</t>
+    <t>606f0e6a54262626e109684907854697</t>
   </si>
   <si>
     <t>03-030075TM</t>
@@ -5324,7 +5324,7 @@
     <t>03-030078A</t>
   </si>
   <si>
-    <t>a447136b3ec45cb38a753621af36b1a1</t>
+    <t>83704c9f8b0c1146eaa105f460f4e997</t>
   </si>
   <si>
     <t>03-02010301-030079A</t>
@@ -5390,7 +5390,7 @@
     <t>03-030077A</t>
   </si>
   <si>
-    <t>15b5dc4dc5faa98bb3621f26de8c466f</t>
+    <t>fd4ca97cb50e7f86a0dbc343b6cb7e49</t>
   </si>
   <si>
     <t>02-020006A</t>
@@ -5432,7 +5432,7 @@
     <t>03-030076A</t>
   </si>
   <si>
-    <t>b8e25565ac2bce670649b01b91fd4069</t>
+    <t>c19cc7bc729c576d2518fb6e0d3d8d81</t>
   </si>
   <si>
     <t>03-030052A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie may 27 00:52:18 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -296,7 +296,7 @@
     <t>01-010063TP</t>
   </si>
   <si>
-    <t>b3f7614824357fe5c8b54b6288c09e92</t>
+    <t>3b43445d9b73e0857df3f4704c4a7c85</t>
   </si>
   <si>
     <t>01-010032A</t>
@@ -314,7 +314,7 @@
     <t>01-010063TM</t>
   </si>
   <si>
-    <t>ad89823b30623527e3baef2253bbb1b1</t>
+    <t>43303048c2aafd4d83a80cd8a9b01d1e</t>
   </si>
   <si>
     <t>01-010056A</t>
@@ -461,7 +461,7 @@
     <t>01-010063TC</t>
   </si>
   <si>
-    <t>c4ba01d46b527d0a4e04edce448dd616</t>
+    <t>bcec07a141b9ca84f2d06cef73af6d4a</t>
   </si>
   <si>
     <t>905-9050607-905060702TC</t>
@@ -3161,7 +3161,7 @@
     <t>01-010064TP</t>
   </si>
   <si>
-    <t>3ca9de3c96b42ebf44712609a2faa9ac</t>
+    <t>afe0a73ee3fe2a5dcde58c5eb61b1aa5</t>
   </si>
   <si>
     <t>03-90205-0205_007A</t>
@@ -3179,7 +3179,7 @@
     <t>01-010064TM</t>
   </si>
   <si>
-    <t>d7cf3a30cc4f1877ed084f815ea8c0f3</t>
+    <t>70a1c1e76d9ab18faf663ff5e1c88184</t>
   </si>
   <si>
     <t>01-080101-010087A</t>
@@ -3359,13 +3359,13 @@
     <t>01-010064TC</t>
   </si>
   <si>
-    <t>04e4ef15c85782cf0fd57222c7efa742</t>
+    <t>219884d96e5e2d599fe6aacfce0a7c72</t>
   </si>
   <si>
     <t>01-010064A</t>
   </si>
   <si>
-    <t>819a318a42b307090b15e32fe333138c</t>
+    <t>0cb8f897ca9a686f4953b5c9d9b3b1bb</t>
   </si>
   <si>
     <t>01-010173A</t>
@@ -4574,7 +4574,7 @@
     <t>03-030075TM</t>
   </si>
   <si>
-    <t>8faee9629b60f43f0634f2f8efb568d4</t>
+    <t>e6205dbae3c37da3fd09656e4beab3e7</t>
   </si>
   <si>
     <t>01-010048TC</t>
@@ -4955,7 +4955,7 @@
     <t>01-010063A</t>
   </si>
   <si>
-    <t>43057fba58fa2f6a9cc65bd8ce502873</t>
+    <t>6f87684c836640367c3019f9a94aed56</t>
   </si>
   <si>
     <t>902-0204-02040101AA</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie jun  3 00:52:39 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>9a50355f3c5257dc784f15d9dbf1b536</t>
+    <t>8110da7db79f633b027f7f932e030822</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>de623e32f99f9821edfa782dd5846359</t>
+    <t>5302541a955be9c27aab7ef523b85948</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -260,7 +260,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>b80911106de4d46b33958d9beea6a4ec</t>
+    <t>796cdc2883e3afaba6f965a4e25db95e</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -521,7 +521,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>44bd868d80778a5842afa4b92b62f266</t>
+    <t>3abfdde57b041f94431774b3191cc97e</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -578,7 +578,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>febe3f9aade4dff8d686a3c1fec9f400</t>
+    <t>db1680d455d313ee6e835a156337b3ef</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -638,7 +638,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>eb4da83630f123d409d90e122a18005e</t>
+    <t>9eebb7e79fd18363d41e918442c3eac7</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -704,7 +704,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>00be445f4366d1a784e9729f473d9782</t>
+    <t>4ffbf58f6b35bcfb89bd267d9c07833e</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -977,7 +977,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>c8037ca7e1a08ae0d6e55fa8941e1e0a</t>
+    <t>c072110028d821dc6778f823bef06a0d</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1148,7 +1148,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>7c399ad9dd9e28c31a3fea1a3c291cd3</t>
+    <t>e1d306de0e49f71f6bcadf4c5b8b702c</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1610,7 +1610,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>33d8871cf069c8e5f3fed801317b1a30</t>
+    <t>c8fc2e258537d341ade9205a57be7ff5</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2696,7 +2696,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>30ac241ca85fdd217430bd9640832c2b</t>
+    <t>dec4548015c5a23cc6ac6a1bf37b1865</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3674,7 +3674,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>815b33e2b068336c1d3a7bf4e5e94de3</t>
+    <t>c748a606b34ae369291277cfc42ee7d1</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3779,7 +3779,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>5a3792f109cc4f35ab550ef6d177444c</t>
+    <t>8832bebc5847b016906227af8a948456</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3815,7 +3815,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>96afe18bc6706b2b540d478366283729</t>
+    <t>a58d064902a7421040128547cd497318</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4457,7 +4457,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>9d7a7b0b6899c1c9b7d740e2e7eb4f94</t>
+    <t>ae47c9251a6c3d56b0e1fc5687d651b5</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4730,7 +4730,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>66e1064db415704b2a73bddc1543894e</t>
+    <t>708ce5bbbcad729bbdcf89bb83c95293</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4799,7 +4799,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>dc0a47dbf8c0035f07c88f781d1c74b8</t>
+    <t>8e50df681af0052957873b1225e49263</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -5024,7 +5024,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>46499adb5b8dab0bcaa84a1b86463358</t>
+    <t>717d59b2dac93f9c4061d0f9a3f0a757</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue jun  9 00:51:56 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -719,7 +719,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>d259f2190eca60d125a157692e7a10b1</t>
+    <t>768ac73e6fe7d6594e38b3f2e36adb60</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -926,7 +926,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>72644e5641e091924f187a8a0560c025</t>
+    <t>2147c978fdb42f617a1a31f21f7b69b9</t>
   </si>
   <si>
     <t>05-050308A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar jun 14 00:48:44 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1514,7 +1514,7 @@
     <t>01-080101-010112TC</t>
   </si>
   <si>
-    <t>cffd45499a810de0f25ac3d2685385f7</t>
+    <t>d006b109bb014545c90f94033680364f</t>
   </si>
   <si>
     <t>01-010036TP</t>
@@ -1580,7 +1580,7 @@
     <t>01-080101-010112TM</t>
   </si>
   <si>
-    <t>8c6e2b75376b8490b816902250befb49</t>
+    <t>85f7fbd715009cfab666983e3b1e6500</t>
   </si>
   <si>
     <t>01-010025TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié jun 15 00:51:35 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1514,7 +1514,7 @@
     <t>01-080101-010112TC</t>
   </si>
   <si>
-    <t>d006b109bb014545c90f94033680364f</t>
+    <t>cffd45499a810de0f25ac3d2685385f7</t>
   </si>
   <si>
     <t>01-010036TP</t>
@@ -1580,7 +1580,7 @@
     <t>01-080101-010112TM</t>
   </si>
   <si>
-    <t>85f7fbd715009cfab666983e3b1e6500</t>
+    <t>8c6e2b75376b8490b816902250befb49</t>
   </si>
   <si>
     <t>01-010025TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié jun 22 00:51:12 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -584,7 +584,7 @@
     <t>04-040021TM</t>
   </si>
   <si>
-    <t>f82bd4a6ab8a9d362f159e5f849a581a</t>
+    <t>7e640525c55ec62c51dd50f3711e4534</t>
   </si>
   <si>
     <t>03-030047A</t>
@@ -605,7 +605,7 @@
     <t>04-040021TP</t>
   </si>
   <si>
-    <t>a6802efafda307dedca9cd91fac20dbb</t>
+    <t>512c5ce5eb6e05429fd065d7dce608fc</t>
   </si>
   <si>
     <t>01-010041TC</t>
@@ -656,7 +656,7 @@
     <t>04-040021TC</t>
   </si>
   <si>
-    <t>96925422ed8dcd6c1e4a3565680a927b</t>
+    <t>48420ca088cfb0b77f018f7e4d7cc8f0</t>
   </si>
   <si>
     <t>04-040010TM</t>
@@ -713,7 +713,7 @@
     <t>04-040014TC</t>
   </si>
   <si>
-    <t>a412ce738c555f504b3c2fc2563a4afe</t>
+    <t>700832bfaf3424f9a265472f5bf5d767</t>
   </si>
   <si>
     <t>05-050301TC</t>
@@ -953,7 +953,7 @@
     <t>04-040021A</t>
   </si>
   <si>
-    <t>256ebcd7c18287ed9edb6e1583c0bb11</t>
+    <t>4c9c6ee99ad88a416d95c37c294e3c92</t>
   </si>
   <si>
     <t>01-010016A</t>
@@ -1322,7 +1322,7 @@
     <t>04-040014TP</t>
   </si>
   <si>
-    <t>a6aa62789d57a04a889943c1037ac8a7</t>
+    <t>ad49497415b10ce433ffcf386920a777</t>
   </si>
   <si>
     <t>03-030042TC</t>
@@ -1337,7 +1337,7 @@
     <t>04-040014TM</t>
   </si>
   <si>
-    <t>492d3a39d5a70a93cd6c37e584ad93d6</t>
+    <t>09ea99858047ccf7b72437173b5439d1</t>
   </si>
   <si>
     <t>03-02010301-030089TM</t>
@@ -1907,7 +1907,7 @@
     <t>04-040018TP</t>
   </si>
   <si>
-    <t>dbdd2b7b5ee70ad0062c30d3238ed5e7</t>
+    <t>a20b2e584834e35dcb0e6388fe136ee6</t>
   </si>
   <si>
     <t>01-010027TC</t>
@@ -1979,13 +1979,13 @@
     <t>04-040018TC</t>
   </si>
   <si>
-    <t>b484710f1808ce05c7d0fc9ebf193d4c</t>
+    <t>158f05bbf80516fbeed41b7f46e86a88</t>
   </si>
   <si>
     <t>04-040018TM</t>
   </si>
   <si>
-    <t>9c7185699656b9ad00d747ef5b87ab50</t>
+    <t>318029387011428aa68c6a369d97e32f</t>
   </si>
   <si>
     <t>01-010008A</t>
@@ -3620,7 +3620,7 @@
     <t>04-040015TC</t>
   </si>
   <si>
-    <t>c45784bab07f9ac4c81fe75c5003f0b4</t>
+    <t>9003d4027669b089f69fad61020b5dbb</t>
   </si>
   <si>
     <t>04-040011A</t>
@@ -3641,7 +3641,7 @@
     <t>04-040015TP</t>
   </si>
   <si>
-    <t>813797c6f824d598032fc5179678bbef</t>
+    <t>c5c8232b2e679d9a5f8d95baf135da8c</t>
   </si>
   <si>
     <t>01-010031TC</t>
@@ -3668,7 +3668,7 @@
     <t>04-040015TM</t>
   </si>
   <si>
-    <t>db9a6243ea441b9a5d876362da809bc2</t>
+    <t>36752aebbd8c89bdfcc8152a551cfd83</t>
   </si>
   <si>
     <t>05-050302TP</t>
@@ -4388,7 +4388,7 @@
     <t>04-040019TP</t>
   </si>
   <si>
-    <t>220ad0e71abd1564eda942dee148b00d</t>
+    <t>1594c7f113fc175f3c9fc930d335094b</t>
   </si>
   <si>
     <t>05-050004TM</t>
@@ -4409,7 +4409,7 @@
     <t>04-040019A</t>
   </si>
   <si>
-    <t>7b0d26b2dbac7fdd05ccdf80f7b0b835</t>
+    <t>f67e314cfbefeed474fc438118f66f2d</t>
   </si>
   <si>
     <t>05-050004TP</t>
@@ -4427,7 +4427,7 @@
     <t>04-040019TC</t>
   </si>
   <si>
-    <t>f187797af40f51a20164c2cea7fadd3f</t>
+    <t>ed34d1d14e6014a9ffd94cc6db1738d7</t>
   </si>
   <si>
     <t>05-0709-070901TP</t>
@@ -4451,7 +4451,7 @@
     <t>04-040019TM</t>
   </si>
   <si>
-    <t>3afcec6017f53355a8786579c83ad373</t>
+    <t>d7fb88893bd1472485577a97aec747a0</t>
   </si>
   <si>
     <t>05-050102TP</t>
@@ -4523,7 +4523,7 @@
     <t>04-040018A</t>
   </si>
   <si>
-    <t>c6fce07af1576e0ff3658d91ef749868</t>
+    <t>7b989eea3b65aa2b8e12ef68ffe5082d</t>
   </si>
   <si>
     <t>04-040008TC</t>
@@ -4742,7 +4742,7 @@
     <t>04-040015A</t>
   </si>
   <si>
-    <t>426105956f2e880c1b35c2f8253edf6f</t>
+    <t>36d3415db0f4c63202fa132d04fd5858</t>
   </si>
   <si>
     <t>05-050202TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie jun 24 00:51:20 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -713,7 +713,7 @@
     <t>04-040014TC</t>
   </si>
   <si>
-    <t>700832bfaf3424f9a265472f5bf5d767</t>
+    <t>28daff3372b07e8a8c0f0b772948767b</t>
   </si>
   <si>
     <t>05-050301TC</t>
@@ -1322,7 +1322,7 @@
     <t>04-040014TP</t>
   </si>
   <si>
-    <t>ad49497415b10ce433ffcf386920a777</t>
+    <t>10488ba104b80518e11dfa1b1d64b50f</t>
   </si>
   <si>
     <t>03-030042TC</t>
@@ -1337,7 +1337,7 @@
     <t>04-040014TM</t>
   </si>
   <si>
-    <t>09ea99858047ccf7b72437173b5439d1</t>
+    <t>422905c1593772255d8ede3643059eaa</t>
   </si>
   <si>
     <t>03-02010301-030089TM</t>
@@ -4598,7 +4598,7 @@
     <t>04-040017A</t>
   </si>
   <si>
-    <t>020ff562b8d75c8031c023584adeec5d</t>
+    <t>dfc1f25dfea8c27236cdf17eda3846af</t>
   </si>
   <si>
     <t>01-010002TM</t>
@@ -4769,7 +4769,7 @@
     <t>04-040017TC</t>
   </si>
   <si>
-    <t>eca80c0354834bfc6e5c621a9c3fa38f</t>
+    <t>32299571fb6c160a7fbf6649f1403d62</t>
   </si>
   <si>
     <t>05-0709-070903TP</t>
@@ -4781,7 +4781,7 @@
     <t>04-040017TM</t>
   </si>
   <si>
-    <t>b2730936be8b224e9d9d3b14e33326ec</t>
+    <t>9c5c47e97257472e227f5aa1b6666314</t>
   </si>
   <si>
     <t>05-050104TM</t>
@@ -4793,7 +4793,7 @@
     <t>04-040017TP</t>
   </si>
   <si>
-    <t>bdc0f7f184c1ebe6336fba506f88d7d2</t>
+    <t>e5a5e4dae5493707d9dc873bb28dc1ee</t>
   </si>
   <si>
     <t>05-050104TP</t>
@@ -5585,7 +5585,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb jun 25 00:47:51 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -4829,7 +4829,7 @@
     <t>04-040014A</t>
   </si>
   <si>
-    <t>3bbeda48cc454f005a899945f7dbc5cd</t>
+    <t>3749acb03611a15ea9521216424d6903</t>
   </si>
   <si>
     <t>915-150012TC</t>
@@ -5585,7 +5585,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom jun 26 00:55:43 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -887,7 +887,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>22fae723c38c974e5b34812047b48fcc</t>
+    <t>aee5c71fa849fb66684ecec5bb0de0e3</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -920,7 +920,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>2279a0120ec4d25c495708aa908ba46a</t>
+    <t>ccb81a8ea57fc5bb809f514ad356e236</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3128,7 +3128,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>6695551493219b637185d0a26aef13b6</t>
+    <t>301210874f57c3ec8891a667b1defaae</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3236,7 +3236,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>c569ecf812618847dc13c400ebdd663b</t>
+    <t>9592128b3958525c9ab6dffba48d2a0c</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>78f8692a11db6e4a97b200a034ee25b7</t>
+    <t>fcdc02f1e3ae4dd197b04db22ecc2d1a</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar jul  5 01:24:59 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>5302541a955be9c27aab7ef523b85948</t>
+    <t>906f9c3068e972e88eed59c34e80dccb</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -704,7 +704,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>4ffbf58f6b35bcfb89bd267d9c07833e</t>
+    <t>62f828d04818a598f9a111eb112f0eed</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -719,7 +719,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>768ac73e6fe7d6594e38b3f2e36adb60</t>
+    <t>0ab213acb6493ac5de80c3f3f97d726e</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -2696,7 +2696,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>dec4548015c5a23cc6ac6a1bf37b1865</t>
+    <t>00930463a16b913ed9a6df3659e325bf</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3674,7 +3674,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>c748a606b34ae369291277cfc42ee7d1</t>
+    <t>a9d243a045c09bd59441351da8c3af06</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3779,7 +3779,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>8832bebc5847b016906227af8a948456</t>
+    <t>5b0f39b06df6d030f07643fc0af4fcd4</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3815,7 +3815,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>a58d064902a7421040128547cd497318</t>
+    <t>1218a53f5870fc794bce89973587e415</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4415,7 +4415,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>21645fb60f3090798330aaa1686e95ff</t>
+    <t>29fbdcdb04e3a16eef7eca72f61f9ec2</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4982,7 +4982,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>152445d28cf7d5a12d36b78d856d69aa</t>
+    <t>e4c9fd82b04466020ec84cd72fbe0dff</t>
   </si>
   <si>
     <t>01-010039TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié jul  6 00:52:51 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -260,7 +260,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>796cdc2883e3afaba6f965a4e25db95e</t>
+    <t>beed4f6de51592780877b63bd072ab6b</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -521,7 +521,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>3abfdde57b041f94431774b3191cc97e</t>
+    <t>87d6fbd7ab7c458ef900c506a2355818</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -578,7 +578,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>db1680d455d313ee6e835a156337b3ef</t>
+    <t>068cef265da19c2368c7c5b98829ac69</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -638,7 +638,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>9eebb7e79fd18363d41e918442c3eac7</t>
+    <t>35ba2ddc07a5f7772aba27b956d03e18</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -977,7 +977,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>c072110028d821dc6778f823bef06a0d</t>
+    <t>7c8a8dfec8634128bfbf926c4f75dd4a</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1610,7 +1610,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>c8fc2e258537d341ade9205a57be7ff5</t>
+    <t>456447a85e52790514275e5c55c941a9</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -4457,7 +4457,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>ae47c9251a6c3d56b0e1fc5687d651b5</t>
+    <t>3c37d8792356d3f56c935f69d7849b82</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4730,7 +4730,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>708ce5bbbcad729bbdcf89bb83c95293</t>
+    <t>51adef7062869d9b612cd364d17991bf</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4799,7 +4799,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>8e50df681af0052957873b1225e49263</t>
+    <t>e6f0ae27eac221ced6b00c8753c35262</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -5024,7 +5024,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>717d59b2dac93f9c4061d0f9a3f0a757</t>
+    <t>93c6b6617400571e2c863a8fa83aafd4</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb jul 30 00:48:39 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>8110da7db79f633b027f7f932e030822</t>
+    <t>578b0b54b1d675ea0e60b511eee6fe12</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -887,7 +887,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>aee5c71fa849fb66684ecec5bb0de0e3</t>
+    <t>665e5e516886685f69230bf47c68c8c1</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -3128,7 +3128,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>301210874f57c3ec8891a667b1defaae</t>
+    <t>ac8df0f190d03b3eb1374b0b8b0f9d3b</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3236,7 +3236,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>9592128b3958525c9ab6dffba48d2a0c</t>
+    <t>9ec39522a80e2ebf7c6d66a3b7b41e74</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>fcdc02f1e3ae4dd197b04db22ecc2d1a</t>
+    <t>b2a82c019a1b2f81e26c4cca5e4a19b5</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ago  3 00:52:06 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -110,7 +110,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>6b39e4d53972faa8cdeb14a543d7b258</t>
+    <t>8ead70d77545b885d65e9afbc312544b</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>906f9c3068e972e88eed59c34e80dccb</t>
+    <t>24e10f8f3e8f4a7418fdd447a1122fac</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -260,7 +260,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>beed4f6de51592780877b63bd072ab6b</t>
+    <t>4b1ec2b089b93a7dd05a6c827c1ac79c</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -521,7 +521,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>87d6fbd7ab7c458ef900c506a2355818</t>
+    <t>eae0d47411f5cf1cb8e7bdf4055c0933</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -578,7 +578,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>068cef265da19c2368c7c5b98829ac69</t>
+    <t>a1fa8524b9b5bd1580c518ad7e3b391f</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -638,7 +638,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>35ba2ddc07a5f7772aba27b956d03e18</t>
+    <t>0efff75ba4e6b5508e6525faddb490e3</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -704,7 +704,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>62f828d04818a598f9a111eb112f0eed</t>
+    <t>01c6b02a6abe9cc89304251272417524</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -977,7 +977,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>7c8a8dfec8634128bfbf926c4f75dd4a</t>
+    <t>59532101b0b46a6d0ab969e0f631d9b9</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1058,7 +1058,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>72452e70fc571abe35f60e9417bd4234</t>
+    <t>d661d0c47e28ffc24dc711433d99f0c1</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1610,7 +1610,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>456447a85e52790514275e5c55c941a9</t>
+    <t>a7a161b5e0ed558ca541eeef284d0163</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2696,7 +2696,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>00930463a16b913ed9a6df3659e325bf</t>
+    <t>3cd31da21222cb2aae5ba6089e9107e1</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3674,7 +3674,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>a9d243a045c09bd59441351da8c3af06</t>
+    <t>2b8d5436306b135e9bd106781e07acc6</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3779,7 +3779,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>5b0f39b06df6d030f07643fc0af4fcd4</t>
+    <t>445ed94267682d10523a97734310c8e9</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3815,7 +3815,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>1218a53f5870fc794bce89973587e415</t>
+    <t>e18fe0e8e75f73ed8327506724a722fd</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4457,7 +4457,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>3c37d8792356d3f56c935f69d7849b82</t>
+    <t>51862ae0db984bf051ebdf104edced21</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4730,7 +4730,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>51adef7062869d9b612cd364d17991bf</t>
+    <t>70f94e852d501067c4167c9472f9aedc</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4799,7 +4799,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>e6f0ae27eac221ced6b00c8753c35262</t>
+    <t>c645d2c53ba4940c9dfdf9324e907da0</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -5024,7 +5024,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>93c6b6617400571e2c863a8fa83aafd4</t>
+    <t>f555f7f8896f38d96d6708231275c0bd</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue ago  4 00:52:17 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -887,7 +887,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>665e5e516886685f69230bf47c68c8c1</t>
+    <t>aa9a4f6cb7e8e085ce9ca4acec207b79</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -926,7 +926,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>1c3182ad52a7cf66de529c607d27b536</t>
+    <t>75302c784f277fbe76d97b6484a5e604</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -3236,7 +3236,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>9ec39522a80e2ebf7c6d66a3b7b41e74</t>
+    <t>31d6423132f6f41e21cde34c1a5ec284</t>
   </si>
   <si>
     <t>03-030036A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie ago  5 00:47:27 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -920,7 +920,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>719ab519548de3df4ae09588adfe9521</t>
+    <t>e33f2bf0c310647b8596715a4fc7258d</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3128,7 +3128,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>ac8df0f190d03b3eb1374b0b8b0f9d3b</t>
+    <t>14d92045e4ececec2c9498eb26e47005</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>b2a82c019a1b2f81e26c4cca5e4a19b5</t>
+    <t>05a597310f8659905ca6ca8e743f45f6</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb sep  3 00:52:09 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>24e10f8f3e8f4a7418fdd447a1122fac</t>
+    <t>b5cd612d2c6dac8bb3b201207559334d</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -260,7 +260,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>4b1ec2b089b93a7dd05a6c827c1ac79c</t>
+    <t>29ba59181e5bdc227bbd88294697b7f2</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -521,7 +521,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>eae0d47411f5cf1cb8e7bdf4055c0933</t>
+    <t>d498bcf9db882e9ae0af127a2245071f</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -578,7 +578,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>a1fa8524b9b5bd1580c518ad7e3b391f</t>
+    <t>148b50439ab62b8bfaea0e62acf56be6</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -638,7 +638,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>0efff75ba4e6b5508e6525faddb490e3</t>
+    <t>c6959d8476176b4a55476e2228c5637c</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -704,7 +704,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>01c6b02a6abe9cc89304251272417524</t>
+    <t>5313f2e5d04bbcb08d1fbe231ce9b1c9</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -926,7 +926,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>75302c784f277fbe76d97b6484a5e604</t>
+    <t>17f4375a9abc216dfedc606e70853f69</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -977,7 +977,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>59532101b0b46a6d0ab969e0f631d9b9</t>
+    <t>5fbc85ea46ad8e2492e35d15b0c47d32</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1217,7 +1217,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>64e69ace98b55b09e65034d3d916d35c</t>
+    <t>dd6d80ed41c319ea1a127b8049aeeb52</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1610,7 +1610,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>a7a161b5e0ed558ca541eeef284d0163</t>
+    <t>52d5b3d2035e54b0fb26ebcf98a28a10</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2696,7 +2696,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>3cd31da21222cb2aae5ba6089e9107e1</t>
+    <t>3453f39f2ef975dc7d1a42d07a96170d</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3674,7 +3674,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>2b8d5436306b135e9bd106781e07acc6</t>
+    <t>ccf561626ed6510d1d97decf8aa73c6b</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3779,7 +3779,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>445ed94267682d10523a97734310c8e9</t>
+    <t>151986209d0e5c4f35a12219d4f38295</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3815,7 +3815,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>e18fe0e8e75f73ed8327506724a722fd</t>
+    <t>f6ffbd82ce06bc5d4c1477a19697f607</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4457,7 +4457,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>51862ae0db984bf051ebdf104edced21</t>
+    <t>7c67f8ac219000a14ec39bbf12f8a920</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4730,7 +4730,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>70f94e852d501067c4167c9472f9aedc</t>
+    <t>16afc30cfba3a355b53aba9a07164618</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4799,7 +4799,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>c645d2c53ba4940c9dfdf9324e907da0</t>
+    <t>996380681212d697ba438c35f5f09c8e</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -5024,7 +5024,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>f555f7f8896f38d96d6708231275c0bd</t>
+    <t>25ff2b47f0f204418aef98a236c47f50</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar sep  6 00:53:00 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2117,7 +2117,7 @@
     <t>03-030070TP</t>
   </si>
   <si>
-    <t>b924d191aa8e6f2ec0e5b6eb33e53617</t>
+    <t>1e352e035f59c7e4e99361f2cd7554f6</t>
   </si>
   <si>
     <t>915-150002TP</t>
@@ -3035,7 +3035,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>cbce97f245d8a2439b22aba0cbdff288</t>
+    <t>c8e6c3e5e02321b4e147a2536c543607</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -4535,7 +4535,7 @@
     <t>03-030071A</t>
   </si>
   <si>
-    <t>d0fbe15fcee421c39a0783645c20ceca</t>
+    <t>85081a218c1e29b9ea9baf916ee33db0</t>
   </si>
   <si>
     <t>915-150010TP</t>
@@ -4616,7 +4616,7 @@
     <t>03-030070A</t>
   </si>
   <si>
-    <t>ca364509a9a7c587bb413d6ed0acb7eb</t>
+    <t>092f2834a470904a92c79a60ba67fdc0</t>
   </si>
   <si>
     <t>03-02010301-030083TM</t>
@@ -5216,7 +5216,7 @@
     <t>03-030071TP</t>
   </si>
   <si>
-    <t>c1f338019655564a84aced240d0f078d</t>
+    <t>0854457b8a8f1f5ebe9928d6f9b4e91c</t>
   </si>
   <si>
     <t>915-150003TP</t>
@@ -5450,7 +5450,7 @@
     <t>02-020004A</t>
   </si>
   <si>
-    <t>1e40f44430b614f8e24ae4d804cc0702</t>
+    <t>f83d65c1b5f5a687abcd63d5956fde41</t>
   </si>
   <si>
     <t>01-010019TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié sep  7 00:51:17 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2117,7 +2117,7 @@
     <t>03-030070TP</t>
   </si>
   <si>
-    <t>1e352e035f59c7e4e99361f2cd7554f6</t>
+    <t>e821b590c7f9137aff10273be414de4f</t>
   </si>
   <si>
     <t>915-150002TP</t>
@@ -3035,7 +3035,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>c8e6c3e5e02321b4e147a2536c543607</t>
+    <t>1ca90b14630ba1351bc522a06972b37a</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -4535,7 +4535,7 @@
     <t>03-030071A</t>
   </si>
   <si>
-    <t>85081a218c1e29b9ea9baf916ee33db0</t>
+    <t>60865b06566a58e10244acf8ca2b22fe</t>
   </si>
   <si>
     <t>915-150010TP</t>
@@ -4616,7 +4616,7 @@
     <t>03-030070A</t>
   </si>
   <si>
-    <t>092f2834a470904a92c79a60ba67fdc0</t>
+    <t>db7e8967b4f4e70aea825c9a0071edce</t>
   </si>
   <si>
     <t>03-02010301-030083TM</t>
@@ -5216,7 +5216,7 @@
     <t>03-030071TP</t>
   </si>
   <si>
-    <t>0854457b8a8f1f5ebe9928d6f9b4e91c</t>
+    <t>5ad41c155ad651a63e78998a5da6c6e9</t>
   </si>
   <si>
     <t>915-150003TP</t>
@@ -5450,7 +5450,7 @@
     <t>02-020004A</t>
   </si>
   <si>
-    <t>f83d65c1b5f5a687abcd63d5956fde41</t>
+    <t>cf3c99e09bf09201cfb5dbc46e18c375</t>
   </si>
   <si>
     <t>01-010019TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue sep 22 00:47:07 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -887,7 +887,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>aa9a4f6cb7e8e085ce9ca4acec207b79</t>
+    <t>e419f033038aabfefe193dc444b4371b</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -920,7 +920,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>e33f2bf0c310647b8596715a4fc7258d</t>
+    <t>99010eb25e098bbc233ff21a84536eee</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3128,7 +3128,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>14d92045e4ececec2c9498eb26e47005</t>
+    <t>b56d9a0a982df5b5c58fc5fe45295455</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3236,7 +3236,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>31d6423132f6f41e21cde34c1a5ec284</t>
+    <t>3b51d75e547d3db94de34ea783e6cf36</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>05a597310f8659905ca6ca8e743f45f6</t>
+    <t>dc4e31b474109ba299d824e6b5ba0625</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb sep 24 00:51:31 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -416,7 +416,7 @@
     <t>01-010079A</t>
   </si>
   <si>
-    <t>140aa16de11cd594101a5aa97504261c</t>
+    <t>3eb0b87eef28e82938fc773d58eb557a</t>
   </si>
   <si>
     <t>03-030049A</t>
@@ -497,7 +497,7 @@
     <t>01-010078A</t>
   </si>
   <si>
-    <t>3fb4a87746a2cc662b3581f61a70bd67</t>
+    <t>dbb1b47fee12c374591a7a1c59f1a531</t>
   </si>
   <si>
     <t>05-0709-070952TP</t>
@@ -947,7 +947,7 @@
     <t>01-010078TC</t>
   </si>
   <si>
-    <t>71e5509fcbc85e5d13e8b15a3eb94bcf</t>
+    <t>2f205366ab7a50e275334f9659d40d01</t>
   </si>
   <si>
     <t>04-040021A</t>
@@ -2093,7 +2093,7 @@
     <t>01-010080TC</t>
   </si>
   <si>
-    <t>d90afa2f2c996bc11061075d071021ac</t>
+    <t>400adca321e5daa663f0578481c6845f</t>
   </si>
   <si>
     <t>05-0709-070910A</t>
@@ -3986,7 +3986,7 @@
     <t>01-010079TC</t>
   </si>
   <si>
-    <t>b7e998c731ad9115eec094b211d81bd9</t>
+    <t>65e90394f770266f23a5fc80aef1f658</t>
   </si>
   <si>
     <t>05-050206TC</t>
@@ -5579,7 +5579,7 @@
     <t>01-010080A</t>
   </si>
   <si>
-    <t>2e79867bc38218bf33e2beadd3d91143</t>
+    <t>43104cfb3d83ed002bf0a70980ee2446</t>
   </si>
   <si>
     <t>03-030050A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié oct  5 00:52:27 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -77,7 +77,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>8473bb76d37ee41bcc9e53d6231c34bc</t>
+    <t>21a8ec20e20ec558561a339ff341a0b8</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -260,7 +260,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>29ba59181e5bdc227bbd88294697b7f2</t>
+    <t>b9e9a771e2130168fe564b1f1843f04b</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -521,7 +521,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>d498bcf9db882e9ae0af127a2245071f</t>
+    <t>22f001efd3bcd4b2ce3cf4224c0ff980</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -578,7 +578,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>148b50439ab62b8bfaea0e62acf56be6</t>
+    <t>dd20ab2429ce23c6f9f92335436401b0</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -638,7 +638,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>c6959d8476176b4a55476e2228c5637c</t>
+    <t>99c07e6d24be62bcd842ff6ca546e1c4</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -704,7 +704,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>5313f2e5d04bbcb08d1fbe231ce9b1c9</t>
+    <t>95a0f8fa494bf7a2ef46889dcba1149e</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -977,7 +977,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>5fbc85ea46ad8e2492e35d15b0c47d32</t>
+    <t>2834892116631fd4fd85a9404170e3e1</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1610,7 +1610,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>52d5b3d2035e54b0fb26ebcf98a28a10</t>
+    <t>f25fc85a4ec4edf90250d10ce209a799</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -2696,7 +2696,7 @@
     <t>05-050313A</t>
   </si>
   <si>
-    <t>3453f39f2ef975dc7d1a42d07a96170d</t>
+    <t>5cebf5cb7bc3e5a14d4b56032a815b08</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -3779,7 +3779,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>151986209d0e5c4f35a12219d4f38295</t>
+    <t>40aaeed5a0d9deac889fbce13d42211f</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3815,7 +3815,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>f6ffbd82ce06bc5d4c1477a19697f607</t>
+    <t>0798183538bc22cc96494be30d059a42</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -4457,7 +4457,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>7c67f8ac219000a14ec39bbf12f8a920</t>
+    <t>669aa215c1d76a1d86b3203112ed9bae</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4730,7 +4730,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>16afc30cfba3a355b53aba9a07164618</t>
+    <t>a8279d7bc59d2e63e02875204e2a41cf</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4799,7 +4799,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>996380681212d697ba438c35f5f09c8e</t>
+    <t>240701a214c8af12783124d1023dde4f</t>
   </si>
   <si>
     <t>05-050202TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue oct  6 00:52:42 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -176,7 +176,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>b5cd612d2c6dac8bb3b201207559334d</t>
+    <t>f80163fce983864e25e52056cdb5c752</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -734,7 +734,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>282d21e391f9decc6fac82e8d5922dcf</t>
+    <t>bb2e1d67a243c2e6559b1aba7811bdf9</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -3674,7 +3674,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>ccf561626ed6510d1d97decf8aa73c6b</t>
+    <t>9a6a3030a02f2483dfc48ceedf2b5e12</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -5024,7 +5024,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>25ff2b47f0f204418aef98a236c47f50</t>
+    <t>957154f268102693751d9b8a6d786a8c</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb oct 15 00:47:37 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -920,7 +920,7 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>99010eb25e098bbc233ff21a84536eee</t>
+    <t>85992cff7168447573d60d1d6491a28a</t>
   </si>
   <si>
     <t>05-050105TC</t>
@@ -3128,7 +3128,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>b56d9a0a982df5b5c58fc5fe45295455</t>
+    <t>b606db288e3a2d61a565b26a0d233518</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3236,7 +3236,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>3b51d75e547d3db94de34ea783e6cf36</t>
+    <t>a5374e896926b1c31e8f628df9448547</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>dc4e31b474109ba299d824e6b5ba0625</t>
+    <t>9a11057bb930844b27b37f9f2312c34a</t>
   </si>
   <si>
     <t>05-050006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom oct 16 00:25:43 CEST 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -719,7 +719,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>83d1582a08d9eac619cb68fd115e583f</t>
+    <t>362390f2bf2549173e826597b92157be</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -3254,7 +3254,7 @@
     <t>03-030012A</t>
   </si>
   <si>
-    <t>81af3bb337018d506e033f52f46e6229</t>
+    <t>038cfcd98115521792563c7ca0e6d203</t>
   </si>
   <si>
     <t>03-030045TC</t>
@@ -3329,7 +3329,7 @@
     <t>03-030012TC</t>
   </si>
   <si>
-    <t>c343b8af9730d9b0f2a1bda9812cad00</t>
+    <t>c82ebb4fbe4601a221d01918b1aeefb9</t>
   </si>
   <si>
     <t>03-030058TC</t>
@@ -3401,7 +3401,7 @@
     <t>03-030012TP</t>
   </si>
   <si>
-    <t>ed5e5f90f4c12819871f5a7a639f3949</t>
+    <t>5cefa3c053a4cc53685a3d735e3c1b5c</t>
   </si>
   <si>
     <t>03-030058TM</t>
@@ -5438,7 +5438,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
+    <t>49e6a091e08e2fc592046231facaf4a0</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie nov  4 00:05:08 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -68,7 +68,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>3bda5ce0644e20a07a1618b28e420208</t>
+    <t>f4ebd7363fdf341d188be16318c6557b</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -80,7 +80,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>21a8ec20e20ec558561a339ff341a0b8</t>
+    <t>749c4d5b01e11705b87dc07f86479174</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>b4426fff955879dc64f8ea894a0eda69</t>
+    <t>a2494e0c8afd6151eb561d43cd6703b3</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -179,7 +179,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>f80163fce983864e25e52056cdb5c752</t>
+    <t>25448ae48cb1b031148e18100512471b</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>7d3364ab3988301c8853f45f45b5d55c</t>
+    <t>7734b6c6e69bdbde362eeee9c071be34</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -263,7 +263,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>b9e9a771e2130168fe564b1f1843f04b</t>
+    <t>bf21ff878f6269d5563b9d1fbc891e4c</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -524,7 +524,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>22f001efd3bcd4b2ce3cf4224c0ff980</t>
+    <t>d7b585ffae9bc74c244546ce4edd7aab</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -581,7 +581,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>dd20ab2429ce23c6f9f92335436401b0</t>
+    <t>5dce3c9476d8774014c46a78f1d4261d</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -641,7 +641,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>99c07e6d24be62bcd842ff6ca546e1c4</t>
+    <t>8a94a3878485d999dda16e0afcdc8353</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -707,7 +707,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>95a0f8fa494bf7a2ef46889dcba1149e</t>
+    <t>49a857d82c9444017d5325ee78433356</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -722,7 +722,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>362390f2bf2549173e826597b92157be</t>
+    <t>3598da0332312edae5a6f9eb52ffcce6</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -737,7 +737,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>bb2e1d67a243c2e6559b1aba7811bdf9</t>
+    <t>ae72e8fc2bf76620db6757bef448b55f</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -890,7 +890,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>1476a59be658fd3a49815ffd2baaf8fc</t>
+    <t>484faa10a9dc8568923bd64f21a383d6</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -917,25 +917,25 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>51718f4bd323e2909b3761b8536f3252</t>
+    <t>292ccbc5e3f692afc43161deaae08d76</t>
   </si>
   <si>
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>85992cff7168447573d60d1d6491a28a</t>
+    <t>7febf9bad5640ea7f08bbe19647ac1bd</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>b20c100e4c5e585977549b4902d420d7</t>
+    <t>4e4de5c27bfee96653623e991fc81630</t>
   </si>
   <si>
     <t>05-050308A</t>
   </si>
   <si>
-    <t>0d51ef238731df4381385fb1f4387c86</t>
+    <t>1aea05aca25e7dd68d270c505568aa6f</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -980,7 +980,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>2834892116631fd4fd85a9404170e3e1</t>
+    <t>5d275663bdc2833f8e70806a70fb33a7</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1016,7 +1016,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>38263510ef74d93da36a1d755ffb2e11</t>
+    <t>924f444090c4979da267490c5830009e</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -1061,7 +1061,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>dcbc3e27e3d2321370eed7220a5fa31e</t>
+    <t>1cc5d59a45496850d69e26a61fc7e622</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1106,7 +1106,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>aed52448adc6ee0ec526fc1e2ea7c92a</t>
+    <t>a045e3b22d16ae9daea8334b33ba5027</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>6e3b2bda1f81a34cdeafb744946a0260</t>
+    <t>b9db21f2415757c883e284460fded200</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1154,7 +1154,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>35dcb7e56936fff8eabb3a4fde41a02d</t>
+    <t>6b4eb9385d17a5c9078a032fa5c79e91</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1223,7 +1223,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>015933737427915ced5122e02e40359a</t>
+    <t>4f1a9bbbec3cdac9f29ac6b627d4ad33</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1277,7 +1277,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>baddb933d5a3596e412789c180b804ae</t>
+    <t>001c2d0cc0c344ec9cf56a3c883f3acd</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1307,7 +1307,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>7bac0c33857ef50343da215a51810365</t>
+    <t>6a27221648bc153be6950e94c156e8f4</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1319,7 +1319,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>1343055c68103a27e68f5ba35e1aa649</t>
+    <t>d6448dca68f3934dcef354f726bba244</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1607,7 +1607,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>595d2b384fd5e47fffb852ab10251d72</t>
+    <t>6c029dbb070cd899a6580427b2bd3b10</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1616,7 +1616,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>f25fc85a4ec4edf90250d10ce209a799</t>
+    <t>f9c061b5ac2bad4941f505cf609f6348</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1631,7 +1631,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>41fa35bf4eb0e4be80a3a043c8f03fe0</t>
+    <t>2ffd08fbf9a1d0616986104af8157dc2</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1748,7 +1748,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>49ee917d4779164995bd5446be45ca62</t>
+    <t>ea539a865ef9376793d880c0e3dbb7b1</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1964,7 +1964,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>cddc58b9f663c7be59581a83c199de9a</t>
+    <t>f9c5fa3a71046bdf0ee2ba95f2ac81ec</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2396,7 +2396,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>712b78cd1ded5872989a559141211c37</t>
+    <t>6aa34bbea9ce0f403f1f2bc8bfba5e84</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2615,7 +2615,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>5b235a7e7ef9f7bd82762bc682ee0e2f</t>
+    <t>fbb927790d972a25216544dadbe09f4a</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2699,13 +2699,13 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>017e55113f2268330fbed440d47e9a42</t>
+    <t>4044cd3ab60e9d55713b844842b92391</t>
   </si>
   <si>
     <t>05-050313A</t>
   </si>
   <si>
-    <t>5cebf5cb7bc3e5a14d4b56032a815b08</t>
+    <t>57ec74df81e8b524260d8b2c8a10fb5e</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2804,7 +2804,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>5ceaf36af4f156793dc0d56b6cdd4f22</t>
+    <t>991f5d3590a92e4f74f10d4255ea9d7e</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>99db28779f04593e312ddb371d2275f5</t>
+    <t>c2aec67fae0c33861e38a16bdf7a2a7e</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2936,19 +2936,19 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>379f538203e7abbf12a16f30e1c25fed</t>
+    <t>ea7053f2ee6af5313c53dfc3e828421d</t>
   </si>
   <si>
     <t>05-050311A</t>
   </si>
   <si>
-    <t>3e69ef22c3639442c18c7be66fc9d473</t>
+    <t>d764be8b88f077189caf89cc735f695f</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>3214f2514b0f1186d630925296a92721</t>
+    <t>e90112853e55f727d3f2e90ce2e0b90e</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2975,7 +2975,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>55c1078fccad956a634368981e2ad89f</t>
+    <t>6cdcf07e084365425147bf3639350134</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -3029,13 +3029,13 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>e225051aefeac8d1f6213b6d4ee6ab66</t>
+    <t>50422d561c0782997311b4c2030bdf74</t>
   </si>
   <si>
     <t>05-050203A</t>
   </si>
   <si>
-    <t>3e922d74e8104e60b44df82319dd9c70</t>
+    <t>77e5e1798fc98c2dbe6524ecfdd1697e</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -3080,7 +3080,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>3315a18da3840d607fe857975ff7b781</t>
+    <t>5f293f77ea0d257ace1a4f1e6a35bc97</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -3140,7 +3140,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>b606db288e3a2d61a565b26a0d233518</t>
+    <t>5fa62b2de11eb69ed805e0965e54cba2</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3212,7 +3212,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>ab228f4770c789809b1f961324e9f5cb</t>
+    <t>b4faf70f1e6d95e452a516c28e4e5acd</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -3230,7 +3230,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>7ac612b536babfdb981f26b30a20c82d</t>
+    <t>affe67c7266226367164c060b352c027</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3248,7 +3248,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>a5374e896926b1c31e8f628df9448547</t>
+    <t>9eb3af630895098fb96f346a837bee12</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3323,7 +3323,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>1577bc6ff21fe197afe8e260d9018b5e</t>
+    <t>bfbc39547a8e98d9d21f5736000873a8</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3359,7 +3359,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>fcd03e34c7e5558e5a547420e51c60df</t>
+    <t>830ae94e00c3824870e10eeffeb16fd2</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3611,7 +3611,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>7f83a43d1997e4ff74b55065e2202c61</t>
+    <t>86609e36109c16fc5f9b3463ad4575fc</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3686,7 +3686,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>9a6a3030a02f2483dfc48ceedf2b5e12</t>
+    <t>2c2f03f8786b60851988af41639c0357</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3791,7 +3791,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>40aaeed5a0d9deac889fbce13d42211f</t>
+    <t>fadd31cfe35aa9f11939cbc12648bc07</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3827,7 +3827,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>0798183538bc22cc96494be30d059a42</t>
+    <t>e4252a54ae9da7f30f983f3d89ad02b5</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3881,13 +3881,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>9a23ce93ad4916b6ee92fb3baee2b92b</t>
+    <t>f0d126eea9042a6e10392d5c1cfa9c2d</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>95383c6db64142a4ff89a5e72b026e10</t>
+    <t>f67a561220c08f822138968868241862</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -4109,7 +4109,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>4d93d6805a09e40e5fd8cadf925df27d</t>
+    <t>5a91ced42a90d754330b4e4c47f12f5b</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -4244,7 +4244,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>660a4be09f6eb9532bcd91139510342e</t>
+    <t>19ad7c36c3b0000ea789a1939a92d5bf</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -4316,7 +4316,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>71fe70c1019701d97de031fdcc5dd5d9</t>
+    <t>af3f8595f2be3c3b13a4ec842be1eac8</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4400,7 +4400,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>a009291efcf5dcf8609e1d4a647eb51c</t>
+    <t>4e7d4a09b66f8c4d082ea380e7e2ed03</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4433,7 +4433,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>01215243d39636e7084808aa001e3c91</t>
+    <t>067de4c48c7a626f16a999a918797c9e</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4475,7 +4475,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>669aa215c1d76a1d86b3203112ed9bae</t>
+    <t>30cba05ee4cac9a1eb75c249997463c7</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4583,7 +4583,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>aac5523a30839f4e88a411fac22632a4</t>
+    <t>cf73c2a02f83912d71e6788809bd57ab</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>851cfc4e4f3dedd6fedddea4566018d4</t>
+    <t>5ef43d346890544b85739605d26b00f5</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4745,7 +4745,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>9a11057bb930844b27b37f9f2312c34a</t>
+    <t>131631299c58d78d1370550c09a6b758</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>a8279d7bc59d2e63e02875204e2a41cf</t>
+    <t>4a88f67db1f252f24200e5dc743e03c2</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4772,7 +4772,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>c5807d127d125dc1cd1540e4ee558a85</t>
+    <t>019d7f3d10f88e3f83a51966f492bd65</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -4811,7 +4811,7 @@
     <t>05-050104TM</t>
   </si>
   <si>
-    <t>50e5f70447a9980c2d767d14b3881f1f</t>
+    <t>217b9af6cfa9c775c4217b50ddf02bec</t>
   </si>
   <si>
     <t>04-040017TP</t>
@@ -4823,7 +4823,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>240701a214c8af12783124d1023dde4f</t>
+    <t>6a34f254cb9b9fde628477b06246aa14</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>8a086330d3bb9ce52dae095640fcce00</t>
+    <t>91187be3a2d29d54101e22110c64d0be</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4892,7 +4892,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>4a97b305d1317da75f69d910c7734534</t>
+    <t>9745b16c85bbf58f544f02feb5984335</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -5003,13 +5003,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>61b167ad8f80549bb2db0301bceb1ef2</t>
+    <t>1edfb9158dc6d8e9811dd7403fa4d9bc</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>8ba2412bfdc2d91fed4a58f916b204cf</t>
+    <t>c9746bfcb75d3d2c5e6ae8dc217c9ec1</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -5051,7 +5051,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>957154f268102693751d9b8a6d786a8c</t>
+    <t>c34e45c139d8aa47c3811eb797e5723c</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5438,7 +5438,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>89e314ce418783a7a496cfa1f36db907</t>
+    <t>1bdd4f372487de4c59ea54807ee7a5d6</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom nov  6 23:55:54 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1940,7 +1940,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>8f1c79af80fbf7f5ad22c00b73d1a3af</t>
+    <t>6ae71450fc132af6fb5f002891117f4a</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -3431,7 +3431,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>c14aed93428637c86582f396bf681f7a</t>
+    <t>fb5f7bee286c6bd966eb3ed684ac6177</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb dic  3 00:10:02 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -68,7 +68,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>f4ebd7363fdf341d188be16318c6557b</t>
+    <t>3fa7e50344ef31f4d763a32d40e947d5</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -80,7 +80,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>749c4d5b01e11705b87dc07f86479174</t>
+    <t>a45e4bb36177404a595bf58f56a6ef0f</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>a2494e0c8afd6151eb561d43cd6703b3</t>
+    <t>a8f38b9afcec4da403e80cbf5c838d47</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -179,7 +179,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>25448ae48cb1b031148e18100512471b</t>
+    <t>382c599400c99cb26d7b8193cc09b408</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>7734b6c6e69bdbde362eeee9c071be34</t>
+    <t>350fe2d2a98632a4eef81ec0cf621aa3</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -263,7 +263,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>bf21ff878f6269d5563b9d1fbc891e4c</t>
+    <t>82d26b76af91af760671fb7d49f708b3</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -524,7 +524,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>d7b585ffae9bc74c244546ce4edd7aab</t>
+    <t>7fe101d6d811caa07bb6f1744c398aa7</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -581,7 +581,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>5dce3c9476d8774014c46a78f1d4261d</t>
+    <t>5a602b1a159769f01094c5f6a4d0a676</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -641,7 +641,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>8a94a3878485d999dda16e0afcdc8353</t>
+    <t>989f91b2b1bef1bd6204fc79f9225558</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -707,7 +707,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>49a857d82c9444017d5325ee78433356</t>
+    <t>60df37676a54034cddf6c42db97905a0</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -722,7 +722,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>3598da0332312edae5a6f9eb52ffcce6</t>
+    <t>4a91e42a8b292735705c73755cce06e7</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -737,7 +737,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>ae72e8fc2bf76620db6757bef448b55f</t>
+    <t>3ec63c39d82d711f0a49ec87d9372394</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -890,7 +890,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>484faa10a9dc8568923bd64f21a383d6</t>
+    <t>9e2e5a554f45cfa6e7204b19b13e1095</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -917,25 +917,25 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>292ccbc5e3f692afc43161deaae08d76</t>
+    <t>76ad3c57121674b4df93d6f148518335</t>
   </si>
   <si>
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>7febf9bad5640ea7f08bbe19647ac1bd</t>
+    <t>0842d3f35806a17668e8161d0ee656a0</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>4e4de5c27bfee96653623e991fc81630</t>
+    <t>30e6ecb456fda382a40fb490652dac08</t>
   </si>
   <si>
     <t>05-050308A</t>
   </si>
   <si>
-    <t>1aea05aca25e7dd68d270c505568aa6f</t>
+    <t>3c1764ca0b721c500c180b7e5b5cb133</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -980,7 +980,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>5d275663bdc2833f8e70806a70fb33a7</t>
+    <t>92fec99f08121b63e6b213eb27213693</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1016,7 +1016,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>924f444090c4979da267490c5830009e</t>
+    <t>5bab52f7c3c486f2267110d2834207a6</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -1061,7 +1061,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>1cc5d59a45496850d69e26a61fc7e622</t>
+    <t>0ca0d0599d59998df412130d23c03184</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1106,7 +1106,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>a045e3b22d16ae9daea8334b33ba5027</t>
+    <t>3de63092b6f34bbf6160eb6355d43c82</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>b9db21f2415757c883e284460fded200</t>
+    <t>975a9c50218d4968ca449007a5a0a6a8</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1154,7 +1154,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>6b4eb9385d17a5c9078a032fa5c79e91</t>
+    <t>8ad6ecc3e78bc477d582a359b1f3c7f1</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1223,7 +1223,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>4f1a9bbbec3cdac9f29ac6b627d4ad33</t>
+    <t>9d4a29e1bd2d6f2bb41ffcc8b761c4b2</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1277,7 +1277,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>001c2d0cc0c344ec9cf56a3c883f3acd</t>
+    <t>fd3cbeb66fd923a5c90d1e014aa0f7e0</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1307,7 +1307,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>6a27221648bc153be6950e94c156e8f4</t>
+    <t>41a352c1a9c7d61f0f63664d267ae866</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1319,7 +1319,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>d6448dca68f3934dcef354f726bba244</t>
+    <t>3bc9763b18421613e8bea65dad947fd7</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1616,7 +1616,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>f9c061b5ac2bad4941f505cf609f6348</t>
+    <t>4514346505571345ea3d991286c1de8d</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1631,7 +1631,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>2ffd08fbf9a1d0616986104af8157dc2</t>
+    <t>c300ef7bd19c2f47574dd33b09f47ef5</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1748,7 +1748,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>ea539a865ef9376793d880c0e3dbb7b1</t>
+    <t>466eae4a92f42ecffaddea3a0041eb79</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1964,7 +1964,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>f9c5fa3a71046bdf0ee2ba95f2ac81ec</t>
+    <t>1b94757c73aa42db2e5db2209eb270b1</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2699,13 +2699,13 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>4044cd3ab60e9d55713b844842b92391</t>
+    <t>b521691864f3b34b53d01a84b9c2b6a7</t>
   </si>
   <si>
     <t>05-050313A</t>
   </si>
   <si>
-    <t>57ec74df81e8b524260d8b2c8a10fb5e</t>
+    <t>d583347d6bb75c21186ec2868f9bc5f2</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2804,7 +2804,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>991f5d3590a92e4f74f10d4255ea9d7e</t>
+    <t>ebc83e42452972ea5b2c00684882ba4e</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>c2aec67fae0c33861e38a16bdf7a2a7e</t>
+    <t>01242bbd34746048971353803b336019</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2936,19 +2936,19 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>ea7053f2ee6af5313c53dfc3e828421d</t>
+    <t>ca126dd4681d497be47aea011838caed</t>
   </si>
   <si>
     <t>05-050311A</t>
   </si>
   <si>
-    <t>d764be8b88f077189caf89cc735f695f</t>
+    <t>a3f1d3830060eb7d3d51ae4a2def12cd</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>e90112853e55f727d3f2e90ce2e0b90e</t>
+    <t>ac9a405440db4f94078675575672a01e</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2975,7 +2975,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>6cdcf07e084365425147bf3639350134</t>
+    <t>84d435c7db145560ca27c9e384c75ae0</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -3029,13 +3029,13 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>50422d561c0782997311b4c2030bdf74</t>
+    <t>856d1114511949753f301e9c62d1cf0c</t>
   </si>
   <si>
     <t>05-050203A</t>
   </si>
   <si>
-    <t>77e5e1798fc98c2dbe6524ecfdd1697e</t>
+    <t>bfa3c92d1f02b235047fa7f8a13f355d</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -3080,7 +3080,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>5f293f77ea0d257ace1a4f1e6a35bc97</t>
+    <t>9842637a7cf4f420dfc0f2afe102fb63</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -3140,7 +3140,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>5fa62b2de11eb69ed805e0965e54cba2</t>
+    <t>57fbe79fdf6f9f8753dd2f5ffecf5103</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3212,7 +3212,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>b4faf70f1e6d95e452a516c28e4e5acd</t>
+    <t>94cc8352fe7b81a723b56a3032fcff02</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -3230,7 +3230,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>affe67c7266226367164c060b352c027</t>
+    <t>b50e3f5e5a7091140bb38ee2195e5123</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3248,7 +3248,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>9eb3af630895098fb96f346a837bee12</t>
+    <t>eec022ec83dee9490dee4e42169b87d2</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3359,7 +3359,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>830ae94e00c3824870e10eeffeb16fd2</t>
+    <t>6e25e01ef9310138f7abb1ba5f2a088f</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3611,7 +3611,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>86609e36109c16fc5f9b3463ad4575fc</t>
+    <t>faded04dff7baac358c61b7e4475e866</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3686,7 +3686,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>2c2f03f8786b60851988af41639c0357</t>
+    <t>dd2e8c4bd1b68cfd23b7c248861bcd42</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3791,7 +3791,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>fadd31cfe35aa9f11939cbc12648bc07</t>
+    <t>cb3ef851ae3c32d92e3436fd2dfc372a</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3827,7 +3827,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>e4252a54ae9da7f30f983f3d89ad02b5</t>
+    <t>509ff422da89da69dd2f8f8b6e971233</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3881,13 +3881,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>f0d126eea9042a6e10392d5c1cfa9c2d</t>
+    <t>1e4c1340db16bd9ba0fdd7cea585a3aa</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>f67a561220c08f822138968868241862</t>
+    <t>5e24b43e95d65e3b4f56857cb19c4e16</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -4109,7 +4109,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>5a91ced42a90d754330b4e4c47f12f5b</t>
+    <t>31056200027158b7108c9d5514bf56a2</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -4244,7 +4244,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>19ad7c36c3b0000ea789a1939a92d5bf</t>
+    <t>856dc65f9868ec6b21768e9b37aca435</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -4316,7 +4316,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>af3f8595f2be3c3b13a4ec842be1eac8</t>
+    <t>7eaa3094776d21117c0a084a9c35e0d7</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4400,7 +4400,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>4e7d4a09b66f8c4d082ea380e7e2ed03</t>
+    <t>5281e96304f9066cd68415f4c157fde7</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4475,7 +4475,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>30cba05ee4cac9a1eb75c249997463c7</t>
+    <t>5c8c0b1be42d6f3ffc3d9b843630f646</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4583,7 +4583,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>cf73c2a02f83912d71e6788809bd57ab</t>
+    <t>666097fc0899e02a9f79b61e0199c9c7</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>5ef43d346890544b85739605d26b00f5</t>
+    <t>ed64315f94319c6efd06835abaa0314a</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4745,7 +4745,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>131631299c58d78d1370550c09a6b758</t>
+    <t>76b6ff9e0b4554318539f6dbaa37a2ef</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>4a88f67db1f252f24200e5dc743e03c2</t>
+    <t>cfa129910529a26d4ee90e173f2fca7c</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4772,7 +4772,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>019d7f3d10f88e3f83a51966f492bd65</t>
+    <t>0aabf2910f682139ee3d8ca03a9d3e68</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -4811,7 +4811,7 @@
     <t>05-050104TM</t>
   </si>
   <si>
-    <t>217b9af6cfa9c775c4217b50ddf02bec</t>
+    <t>23f9bd0e4a6f472bc765801066c0a47c</t>
   </si>
   <si>
     <t>04-040017TP</t>
@@ -4823,7 +4823,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>6a34f254cb9b9fde628477b06246aa14</t>
+    <t>6ed34f4064337fc11ebac822bbf2d8c5</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>91187be3a2d29d54101e22110c64d0be</t>
+    <t>4737c01a08905bf41bdde81090bbfc03</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4892,7 +4892,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>9745b16c85bbf58f544f02feb5984335</t>
+    <t>bf4f198cc23cd1d54ccb3f1e5c4d3f3c</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -5003,13 +5003,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>1edfb9158dc6d8e9811dd7403fa4d9bc</t>
+    <t>7ea95490b52784473cd40d8b3ed31393</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>c9746bfcb75d3d2c5e6ae8dc217c9ec1</t>
+    <t>cd2b7b2e34ddc29eeb0afa910b92bbdf</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -5051,7 +5051,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>c34e45c139d8aa47c3811eb797e5723c</t>
+    <t>c83a34e208afd44c6926726ac9b04d0b</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5438,7 +5438,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>1bdd4f372487de4c59ea54807ee7a5d6</t>
+    <t>ce713e52577580de7209ebf58934681d</t>
   </si>
   <si>
     <t>05-050002TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom dic  4 23:50:36 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1940,7 +1940,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>6ae71450fc132af6fb5f002891117f4a</t>
+    <t>c64b892afee8db9a2220835c195d0496</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2396,7 +2396,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>6aa34bbea9ce0f403f1f2bc8bfba5e84</t>
+    <t>8220e6ac762dee5798a09a050e93c2fe</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2615,7 +2615,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>fbb927790d972a25216544dadbe09f4a</t>
+    <t>667553df4525200068ff28f50912407e</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -3323,7 +3323,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>bfbc39547a8e98d9d21f5736000873a8</t>
+    <t>3b5c37c77b3b579461dea776d2c43065</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3431,7 +3431,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>fb5f7bee286c6bd966eb3ed684ac6177</t>
+    <t>0faa60a459752a8eda622ab6ebd9bf78</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4433,7 +4433,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>067de4c48c7a626f16a999a918797c9e</t>
+    <t>4a2cdda1164948d4b0ab8266aa5b4112</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -5294,7 +5294,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>3316eb4d29eb45383f0f998f35573282</t>
+    <t>97223fc32ecaa11dc7f7f3e31ef94a31</t>
   </si>
   <si>
     <t>01-010006TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar dic  6 23:40:27 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -872,7 +872,7 @@
     <t>01-010017A</t>
   </si>
   <si>
-    <t>8c426e7290c4d1f01eeb3fbf2ba62f3e</t>
+    <t>94e3bdce9575af42f713c012e310963c</t>
   </si>
   <si>
     <t>03-030033TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié dic  7 23:59:38 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -872,7 +872,7 @@
     <t>01-010017A</t>
   </si>
   <si>
-    <t>94e3bdce9575af42f713c012e310963c</t>
+    <t>8c426e7290c4d1f01eeb3fbf2ba62f3e</t>
   </si>
   <si>
     <t>03-030033TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie dic  9 23:57:09 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1211,7 +1211,7 @@
     <t>01-010037A</t>
   </si>
   <si>
-    <t>fc795c55bbfe74f261482f33c8d7a73e</t>
+    <t>64ea4c3e42c23b4fb252b20df7b0e2ea</t>
   </si>
   <si>
     <t>03-030066TP</t>
@@ -4679,7 +4679,7 @@
     <t>01-010037TC</t>
   </si>
   <si>
-    <t>c53118ba7c24dc0f68dcf9bdc10a9046</t>
+    <t>3649d94c57036f9902258b739df13e97</t>
   </si>
   <si>
     <t>03-90205-0205_006TP</t>
@@ -4688,7 +4688,7 @@
     <t>01-010037TP</t>
   </si>
   <si>
-    <t>fa43e024b258256eb4b62608f1de527c</t>
+    <t>e757cf086ad2a371abf828f68cb7ef7a</t>
   </si>
   <si>
     <t>01-010037TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié dic 21 23:50:38 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2585,7 +2585,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>6f604c66bf55c7354d0b02b41b484b06</t>
+    <t>132cb2ce7322a45f69527701ed8a4d23</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -5468,7 +5468,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
+    <t>49e6a091e08e2fc592046231facaf4a0</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie dic 23 00:01:09 CET 2022
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -2585,7 +2585,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>132cb2ce7322a45f69527701ed8a4d23</t>
+    <t>6f604c66bf55c7354d0b02b41b484b06</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -5468,7 +5468,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>49e6a091e08e2fc592046231facaf4a0</t>
+    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ene  4 00:00:04 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -68,7 +68,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>3fa7e50344ef31f4d763a32d40e947d5</t>
+    <t>74757a3ab198d63460d91a8ad555ca74</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -80,7 +80,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>a45e4bb36177404a595bf58f56a6ef0f</t>
+    <t>8837dbb0ce3ba1b7cc8ce1e85ec6f397</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>a8f38b9afcec4da403e80cbf5c838d47</t>
+    <t>0d307c91eb0bdd5fc47e6f576ac8d270</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -179,7 +179,7 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>382c599400c99cb26d7b8193cc09b408</t>
+    <t>ea7df4bca281ce91279e5f4eea074d52</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>350fe2d2a98632a4eef81ec0cf621aa3</t>
+    <t>0068cde8ccb12e0ddfd3f356aa9ef836</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -737,7 +737,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>3ec63c39d82d711f0a49ec87d9372394</t>
+    <t>2cf100afeee1d4ad9ce52000a9471921</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -917,7 +917,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>76ad3c57121674b4df93d6f148518335</t>
+    <t>9d64d731b8995b31e9e54f20e50c3f0d</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -935,7 +935,7 @@
     <t>05-050308A</t>
   </si>
   <si>
-    <t>3c1764ca0b721c500c180b7e5b5cb133</t>
+    <t>1167a1b029778b1778cbe7efb39a49fb</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -1016,7 +1016,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>5bab52f7c3c486f2267110d2834207a6</t>
+    <t>cc9d782f9018120b5220f6bc199794e0</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -1061,7 +1061,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>0ca0d0599d59998df412130d23c03184</t>
+    <t>c4a0779cf5eeafc3f294c3e96702fa26</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1106,7 +1106,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>3de63092b6f34bbf6160eb6355d43c82</t>
+    <t>f51595aa8f13aaaf8ca107bc3c740b96</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>975a9c50218d4968ca449007a5a0a6a8</t>
+    <t>ad082ec4ca68d25305d3ba21321dcc56</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1154,7 +1154,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>8ad6ecc3e78bc477d582a359b1f3c7f1</t>
+    <t>a99a13264a58ed29ded4d0febfa5c85c</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1223,7 +1223,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>9d4a29e1bd2d6f2bb41ffcc8b761c4b2</t>
+    <t>b6000e92168606430770255adab62f1a</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1307,7 +1307,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>41a352c1a9c7d61f0f63664d267ae866</t>
+    <t>014575c4519c85d3480b0cb26a49d141</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1631,7 +1631,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>c300ef7bd19c2f47574dd33b09f47ef5</t>
+    <t>e5766273f1cce726119b3cd5097d3746</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1748,7 +1748,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>466eae4a92f42ecffaddea3a0041eb79</t>
+    <t>37c813352c241bb12ce5fe79bf950001</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1964,7 +1964,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>1b94757c73aa42db2e5db2209eb270b1</t>
+    <t>320e73014cd1f4e5e2a3bb64c9e46fd5</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2699,13 +2699,13 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>b521691864f3b34b53d01a84b9c2b6a7</t>
+    <t>d4812539e56ac17bd6c3f3b54513a56c</t>
   </si>
   <si>
     <t>05-050313A</t>
   </si>
   <si>
-    <t>d583347d6bb75c21186ec2868f9bc5f2</t>
+    <t>be53d3fcf1f3cd1fc1ee96a54d01c015</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2804,7 +2804,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>ebc83e42452972ea5b2c00684882ba4e</t>
+    <t>cab69b4fc87f0347bdb9fd004748d32b</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>01242bbd34746048971353803b336019</t>
+    <t>0a8d538645bb15949e2d3c4589521a60</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2936,19 +2936,19 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>ca126dd4681d497be47aea011838caed</t>
+    <t>fe171e9376fecbd517b967e834940ba0</t>
   </si>
   <si>
     <t>05-050311A</t>
   </si>
   <si>
-    <t>a3f1d3830060eb7d3d51ae4a2def12cd</t>
+    <t>1f50f2091afdd295e543e2040b0f9bec</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>ac9a405440db4f94078675575672a01e</t>
+    <t>f3bb4cb5828e87e9ceef2c0db12f13f5</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2975,7 +2975,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>84d435c7db145560ca27c9e384c75ae0</t>
+    <t>b99c67095cd9e63fb384c8c09f6b17f6</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -3035,7 +3035,7 @@
     <t>05-050203A</t>
   </si>
   <si>
-    <t>bfa3c92d1f02b235047fa7f8a13f355d</t>
+    <t>9c8b424ecde934d2877e8098b65ab290</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -3080,7 +3080,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>9842637a7cf4f420dfc0f2afe102fb63</t>
+    <t>5d2df468419f561b78a9ec7179c6c79a</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -3212,7 +3212,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>94cc8352fe7b81a723b56a3032fcff02</t>
+    <t>9534f6230a9ce0ed7ecb55135740159f</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -3230,7 +3230,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>b50e3f5e5a7091140bb38ee2195e5123</t>
+    <t>001e9bdac1fb764e8a3fcf269c90ce91</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3359,7 +3359,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>6e25e01ef9310138f7abb1ba5f2a088f</t>
+    <t>662bde8a0aec70f71afdf5f0168ed6da</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3611,7 +3611,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>faded04dff7baac358c61b7e4475e866</t>
+    <t>57def0af2ad9ee722aac7c968ae8a8aa</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3686,7 +3686,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>dd2e8c4bd1b68cfd23b7c248861bcd42</t>
+    <t>febacaf057643fbeaab274e4436af4db</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3791,7 +3791,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>cb3ef851ae3c32d92e3436fd2dfc372a</t>
+    <t>125a7a276b793fd407405c5f2358a1a6</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3827,7 +3827,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>509ff422da89da69dd2f8f8b6e971233</t>
+    <t>21ba2ec5ce86f6cd803dde8f51b19a82</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3881,13 +3881,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>1e4c1340db16bd9ba0fdd7cea585a3aa</t>
+    <t>f659e09694b30af8ab5740e0665242a6</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>5e24b43e95d65e3b4f56857cb19c4e16</t>
+    <t>91c9383ab4c19f3d94d699b21913ebe2</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -4109,7 +4109,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>31056200027158b7108c9d5514bf56a2</t>
+    <t>af38956071df966b1c0ea983283bebc4</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -4244,7 +4244,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>856dc65f9868ec6b21768e9b37aca435</t>
+    <t>032c8a2c569fb6e1669209ceff632d95</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -4316,7 +4316,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>7eaa3094776d21117c0a084a9c35e0d7</t>
+    <t>acfe405447c4b6c3bd5848389cfe585d</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4772,7 +4772,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>0aabf2910f682139ee3d8ca03a9d3e68</t>
+    <t>fae53044e74c1293d541d54aebe7f97d</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>4737c01a08905bf41bdde81090bbfc03</t>
+    <t>c742f4b7386581c5b554ff833c2c8659</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4892,7 +4892,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>bf4f198cc23cd1d54ccb3f1e5c4d3f3c</t>
+    <t>68e72f55a5c2b3099e58cd4a5940265d</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -5003,7 +5003,7 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>7ea95490b52784473cd40d8b3ed31393</t>
+    <t>48af740400793a9769593e669df7696f</t>
   </si>
   <si>
     <t>05-050002A</t>
@@ -5051,7 +5051,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>c83a34e208afd44c6926726ac9b04d0b</t>
+    <t>de59f89792c082c0195ef528c5cf8b6f</t>
   </si>
   <si>
     <t>05-050309TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ene  4 23:58:08 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -707,7 +707,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>60df37676a54034cddf6c42db97905a0</t>
+    <t>c3cd0711b4162a4071d33247b19c41ed</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -722,7 +722,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>4a91e42a8b292735705c73755cce06e7</t>
+    <t>7c2b4c1f78da1ce049c94cef983e6388</t>
   </si>
   <si>
     <t>01-010054TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié ene 11 00:02:48 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -263,7 +263,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>82d26b76af91af760671fb7d49f708b3</t>
+    <t>92ebe9f734dd9a687f862e4733ca73ab</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -524,7 +524,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>7fe101d6d811caa07bb6f1744c398aa7</t>
+    <t>0f26d93d01994c1d7f90d188812bcd2b</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -581,7 +581,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>5a602b1a159769f01094c5f6a4d0a676</t>
+    <t>be4dd03e043f8527068916697d07f630</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -641,7 +641,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>989f91b2b1bef1bd6204fc79f9225558</t>
+    <t>30aeda100e7e05bb9c0d833d7cb1ed85</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -890,7 +890,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>9e2e5a554f45cfa6e7204b19b13e1095</t>
+    <t>97cc8c11307364ed3675fbce90872e00</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -923,13 +923,13 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>0842d3f35806a17668e8161d0ee656a0</t>
+    <t>8f769252f461b20ee1fe544263130d15</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>30e6ecb456fda382a40fb490652dac08</t>
+    <t>f6a1ac26ebc45f73b3bfa354077eb7b8</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -980,7 +980,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>92fec99f08121b63e6b213eb27213693</t>
+    <t>073fa4dc897f02d77b76574130ebb954</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1277,7 +1277,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>fd3cbeb66fd923a5c90d1e014aa0f7e0</t>
+    <t>e8b31388191e19339b918056269dcbbc</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1319,7 +1319,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>3bc9763b18421613e8bea65dad947fd7</t>
+    <t>8a2a0df8c890c353a5b7fa21d8e21850</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1616,7 +1616,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>4514346505571345ea3d991286c1de8d</t>
+    <t>4e00435bb4e662a3eb66902f3ef1d94a</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1940,7 +1940,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>c64b892afee8db9a2220835c195d0496</t>
+    <t>241fec6a81eb74b4f8a3cd27171089ba</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2396,7 +2396,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>8220e6ac762dee5798a09a050e93c2fe</t>
+    <t>7130feebff75cb4901f2b3d7110d2436</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2615,7 +2615,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>667553df4525200068ff28f50912407e</t>
+    <t>c275210867d34a02ea348b9ca5783aff</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -3029,7 +3029,7 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>856d1114511949753f301e9c62d1cf0c</t>
+    <t>1ac6ecf6fac82e9c80bfc021712cc531</t>
   </si>
   <si>
     <t>05-050203A</t>
@@ -3140,7 +3140,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>57fbe79fdf6f9f8753dd2f5ffecf5103</t>
+    <t>7b921dd1d17d2e38797522ca2d0d0732</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3248,7 +3248,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>eec022ec83dee9490dee4e42169b87d2</t>
+    <t>00dfa2fd34f51cce3dee693e056442cb</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3323,7 +3323,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>3b5c37c77b3b579461dea776d2c43065</t>
+    <t>1c4bf29b0de81339363853acf2078539</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3431,7 +3431,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>0faa60a459752a8eda622ab6ebd9bf78</t>
+    <t>7de4f076836e5395d985b451fa827776</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -4400,7 +4400,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>5281e96304f9066cd68415f4c157fde7</t>
+    <t>c7d4f9d495ec449d41538804a206dac4</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4433,7 +4433,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>4a2cdda1164948d4b0ab8266aa5b4112</t>
+    <t>1bae1272e3cbfb8ebf2fbb38842bf00d</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4475,7 +4475,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>5c8c0b1be42d6f3ffc3d9b843630f646</t>
+    <t>289c4915d74e9b052fd29bf199a2b64b</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4583,7 +4583,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>666097fc0899e02a9f79b61e0199c9c7</t>
+    <t>46389d2b930154e3a122348c32335730</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>ed64315f94319c6efd06835abaa0314a</t>
+    <t>3fd3c54e0a15a356b230901cdff17881</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4745,7 +4745,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>76b6ff9e0b4554318539f6dbaa37a2ef</t>
+    <t>c9afb64b653fe7652b0e3d47a1cc1f33</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>cfa129910529a26d4ee90e173f2fca7c</t>
+    <t>253c066a9a9fefd953fd0d01e62faee6</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4811,7 +4811,7 @@
     <t>05-050104TM</t>
   </si>
   <si>
-    <t>23f9bd0e4a6f472bc765801066c0a47c</t>
+    <t>0bf1d74f90fddb6cd05ced28221e6bf8</t>
   </si>
   <si>
     <t>04-040017TP</t>
@@ -4823,7 +4823,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>6ed34f4064337fc11ebac822bbf2d8c5</t>
+    <t>d039d84896b3d2088797c920a884bbf3</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -5009,7 +5009,7 @@
     <t>05-050002A</t>
   </si>
   <si>
-    <t>cd2b7b2e34ddc29eeb0afa910b92bbdf</t>
+    <t>a45db632304111132d7e578bb9464a98</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -5294,7 +5294,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>97223fc32ecaa11dc7f7f3e31ef94a31</t>
+    <t>4f07ac426755b47b14a61696f006f962</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -5438,7 +5438,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>ce713e52577580de7209ebf58934681d</t>
+    <t>66bb415697f742311c8533a8f03d77c8</t>
   </si>
   <si>
     <t>05-050002TM</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue feb  2 00:04:37 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -191,7 +191,7 @@
     <t>05-0709-070921BTC</t>
   </si>
   <si>
-    <t>8c5f93e32e31050b3f76f0a0e7948781</t>
+    <t>1b4dcea69311e7b055b0ac1f10557629</t>
   </si>
   <si>
     <t>03-030004A</t>
@@ -257,7 +257,7 @@
     <t>05-0709-070908TC</t>
   </si>
   <si>
-    <t>88ce1735532480c72b32ef51646daa05</t>
+    <t>ec4fa821bf265258c9c3f7cdec90a2fe</t>
   </si>
   <si>
     <t>05-050105A</t>
@@ -488,7 +488,7 @@
     <t>05-0709-070952TC</t>
   </si>
   <si>
-    <t>a51f7748889faaecd4eb06c74c666900</t>
+    <t>ee7e6f6fdeb61bf10ca0d9579337518f</t>
   </si>
   <si>
     <t>01-010041TM</t>
@@ -779,7 +779,7 @@
     <t>05-0709-070954TC</t>
   </si>
   <si>
-    <t>95985cb9733b6d87c6293b5eb69488f3</t>
+    <t>57f616f5fdcfbacde4bb2feb221849c1</t>
   </si>
   <si>
     <t>04-040003TC</t>
@@ -929,7 +929,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>f6a1ac26ebc45f73b3bfa354077eb7b8</t>
+    <t>6556c02f3b6a4b066cb60cab284da968</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -1127,7 +1127,7 @@
     <t>05-0709-070910TC</t>
   </si>
   <si>
-    <t>1292de644e0e91823db29e72f7a2a593</t>
+    <t>f0aec170e5c0bb3d8a5160667d908b4a</t>
   </si>
   <si>
     <t>05-0709-070910TM</t>
@@ -1835,7 +1835,7 @@
     <t>05-0709-070902TC</t>
   </si>
   <si>
-    <t>e91a8bb3e8e757dd0d222541df0ee727</t>
+    <t>ebb0468615e604f91c2f7b173c7a09bf</t>
   </si>
   <si>
     <t>03-02010301-030097TC</t>
@@ -1970,7 +1970,7 @@
     <t>05-0709-070902TM</t>
   </si>
   <si>
-    <t>698ab646403cf6bca4514ee4f655526e</t>
+    <t>223e194bf733c3a005d4be1af189296e</t>
   </si>
   <si>
     <t>915-150009A</t>
@@ -2015,7 +2015,7 @@
     <t>05-0709-070906ATC</t>
   </si>
   <si>
-    <t>3e634d60428857b97f54e37c1e206330</t>
+    <t>8bc1abfc4b560ab776c2a2ff430e4144</t>
   </si>
   <si>
     <t>915-150013TP</t>
@@ -2222,7 +2222,7 @@
     <t>05-0709-070904TC</t>
   </si>
   <si>
-    <t>fe8de9a31d9deb0d2fa9bdd1836c8aa4</t>
+    <t>733f6ff32f55de1d261ba1cee2218418</t>
   </si>
   <si>
     <t>01-010073A</t>
@@ -2450,7 +2450,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>5b2c0d0326c47594739aa71f2adb3e6e</t>
+    <t>bcce5d7c9c4c798edadb0fb4a39f7e6e</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2693,7 +2693,7 @@
     <t>05-0709-070909TC</t>
   </si>
   <si>
-    <t>3a9669a6089f20a9d3c870fbba3cb4cc</t>
+    <t>31e70158ddcf81493d62123c0bb55551</t>
   </si>
   <si>
     <t>05-050204A</t>
@@ -3047,7 +3047,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>1ca90b14630ba1351bc522a06972b37a</t>
+    <t>513966b63122c421e1d9ec00e4957236</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -3809,7 +3809,7 @@
     <t>05-0709-070953TC</t>
   </si>
   <si>
-    <t>6525697d4f8377e1d8eae6c3a6308700</t>
+    <t>db6e075564c182138575c4db2cc6e6ba</t>
   </si>
   <si>
     <t>05-0709-070953TP</t>
@@ -4178,7 +4178,7 @@
     <t>05-0709-070955TC</t>
   </si>
   <si>
-    <t>3cb2a3fe2dbe2798f113a586cc7b1b66</t>
+    <t>a6c3fc3965f5e27ca5e82a459521d541</t>
   </si>
   <si>
     <t>03-030054TM</t>
@@ -4259,7 +4259,7 @@
     <t>05-0709-070921ATC</t>
   </si>
   <si>
-    <t>77d7c1a0f6b4aa4c63452ee3164f851b</t>
+    <t>14cfd59c9623d8233a40765b2c7d0819</t>
   </si>
   <si>
     <t>05-050207A</t>
@@ -4271,7 +4271,7 @@
     <t>02-020006TM</t>
   </si>
   <si>
-    <t>85327766952c59c3a659c3f442d5bcba</t>
+    <t>a750645b232901da9d8fd47c19707766</t>
   </si>
   <si>
     <t>902-0204-02040101BTM</t>
@@ -4334,7 +4334,7 @@
     <t>05-0709-070901TC</t>
   </si>
   <si>
-    <t>c140a13e825c462304778c0dd1cbd5d1</t>
+    <t>21f104fc9d36014e6e03049e7f10bd4e</t>
   </si>
   <si>
     <t>03-02010301-030096TC</t>
@@ -4673,7 +4673,7 @@
     <t>05-0709-070903TC</t>
   </si>
   <si>
-    <t>59dab8a7c07c3f0cee96a36884cdc7d5</t>
+    <t>ea32f4730106efd074f1d48d4359a000</t>
   </si>
   <si>
     <t>01-010037TC</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>253c066a9a9fefd953fd0d01e62faee6</t>
+    <t>63322bd12154315c4c07ef3afa084106</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -5138,7 +5138,7 @@
     <t>05-0709-070906BTC</t>
   </si>
   <si>
-    <t>0a340aa945c5c201bc628fa97d15dcfd</t>
+    <t>3700f6cfd4d1cd15f607c91913a89671</t>
   </si>
   <si>
     <t>01-010017TC</t>
@@ -5264,7 +5264,7 @@
     <t>05-0709-070905ATC</t>
   </si>
   <si>
-    <t>01df1df69a676cb2b68302ebf35e251b</t>
+    <t>1bda4e9b33f3f0b7d718c9b811444ce2</t>
   </si>
   <si>
     <t>01-010006TC</t>
@@ -5480,7 +5480,7 @@
     <t>02-020004A</t>
   </si>
   <si>
-    <t>cf3c99e09bf09201cfb5dbc46e18c375</t>
+    <t>6bb37e00f5458e4583fe793a06764b9f</t>
   </si>
   <si>
     <t>01-010019TC</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie feb  3 00:02:57 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -62,13 +62,13 @@
     <t>03-030005A</t>
   </si>
   <si>
-    <t>0169e37e3988212261d59205cf57eaf4</t>
+    <t>1aa327567c9f654b5fc4cef4f5aa509a</t>
   </si>
   <si>
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>74757a3ab198d63460d91a8ad555ca74</t>
+    <t>74fa8613314b3a5047d4330ce78c7fda</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -80,7 +80,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>8837dbb0ce3ba1b7cc8ce1e85ec6f397</t>
+    <t>093253b2bf8775922aec511e92ece479</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>0d307c91eb0bdd5fc47e6f576ac8d270</t>
+    <t>4a4dcc42b91e8609b6473b1af0d49aa5</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -179,13 +179,13 @@
     <t>05-050302A</t>
   </si>
   <si>
-    <t>ea7df4bca281ce91279e5f4eea074d52</t>
+    <t>910b082ecce2746512c30b6def806d25</t>
   </si>
   <si>
     <t>02-020005TC</t>
   </si>
   <si>
-    <t>e8db67910fb1f6d3504293c333c436bc</t>
+    <t>3fcdb28481ccee57041708ac8fcfc946</t>
   </si>
   <si>
     <t>05-0709-070921BTC</t>
@@ -197,7 +197,7 @@
     <t>03-030004A</t>
   </si>
   <si>
-    <t>5edbfa08927dfe7c01263719cfb649d7</t>
+    <t>66f6811421cf360e5a8fba1663a3c0cc</t>
   </si>
   <si>
     <t>915-150011A</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>0068cde8ccb12e0ddfd3f356aa9ef836</t>
+    <t>e33ab454cba13cd28b2dc25e32c1688f</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -263,7 +263,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>92ebe9f734dd9a687f862e4733ca73ab</t>
+    <t>75bea41c6a27691042658b9c6297a011</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -272,7 +272,7 @@
     <t>03-030003A</t>
   </si>
   <si>
-    <t>c2509abefb4d160861c68976c38e0e4b</t>
+    <t>51f0f65af68137a4e22ccd4aff53674b</t>
   </si>
   <si>
     <t>915-150010A</t>
@@ -524,7 +524,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>0f26d93d01994c1d7f90d188812bcd2b</t>
+    <t>151df40e8219f2adb6e5664643db0293</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -581,7 +581,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>be4dd03e043f8527068916697d07f630</t>
+    <t>446cd5689bf238428a9870a691bf95d8</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -641,7 +641,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>30aeda100e7e05bb9c0d833d7cb1ed85</t>
+    <t>4cd5077b6082fb87a81e4364f3a97fc8</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -707,7 +707,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>c3cd0711b4162a4071d33247b19c41ed</t>
+    <t>ce03f9a65392bb1f4a7723e5ed602b6a</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -722,7 +722,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>7c2b4c1f78da1ce049c94cef983e6388</t>
+    <t>b5ca0585bae224bb7318b2302c436dfb</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -737,7 +737,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>2cf100afeee1d4ad9ce52000a9471921</t>
+    <t>418bf58892e1570773fd838fd1a3d665</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -890,7 +890,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>97cc8c11307364ed3675fbce90872e00</t>
+    <t>4df3727990afd77367e54b2746643fe0</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -923,19 +923,19 @@
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>8f769252f461b20ee1fe544263130d15</t>
+    <t>15b741bcba61482c8e8891072d1a4395</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>6556c02f3b6a4b066cb60cab284da968</t>
+    <t>7bd9a05b033e2ae85ba6e761be718233</t>
   </si>
   <si>
     <t>05-050308A</t>
   </si>
   <si>
-    <t>1167a1b029778b1778cbe7efb39a49fb</t>
+    <t>36cb197534b28a161a857beea6a427b4</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -980,7 +980,7 @@
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>073fa4dc897f02d77b76574130ebb954</t>
+    <t>b7f8f8ba212e6c95206fc0c057751451</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1016,7 +1016,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>cc9d782f9018120b5220f6bc199794e0</t>
+    <t>5805d9657f7c365a81b64b0080622806</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -1061,7 +1061,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>c4a0779cf5eeafc3f294c3e96702fa26</t>
+    <t>7a973c8cf325fd157a239a8f1467c59d</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1106,7 +1106,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>f51595aa8f13aaaf8ca107bc3c740b96</t>
+    <t>424d1226e64b2fb5df8cf010ef85bec0</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1115,7 +1115,7 @@
     <t>03-030008A</t>
   </si>
   <si>
-    <t>d08173185aa878798c80e1af79d01b17</t>
+    <t>97b826b6fa47a086d8980f3472c701e3</t>
   </si>
   <si>
     <t>01-010014A</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>ad082ec4ca68d25305d3ba21321dcc56</t>
+    <t>ed8dbfb8c75bcf48e9120a9231052f32</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1154,7 +1154,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>a99a13264a58ed29ded4d0febfa5c85c</t>
+    <t>8b1ec063c7706c275a1c0aeea0dff766</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1202,7 +1202,7 @@
     <t>03-030007A</t>
   </si>
   <si>
-    <t>0d6bebfa0ba614499f333a9f01db471a</t>
+    <t>8b7b656d40f9247ede35398c703933c6</t>
   </si>
   <si>
     <t>786ec56dea11e219899fc3f56cae75xx</t>
@@ -1223,7 +1223,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>b6000e92168606430770255adab62f1a</t>
+    <t>6c882e6fbacbcb4e6b0573718dc299b6</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1277,7 +1277,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e8b31388191e19339b918056269dcbbc</t>
+    <t>e7903ebf39a7d843d2faeb47025cf610</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1286,7 +1286,7 @@
     <t>03-030006A</t>
   </si>
   <si>
-    <t>fbdbd89fe4c8a3e0b5263adc22dcecda</t>
+    <t>183848981187dfbfebee04d913691a1f</t>
   </si>
   <si>
     <t>05-050009TM</t>
@@ -1307,7 +1307,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>014575c4519c85d3480b0cb26a49d141</t>
+    <t>66c780f11ef0e907be41cb756ac00af5</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1319,7 +1319,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>8a2a0df8c890c353a5b7fa21d8e21850</t>
+    <t>92c36c26f5a309ed9c79cab12f216737</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1607,7 +1607,7 @@
     <t>05-050003TP</t>
   </si>
   <si>
-    <t>c41bde1e7401f2282c09c38c8d109a33</t>
+    <t>7057f19ed697ea4fb8da43e2e636de39</t>
   </si>
   <si>
     <t>01-010036TC</t>
@@ -1616,7 +1616,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>4e00435bb4e662a3eb66902f3ef1d94a</t>
+    <t>6789298f0831a72fc2874037ab900fdf</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1718,7 +1718,7 @@
     <t>03-030008TP</t>
   </si>
   <si>
-    <t>c2b0ffd73d8f0e650ecb9479fc19bdc3</t>
+    <t>56c55fd7efc60fc5510a822e15515396</t>
   </si>
   <si>
     <t>01-010025TC</t>
@@ -1736,7 +1736,7 @@
     <t>03-030072TP</t>
   </si>
   <si>
-    <t>7e401525bef9802cbb1fb418d783a0c8</t>
+    <t>6485a036b60ab533198bf814f44df652</t>
   </si>
   <si>
     <t>01-080101-010082TC</t>
@@ -1748,7 +1748,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>37c813352c241bb12ce5fe79bf950001</t>
+    <t>ec31ff71890046b6c689412fc8a5de93</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1940,7 +1940,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>241fec6a81eb74b4f8a3cd27171089ba</t>
+    <t>069541344b050b6681eb7d7cc643fe18</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -2027,7 +2027,7 @@
     <t>03-030006TC</t>
   </si>
   <si>
-    <t>78de7d0156a844a2f8b0f8580cf6bf5a</t>
+    <t>90350e10291a5d7900df87a3515605ed</t>
   </si>
   <si>
     <t>03-030006TM</t>
@@ -2048,7 +2048,7 @@
     <t>03-030006TP</t>
   </si>
   <si>
-    <t>c688fd3d455afcb71bdad83bdd5dccd8</t>
+    <t>3237b236ee0175c958fa968d615ddba5</t>
   </si>
   <si>
     <t>01-010016TM</t>
@@ -2072,7 +2072,7 @@
     <t>03-030070TC</t>
   </si>
   <si>
-    <t>4c18b1ab24b29334cb04914c575c3959</t>
+    <t>01b40c2dc9d556208fc5b7ac80f46a59</t>
   </si>
   <si>
     <t>05-0709-070906ATP</t>
@@ -2126,7 +2126,7 @@
     <t>03-030070TP</t>
   </si>
   <si>
-    <t>e821b590c7f9137aff10273be414de4f</t>
+    <t>5be30c8fdd43dd980ea5cddd94b2f49c</t>
   </si>
   <si>
     <t>915-150002TP</t>
@@ -2318,7 +2318,7 @@
     <t>03-030004TC</t>
   </si>
   <si>
-    <t>85d73053d6bd2ddfbfe94826f269c34f</t>
+    <t>509bddd30b141435625467ff7f24c4a7</t>
   </si>
   <si>
     <t>01-010018TC</t>
@@ -2351,7 +2351,7 @@
     <t>03-030004TP</t>
   </si>
   <si>
-    <t>6ba5cbfe528424fdaa8ce50b3ac4c668</t>
+    <t>3604afdb6481353116334077dce19662</t>
   </si>
   <si>
     <t>03-030004TM</t>
@@ -2426,7 +2426,7 @@
     <t>03-030015TC</t>
   </si>
   <si>
-    <t>b3c4b2fb1f0217bb6b2b3e81e013dcb9</t>
+    <t>3339f04eb82b2a48f8b987aa8fdc8bf5</t>
   </si>
   <si>
     <t>01-010007TC</t>
@@ -2462,7 +2462,7 @@
     <t>03-030015TP</t>
   </si>
   <si>
-    <t>6759f7e9b1f1f5c2c479e44ea398f3b1</t>
+    <t>b11c4eb476161140f2afdf46855d67ea</t>
   </si>
   <si>
     <t>01-080101-010086TM</t>
@@ -2699,13 +2699,13 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>d4812539e56ac17bd6c3f3b54513a56c</t>
+    <t>6824dcbff9b9b18470a696eafad3ed22</t>
   </si>
   <si>
     <t>05-050313A</t>
   </si>
   <si>
-    <t>be53d3fcf1f3cd1fc1ee96a54d01c015</t>
+    <t>ef1989b9ed4fe94a13257181ff2b5b2a</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2771,7 +2771,7 @@
     <t>03-030016A</t>
   </si>
   <si>
-    <t>02f2bd6e6d934cb7f2dec0a74c8feaa1</t>
+    <t>af2d329de32d5663c6ff40b40b73fd1b</t>
   </si>
   <si>
     <t>03-030036TP</t>
@@ -2804,7 +2804,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>cab69b4fc87f0347bdb9fd004748d32b</t>
+    <t>6cac8ff44d664cecbac54fc326f40181</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>0a8d538645bb15949e2d3c4589521a60</t>
+    <t>09fc7fc3756e43d07691bb5adbe24dc9</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2915,7 +2915,7 @@
     <t>03-030003TP</t>
   </si>
   <si>
-    <t>4885538d2619b692ce63f642a9459cd6</t>
+    <t>4b986c5753b6bcdcb40d7e8a2bde3881</t>
   </si>
   <si>
     <t>03-030049TP</t>
@@ -2936,19 +2936,19 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>fe171e9376fecbd517b967e834940ba0</t>
+    <t>57893c8170a1cc2ba69151ae3cf2baf6</t>
   </si>
   <si>
     <t>05-050311A</t>
   </si>
   <si>
-    <t>1f50f2091afdd295e543e2040b0f9bec</t>
+    <t>9d2e569c293a312882f4ae50f8ac2487</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>f3bb4cb5828e87e9ceef2c0db12f13f5</t>
+    <t>55e9ed5eed7c904073f06c23be8acf3b</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2957,13 +2957,13 @@
     <t>03-030015A</t>
   </si>
   <si>
-    <t>877e7c3d22c24d7d1914aa2aceb67ec1</t>
+    <t>8c7c89b7ef9ae576e50ca53b1b8cbd41</t>
   </si>
   <si>
     <t>03-030014TC</t>
   </si>
   <si>
-    <t>eefff1636a79415d3da7ef860713c062</t>
+    <t>ea685b6a795d9f7c0849e857d1451411</t>
   </si>
   <si>
     <t>05-0709-070904A</t>
@@ -2975,7 +2975,7 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>b99c67095cd9e63fb384c8c09f6b17f6</t>
+    <t>bd4fe69c8947ef041f3002f71a088484</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
@@ -3017,7 +3017,7 @@
     <t>03-030014TP</t>
   </si>
   <si>
-    <t>524de80c25f6a950f1045cc594eee0e7</t>
+    <t>7e2e57dd652bbec0f3ab59373e1d87b3</t>
   </si>
   <si>
     <t>05-050317TC</t>
@@ -3029,13 +3029,13 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>1ac6ecf6fac82e9c80bfc021712cc531</t>
+    <t>16d892eb89e3b8eccd413ed0fdc2e295</t>
   </si>
   <si>
     <t>05-050203A</t>
   </si>
   <si>
-    <t>9c8b424ecde934d2877e8098b65ab290</t>
+    <t>4ba3200a8ee5e1bd77d51166edc4cea4</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -3047,7 +3047,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>513966b63122c421e1d9ec00e4957236</t>
+    <t>4f8bc5cbbdd008a2e60f2f581350dffb</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -3062,7 +3062,7 @@
     <t>03-030014A</t>
   </si>
   <si>
-    <t>0f7ee37177b494487dc85696289c131e</t>
+    <t>f3854ee86e9e204a0c4d3cc0839e08c9</t>
   </si>
   <si>
     <t>03-030025TC</t>
@@ -3080,7 +3080,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>5d2df468419f561b78a9ec7179c6c79a</t>
+    <t>3b4e5365c34d2a75f2016c13abd0727b</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -3140,7 +3140,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>7b921dd1d17d2e38797522ca2d0d0732</t>
+    <t>94f5b8ddba84c7717ca6ae7a704cbe5f</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3212,7 +3212,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>9534f6230a9ce0ed7ecb55135740159f</t>
+    <t>2f5b356fa3b756c42ddc16fde5069490</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -3230,7 +3230,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>001e9bdac1fb764e8a3fcf269c90ce91</t>
+    <t>09f3d1a7411ff0ee3ed0fc08be92ca1f</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3248,7 +3248,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>00dfa2fd34f51cce3dee693e056442cb</t>
+    <t>19b5e71c9abcccb9dde06f9fd113f1fa</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3266,7 +3266,7 @@
     <t>03-030012A</t>
   </si>
   <si>
-    <t>038cfcd98115521792563c7ca0e6d203</t>
+    <t>0de5004b00ad0dbc84cccdaf989285cb</t>
   </si>
   <si>
     <t>03-030045TC</t>
@@ -3341,7 +3341,7 @@
     <t>03-030012TC</t>
   </si>
   <si>
-    <t>c82ebb4fbe4601a221d01918b1aeefb9</t>
+    <t>ba8565ff9ce84577cfa4985000870069</t>
   </si>
   <si>
     <t>03-030058TC</t>
@@ -3359,7 +3359,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>662bde8a0aec70f71afdf5f0168ed6da</t>
+    <t>e33003a15fe254e9974c06ed62bd2b9b</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3413,7 +3413,7 @@
     <t>03-030012TP</t>
   </si>
   <si>
-    <t>5cefa3c053a4cc53685a3d735e3c1b5c</t>
+    <t>16d72775f1082d9dd7521e0c4fb69dd3</t>
   </si>
   <si>
     <t>03-030058TM</t>
@@ -3431,7 +3431,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>7de4f076836e5395d985b451fa827776</t>
+    <t>679d6517ecd875770c5ac30ac133f5fc</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3611,7 +3611,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>57def0af2ad9ee722aac7c968ae8a8aa</t>
+    <t>4d04e450dbd4294233557cbf3c065cd9</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3686,7 +3686,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>febacaf057643fbeaab274e4436af4db</t>
+    <t>333380440a79efa207e42ccdee6e6a24</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3791,7 +3791,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>125a7a276b793fd407405c5f2358a1a6</t>
+    <t>711b52eb3bff41710ab4da4b34e82eaa</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3827,7 +3827,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>21ba2ec5ce86f6cd803dde8f51b19a82</t>
+    <t>8a584d0238f8a904f44e746922b31585</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3881,13 +3881,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>f659e09694b30af8ab5740e0665242a6</t>
+    <t>750f724609df41ec244169e2573685e3</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>91c9383ab4c19f3d94d699b21913ebe2</t>
+    <t>d6efa44b50598db7e91db8daa4b737e1</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -4109,7 +4109,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>af38956071df966b1c0ea983283bebc4</t>
+    <t>5369912adaba6ec20b0b0ee581b31e15</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -4244,7 +4244,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>032c8a2c569fb6e1669209ceff632d95</t>
+    <t>42ce0f8056c3dd390f5b7b8147ad97a9</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -4253,7 +4253,7 @@
     <t>02-020006TC</t>
   </si>
   <si>
-    <t>179f3f0ad5983380b4d715dcc58e6ed8</t>
+    <t>0f40f04bcc621925417d19dedb02c9eb</t>
   </si>
   <si>
     <t>05-0709-070921ATC</t>
@@ -4271,7 +4271,7 @@
     <t>02-020006TM</t>
   </si>
   <si>
-    <t>a750645b232901da9d8fd47c19707766</t>
+    <t>ff77393e28cf41a844cf4016d5a53d64</t>
   </si>
   <si>
     <t>902-0204-02040101BTM</t>
@@ -4298,7 +4298,7 @@
     <t>02-020006TP</t>
   </si>
   <si>
-    <t>16d862b5b45348824aa3b9f98f2217b8</t>
+    <t>c76eac2cc1342c48338011eb135cd913</t>
   </si>
   <si>
     <t>915-150001A</t>
@@ -4316,7 +4316,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>acfe405447c4b6c3bd5848389cfe585d</t>
+    <t>5a982386af55a6d742729e620d1c811f</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4433,13 +4433,13 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>1bae1272e3cbfb8ebf2fbb38842bf00d</t>
+    <t>a87fa5e1dd60653b4706263526353b54</t>
   </si>
   <si>
     <t>03-030072A</t>
   </si>
   <si>
-    <t>cdc7797eb778eee8606b68e60f838635</t>
+    <t>09f776c647c3a9ec5ea7fb61057f6eec</t>
   </si>
   <si>
     <t>04-040019TC</t>
@@ -4475,7 +4475,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>289c4915d74e9b052fd29bf199a2b64b</t>
+    <t>cc857f2f548c99e88ad33c1a942ab4bf</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4553,7 +4553,7 @@
     <t>03-030071A</t>
   </si>
   <si>
-    <t>60865b06566a58e10244acf8ca2b22fe</t>
+    <t>90fd7f84ec2de0f863e2ae24099664de</t>
   </si>
   <si>
     <t>915-150010TP</t>
@@ -4583,7 +4583,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>46389d2b930154e3a122348c32335730</t>
+    <t>98c72d631b07bacffb2c924ebc773aae</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4637,7 +4637,7 @@
     <t>03-030070A</t>
   </si>
   <si>
-    <t>db7e8967b4f4e70aea825c9a0071edce</t>
+    <t>f16deda779096d2f01e7c474f5c5a2bd</t>
   </si>
   <si>
     <t>03-02010301-030083TM</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>3fd3c54e0a15a356b230901cdff17881</t>
+    <t>a909007421dd2de390ceb996dda21b76</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4745,7 +4745,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>c9afb64b653fe7652b0e3d47a1cc1f33</t>
+    <t>a2992dd83e22bc7f15c931e5f1ee4853</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>63322bd12154315c4c07ef3afa084106</t>
+    <t>3cf42e69b202c6f2c19401f888dcf935</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4811,7 +4811,7 @@
     <t>05-050104TM</t>
   </si>
   <si>
-    <t>0bf1d74f90fddb6cd05ced28221e6bf8</t>
+    <t>71ded6a4fe3b064d64c4dadf702fa436</t>
   </si>
   <si>
     <t>04-040017TP</t>
@@ -4823,7 +4823,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>d039d84896b3d2088797c920a884bbf3</t>
+    <t>7f3583297e5bf75d0fc5cb0aef60b0a8</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>c742f4b7386581c5b554ff833c2c8659</t>
+    <t>51846f505a2036af7a34bd83eddab251</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4892,7 +4892,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>68e72f55a5c2b3099e58cd4a5940265d</t>
+    <t>4766dbefc02fb27e78e178e1f5fdfab7</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -5003,13 +5003,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>48af740400793a9769593e669df7696f</t>
+    <t>a69128b438702ce5b1c5f447e718de89</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>a45db632304111132d7e578bb9464a98</t>
+    <t>859448e77e2bc8ddc6531a8347e170c6</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -5051,7 +5051,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>de59f89792c082c0195ef528c5cf8b6f</t>
+    <t>09b39441b0843889e708999649d8efb6</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5150,7 +5150,7 @@
     <t>03-030007TC</t>
   </si>
   <si>
-    <t>69824790963390cecea97dd6ecd10bbd</t>
+    <t>b623c7f02a074c67597f55104a833152</t>
   </si>
   <si>
     <t>03-030060TM</t>
@@ -5225,7 +5225,7 @@
     <t>03-030007TP</t>
   </si>
   <si>
-    <t>69260edc45399a9e74fcd2b59b20a84b</t>
+    <t>1e3a55c7c38e0e54abf6538e8611cebb</t>
   </si>
   <si>
     <t>03-030055A</t>
@@ -5246,7 +5246,7 @@
     <t>03-030071TP</t>
   </si>
   <si>
-    <t>5ad41c155ad651a63e78998a5da6c6e9</t>
+    <t>814e614254481ce9d9ed3f00e0fac343</t>
   </si>
   <si>
     <t>915-150003TP</t>
@@ -5426,7 +5426,7 @@
     <t>02-020006A</t>
   </si>
   <si>
-    <t>34ed1d8adeba8de35d50444181be245d</t>
+    <t>345da6c9ac0783b1530866618a8cba4d</t>
   </si>
   <si>
     <t>03-030053A</t>
@@ -5438,7 +5438,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>66bb415697f742311c8533a8f03d77c8</t>
+    <t>a8520a0ba8fb4cc190e727b6f3675bbf</t>
   </si>
   <si>
     <t>05-050002TM</t>
@@ -5474,13 +5474,13 @@
     <t>02-020005A</t>
   </si>
   <si>
-    <t>6ae2c5c35eb4f600baf3c2fffc6ade50</t>
+    <t>c728738be7779e81e66021721a17b2e3</t>
   </si>
   <si>
     <t>02-020004A</t>
   </si>
   <si>
-    <t>6bb37e00f5458e4583fe793a06764b9f</t>
+    <t>f426715c91a1949616d434fca0c6aef7</t>
   </si>
   <si>
     <t>01-010019TC</t>
@@ -5498,7 +5498,7 @@
     <t>03-030005TC</t>
   </si>
   <si>
-    <t>51bf60829c0e2a7b1e95dd5a446cc284</t>
+    <t>401f3369c5c0cb3beaa47affc8c0d3b0</t>
   </si>
   <si>
     <t>915-150016TM</t>
@@ -5513,7 +5513,7 @@
     <t>03-030005TP</t>
   </si>
   <si>
-    <t>af22f4a95f974c28e1577a463bb81f43</t>
+    <t>74faf610777b8b037c557f80d5010d5f</t>
   </si>
   <si>
     <t>01-010019TM</t>
@@ -5579,7 +5579,7 @@
     <t>03-030016TC</t>
   </si>
   <si>
-    <t>cfd3dbf8f62cde614784deec086088dd</t>
+    <t>054397e6c1d0b1000cd97331b81b5a91</t>
   </si>
   <si>
     <t>915-150005TM</t>
@@ -5603,7 +5603,7 @@
     <t>03-030016TP</t>
   </si>
   <si>
-    <t>fee48c7deafa82713e9c9af486c3842b</t>
+    <t>5d3bfae704c277155b2be05c05796aa1</t>
   </si>
   <si>
     <t>01-010080A</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb feb  4 00:03:19 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -917,7 +917,7 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>9d64d731b8995b31e9e54f20e50c3f0d</t>
+    <t>6d1c077b514015e5376d940d89c18759</t>
   </si>
   <si>
     <t>05-050007TP</t>
@@ -1631,7 +1631,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>e5766273f1cce726119b3cd5097d3746</t>
+    <t>7b91a8aa66b1890de91217ff17e80ae7</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1964,7 +1964,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>320e73014cd1f4e5e2a3bb64c9e46fd5</t>
+    <t>524c3dd1e30ccfe1fb367287c0f6866e</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -2396,7 +2396,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>7130feebff75cb4901f2b3d7110d2436</t>
+    <t>12f231633124e4f4123cb107816595bc</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -3323,7 +3323,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>1c4bf29b0de81339363853acf2078539</t>
+    <t>2f4b69fbba4eb28d2af56a95aeac2216</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -4346,7 +4346,7 @@
     <t>05-0709-070901TM</t>
   </si>
   <si>
-    <t>ea17c22c4563d2752ae5ddea4add6cb9</t>
+    <t>7478d81de6f52608ee2450848cb17f24</t>
   </si>
   <si>
     <t>01-010035TP</t>
@@ -4400,7 +4400,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>c7d4f9d495ec449d41538804a206dac4</t>
+    <t>42346e59fadb64b493fa77241991555b</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4772,7 +4772,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>fae53044e74c1293d541d54aebe7f97d</t>
+    <t>baedf182ad6a81af57d78f57524c4106</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar feb 14 00:03:36 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -455,7 +455,7 @@
     <t>03-030001A</t>
   </si>
   <si>
-    <t>2aa1d70e294d3f855869abded550101b</t>
+    <t>7d5da48a8bd8993a5e072e01f9f50552</t>
   </si>
   <si>
     <t>05-050307TP</t>
@@ -2036,7 +2036,7 @@
     <t>02-020001TC</t>
   </si>
   <si>
-    <t>c09f637a916343cbf944a5182b0ea660</t>
+    <t>f8a26f15e725de2ffad7fd398e4ebc36</t>
   </si>
   <si>
     <t>01-010016TP</t>
@@ -2174,7 +2174,7 @@
     <t>02-020001TM</t>
   </si>
   <si>
-    <t>da5b87f6d7969e339097a5ee6c3c04ad</t>
+    <t>230310eea625cf93d0a364fc915f9f9f</t>
   </si>
   <si>
     <t>01-080101-010084TP</t>
@@ -2210,7 +2210,7 @@
     <t>02-020001TP</t>
   </si>
   <si>
-    <t>1df16c9e277baf30a157cee4dca37275</t>
+    <t>c181a1804835600ccdf575836d3605c9</t>
   </si>
   <si>
     <t>03-02010301-030091TC</t>
@@ -2837,7 +2837,7 @@
     <t>03-030001TC</t>
   </si>
   <si>
-    <t>d1020ec2c5dafea497bf49ab17c149e7</t>
+    <t>89da1243052404e75116934c786c8225</t>
   </si>
   <si>
     <t>03-030047TC</t>
@@ -3302,7 +3302,7 @@
     <t>03-030001TM</t>
   </si>
   <si>
-    <t>040783e3155e41ea714a9b89a3277a28</t>
+    <t>dacba0ac388b68747b3f9afc77083791</t>
   </si>
   <si>
     <t>05-050308TC</t>
@@ -3329,7 +3329,7 @@
     <t>03-030001TP</t>
   </si>
   <si>
-    <t>7aa025559d8c2585f33a4b2adc895bc1</t>
+    <t>006308c3222980d07f5df84ae06a7e4c</t>
   </si>
   <si>
     <t>03-030047TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom feb 19 23:39:38 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar feb 21 00:01:27 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié mar  1 00:05:22 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -68,7 +68,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>74fa8613314b3a5047d4330ce78c7fda</t>
+    <t>d0d1156c0d1209bc7f556fe90eb4c545</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -185,13 +185,13 @@
     <t>02-020005TC</t>
   </si>
   <si>
-    <t>3fcdb28481ccee57041708ac8fcfc946</t>
+    <t>1b758c59bdf5310ac7ddf6a7aa8d8a20</t>
   </si>
   <si>
     <t>05-0709-070921BTC</t>
   </si>
   <si>
-    <t>1b4dcea69311e7b055b0ac1f10557629</t>
+    <t>5bfd40fb7fc280aaa714254894c47bba</t>
   </si>
   <si>
     <t>03-030004A</t>
@@ -257,7 +257,7 @@
     <t>05-0709-070908TC</t>
   </si>
   <si>
-    <t>ec4fa821bf265258c9c3f7cdec90a2fe</t>
+    <t>e7280369bec73f344ac204675f3ed28c</t>
   </si>
   <si>
     <t>05-050105A</t>
@@ -338,7 +338,7 @@
     <t>05-0709-070908TM</t>
   </si>
   <si>
-    <t>5825b7d3596921e31aca9320332509b2</t>
+    <t>b09ab385410ab6519f2c5c01b0d8e8d4</t>
   </si>
   <si>
     <t>03-030026A</t>
@@ -488,7 +488,7 @@
     <t>05-0709-070952TC</t>
   </si>
   <si>
-    <t>ee7e6f6fdeb61bf10ca0d9579337518f</t>
+    <t>8dddd0fd620bce146d55133f82e739e5</t>
   </si>
   <si>
     <t>01-010041TM</t>
@@ -671,7 +671,7 @@
     <t>01-010076TC</t>
   </si>
   <si>
-    <t>d273e51e74591f574e39b504f15525d6</t>
+    <t>3577972e62ceaf98b52d565e9006cb3c</t>
   </si>
   <si>
     <t>03-030046A</t>
@@ -722,7 +722,7 @@
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>b5ca0585bae224bb7318b2302c436dfb</t>
+    <t>2f77ef0d2fe746a94be600df5c842543</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -779,7 +779,7 @@
     <t>05-0709-070954TC</t>
   </si>
   <si>
-    <t>57f616f5fdcfbacde4bb2feb221849c1</t>
+    <t>672e231ce856a7699d969f2f02ad1fe5</t>
   </si>
   <si>
     <t>04-040003TC</t>
@@ -890,7 +890,7 @@
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>4df3727990afd77367e54b2746643fe0</t>
+    <t>5c1ce96e0672a894c7d1503ae1e2ee33</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -929,7 +929,7 @@
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>7bd9a05b033e2ae85ba6e761be718233</t>
+    <t>59f26dfbf1210f82e8a0cbdec574cd6a</t>
   </si>
   <si>
     <t>05-050308A</t>
@@ -1127,13 +1127,13 @@
     <t>05-0709-070910TC</t>
   </si>
   <si>
-    <t>f0aec170e5c0bb3d8a5160667d908b4a</t>
+    <t>3b13b77e1ba7650bd966fe990ef71644</t>
   </si>
   <si>
     <t>05-0709-070910TM</t>
   </si>
   <si>
-    <t>9d53101d83aec8012af958899f8f2dd8</t>
+    <t>ae4025a4e458212368bd492f3e3f1b67</t>
   </si>
   <si>
     <t>01-010045TP</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>ed8dbfb8c75bcf48e9120a9231052f32</t>
+    <t>3041c0e03b385af85d993d9797ef8f50</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1241,7 +1241,7 @@
     <t>03-030077TC</t>
   </si>
   <si>
-    <t>62158517bbca30370868dab96e2b992c</t>
+    <t>8c681427d8a8bdfef77fbf94f81522cf</t>
   </si>
   <si>
     <t>03-030031TC</t>
@@ -1277,7 +1277,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>e7903ebf39a7d843d2faeb47025cf610</t>
+    <t>60941dd009ad6aaf73fc845f8e779b79</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1631,7 +1631,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>7b91a8aa66b1890de91217ff17e80ae7</t>
+    <t>48a29a74bd1d19a8d71958ea4775a844</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1835,7 +1835,7 @@
     <t>05-0709-070902TC</t>
   </si>
   <si>
-    <t>ebb0468615e604f91c2f7b173c7a09bf</t>
+    <t>f7be0b1f684977c506f4fde0fe3e417a</t>
   </si>
   <si>
     <t>03-02010301-030097TC</t>
@@ -2015,7 +2015,7 @@
     <t>05-0709-070906ATC</t>
   </si>
   <si>
-    <t>8bc1abfc4b560ab776c2a2ff430e4144</t>
+    <t>451cdc8e7e60f577abc056f972a86f53</t>
   </si>
   <si>
     <t>915-150013TP</t>
@@ -2027,7 +2027,7 @@
     <t>03-030006TC</t>
   </si>
   <si>
-    <t>90350e10291a5d7900df87a3515605ed</t>
+    <t>a928fe8ac33bf810a2c142803df9e543</t>
   </si>
   <si>
     <t>03-030006TM</t>
@@ -2066,13 +2066,13 @@
     <t>05-0709-070906ATM</t>
   </si>
   <si>
-    <t>8cc5a4d99bf226aa2995aa0d14699b32</t>
+    <t>41a860e496fa1c7c4b580ccce6b3de8e</t>
   </si>
   <si>
     <t>03-030070TC</t>
   </si>
   <si>
-    <t>01b40c2dc9d556208fc5b7ac80f46a59</t>
+    <t>1220a3a43569268e941ca1211248a9cc</t>
   </si>
   <si>
     <t>05-0709-070906ATP</t>
@@ -2222,7 +2222,7 @@
     <t>05-0709-070904TC</t>
   </si>
   <si>
-    <t>733f6ff32f55de1d261ba1cee2218418</t>
+    <t>e9e0c9633698ab6f31af882f3aa87554</t>
   </si>
   <si>
     <t>01-010073A</t>
@@ -2276,7 +2276,7 @@
     <t>05-0709-070904TM</t>
   </si>
   <si>
-    <t>e9716c23cd2b38929b66696199d804ab</t>
+    <t>6e38df94a15d4148e51554dbcd58600c</t>
   </si>
   <si>
     <t>01-010029TP</t>
@@ -2318,7 +2318,7 @@
     <t>03-030004TC</t>
   </si>
   <si>
-    <t>509bddd30b141435625467ff7f24c4a7</t>
+    <t>b1139d944a1fc002195b196a4da7598e</t>
   </si>
   <si>
     <t>01-010018TC</t>
@@ -2396,7 +2396,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>12f231633124e4f4123cb107816595bc</t>
+    <t>95faf70c272e0c86f38d79c662cfe83e</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2426,7 +2426,7 @@
     <t>03-030015TC</t>
   </si>
   <si>
-    <t>3339f04eb82b2a48f8b987aa8fdc8bf5</t>
+    <t>c1da0b46f4ad9a774bb7ac6a00ee3a3b</t>
   </si>
   <si>
     <t>01-010007TC</t>
@@ -2450,7 +2450,7 @@
     <t>05-0709-070905BTC</t>
   </si>
   <si>
-    <t>bcce5d7c9c4c798edadb0fb4a39f7e6e</t>
+    <t>dc9a2ed5a3d6cb3550d0c98cb1647661</t>
   </si>
   <si>
     <t>01-010007TM</t>
@@ -2693,7 +2693,7 @@
     <t>05-0709-070909TC</t>
   </si>
   <si>
-    <t>31e70158ddcf81493d62123c0bb55551</t>
+    <t>8f8eae294fa42e1517163b922b5ae8c4</t>
   </si>
   <si>
     <t>05-050204A</t>
@@ -2963,7 +2963,7 @@
     <t>03-030014TC</t>
   </si>
   <si>
-    <t>ea685b6a795d9f7c0849e857d1451411</t>
+    <t>7698970169376a49b577d1110b892dd0</t>
   </si>
   <si>
     <t>05-0709-070904A</t>
@@ -3047,7 +3047,7 @@
     <t>02-020004TC</t>
   </si>
   <si>
-    <t>4f8bc5cbbdd008a2e60f2f581350dffb</t>
+    <t>e3c110e7f7e0a23a661b2c406884f4a0</t>
   </si>
   <si>
     <t>901-010202-9010102021A</t>
@@ -3341,7 +3341,7 @@
     <t>03-030012TC</t>
   </si>
   <si>
-    <t>ba8565ff9ce84577cfa4985000870069</t>
+    <t>019a16a26a35ea2cb721460980e7da64</t>
   </si>
   <si>
     <t>03-030058TC</t>
@@ -3530,7 +3530,7 @@
     <t>03-030078TC</t>
   </si>
   <si>
-    <t>df6ff6b1695b7eefa42548864db43dd2</t>
+    <t>81cf198796557ca8b33bd82d4943e53c</t>
   </si>
   <si>
     <t>01-010007A</t>
@@ -3626,7 +3626,7 @@
     <t>01-010077TC</t>
   </si>
   <si>
-    <t>1aca8a6dd32b3e7d0123260f78fa0ad0</t>
+    <t>c897e47c581bbf801f0723d4a131b5f3</t>
   </si>
   <si>
     <t>04-040015TC</t>
@@ -3809,7 +3809,7 @@
     <t>05-0709-070953TC</t>
   </si>
   <si>
-    <t>db6e075564c182138575c4db2cc6e6ba</t>
+    <t>8bb2da2353fe098265ba073cf6d533f7</t>
   </si>
   <si>
     <t>05-0709-070953TP</t>
@@ -3827,7 +3827,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>8a584d0238f8a904f44e746922b31585</t>
+    <t>a0434bd934177faeff6d69a08937a7f0</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3917,7 +3917,7 @@
     <t>03-030076TC</t>
   </si>
   <si>
-    <t>de2e08bac9749604acc11641c8a0b651</t>
+    <t>06d7e7a5cd07f02126e971aba46eabd9</t>
   </si>
   <si>
     <t>03-030076TM</t>
@@ -4178,7 +4178,7 @@
     <t>05-0709-070955TC</t>
   </si>
   <si>
-    <t>a6c3fc3965f5e27ca5e82a459521d541</t>
+    <t>e593bfc60934c54749f1a9e8804d63dc</t>
   </si>
   <si>
     <t>03-030054TM</t>
@@ -4259,7 +4259,7 @@
     <t>05-0709-070921ATC</t>
   </si>
   <si>
-    <t>14cfd59c9623d8233a40765b2c7d0819</t>
+    <t>c77e688dcb662b21bbe8030648b208a0</t>
   </si>
   <si>
     <t>05-050207A</t>
@@ -4334,7 +4334,7 @@
     <t>05-0709-070901TC</t>
   </si>
   <si>
-    <t>21f104fc9d36014e6e03049e7f10bd4e</t>
+    <t>269f229c212b2374e74688859011a13d</t>
   </si>
   <si>
     <t>03-02010301-030096TC</t>
@@ -4400,7 +4400,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>42346e59fadb64b493fa77241991555b</t>
+    <t>dd19106b6296b94fbe2beff96f8b6904</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4577,13 +4577,13 @@
     <t>03-030075TC</t>
   </si>
   <si>
-    <t>4fb535522848c113e4e3264ba618decc</t>
+    <t>b3798ef9ab5db9680bdc354b51881249</t>
   </si>
   <si>
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>98c72d631b07bacffb2c924ebc773aae</t>
+    <t>292ac7fc92e0b9bcb8b8e74b63cdd9a3</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4673,7 +4673,7 @@
     <t>05-0709-070903TC</t>
   </si>
   <si>
-    <t>ea32f4730106efd074f1d48d4359a000</t>
+    <t>c1b6ecf546b927cb406f17ac71de9754</t>
   </si>
   <si>
     <t>01-010037TC</t>
@@ -4721,7 +4721,7 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>a909007421dd2de390ceb996dda21b76</t>
+    <t>33e9ab2941bf742b5c51dd3d8c1c4d71</t>
   </si>
   <si>
     <t>01-010026TC</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>3cf42e69b202c6f2c19401f888dcf935</t>
+    <t>2e91159c4e9e881bcad80bfed883f9c0</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4778,7 +4778,7 @@
     <t>05-0709-070903TM</t>
   </si>
   <si>
-    <t>8d80d2d73cc5f33a32758b3a83592ca5</t>
+    <t>298c528aeda213f18e28ab043ae8fbca</t>
   </si>
   <si>
     <t>03-02010301-030093A</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>51846f505a2036af7a34bd83eddab251</t>
+    <t>f7ace73729e01af1ea1690b5b3e48612</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -5003,7 +5003,7 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>a69128b438702ce5b1c5f447e718de89</t>
+    <t>188b27af421fe22a0e14d932b7ee19c6</t>
   </si>
   <si>
     <t>05-050002A</t>
@@ -5138,7 +5138,7 @@
     <t>05-0709-070906BTC</t>
   </si>
   <si>
-    <t>3700f6cfd4d1cd15f607c91913a89671</t>
+    <t>d2d580b87f58ae626b10adacb40529d5</t>
   </si>
   <si>
     <t>01-010017TC</t>
@@ -5150,7 +5150,7 @@
     <t>03-030007TC</t>
   </si>
   <si>
-    <t>b623c7f02a074c67597f55104a833152</t>
+    <t>36f5fcc743522ac06301aca8ba323599</t>
   </si>
   <si>
     <t>03-030060TM</t>
@@ -5264,7 +5264,7 @@
     <t>05-0709-070905ATC</t>
   </si>
   <si>
-    <t>1bda4e9b33f3f0b7d718c9b811444ce2</t>
+    <t>32d21c245b8ce615a5ed3d800bb36348</t>
   </si>
   <si>
     <t>01-010006TC</t>
@@ -5498,7 +5498,7 @@
     <t>03-030005TC</t>
   </si>
   <si>
-    <t>401f3369c5c0cb3beaa47affc8c0d3b0</t>
+    <t>58ec5de2881c0ef81a5df3db136480b4</t>
   </si>
   <si>
     <t>915-150016TM</t>
@@ -5579,7 +5579,7 @@
     <t>03-030016TC</t>
   </si>
   <si>
-    <t>054397e6c1d0b1000cd97331b81b5a91</t>
+    <t>185ef5d2120d0dcabe80935f55628928</t>
   </si>
   <si>
     <t>915-150005TM</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie mar  3 00:10:51 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -68,7 +68,7 @@
     <t>05-050305TC</t>
   </si>
   <si>
-    <t>d0d1156c0d1209bc7f556fe90eb4c545</t>
+    <t>5c7a600fdacd23fe2364184c53f54203</t>
   </si>
   <si>
     <t>03-030002TM</t>
@@ -80,7 +80,7 @@
     <t>05-050301A</t>
   </si>
   <si>
-    <t>093253b2bf8775922aec511e92ece479</t>
+    <t>ce5c1f8498c39d4b347c4884a7c8bb0a</t>
   </si>
   <si>
     <t>03-030002TP</t>
@@ -98,7 +98,7 @@
     <t>01-010061TC</t>
   </si>
   <si>
-    <t>8b1882bbbc790866be7a7bea221940bc</t>
+    <t>d0bf281948bd62d2d0cb8099956d70c5</t>
   </si>
   <si>
     <t>05-050207TP</t>
@@ -113,7 +113,7 @@
     <t>05-050305TP</t>
   </si>
   <si>
-    <t>4a4dcc42b91e8609b6473b1af0d49aa5</t>
+    <t>052c16c16dc1093248dd8991fd89e7db</t>
   </si>
   <si>
     <t>05-0709-070921BTP</t>
@@ -173,13 +173,13 @@
     <t>01-010050TC</t>
   </si>
   <si>
-    <t>f701fc6735e33393ae9dfc09dc1f862b</t>
+    <t>636b4cd48e8fad4bc2c96db508c00037</t>
   </si>
   <si>
     <t>05-050302A</t>
   </si>
   <si>
-    <t>910b082ecce2746512c30b6def806d25</t>
+    <t>2597d288dc99a436f6f305f8be926ddc</t>
   </si>
   <si>
     <t>02-020005TC</t>
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>e33ab454cba13cd28b2dc25e32c1688f</t>
+    <t>472edfaa05e1207d58533aec747cc1a0</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -263,7 +263,7 @@
     <t>05-050105A</t>
   </si>
   <si>
-    <t>75bea41c6a27691042658b9c6297a011</t>
+    <t>626d565dfdbc5f3af46c60567ddc1231</t>
   </si>
   <si>
     <t>902-0204-02040102BTC</t>
@@ -350,7 +350,7 @@
     <t>03-030002TC</t>
   </si>
   <si>
-    <t>72c746904bc6a3638b39bd2bcc1d99fb</t>
+    <t>f981c1a875be79ee51b5a62935f1b902</t>
   </si>
   <si>
     <t>05-0709-070908TP</t>
@@ -464,13 +464,13 @@
     <t>01-010063TC</t>
   </si>
   <si>
-    <t>bcec07a141b9ca84f2d06cef73af6d4a</t>
+    <t>f57f4324ef04cf0d6cd8ea51e09fc488</t>
   </si>
   <si>
     <t>905-9050607-905060702TC</t>
   </si>
   <si>
-    <t>bc13665eac829680b6a0efac910209a9</t>
+    <t>f265a37417ad0a741fddde5c172bc94b</t>
   </si>
   <si>
     <t>01-010030A</t>
@@ -524,7 +524,7 @@
     <t>05-050104A</t>
   </si>
   <si>
-    <t>151df40e8219f2adb6e5664643db0293</t>
+    <t>e5dc30ffcac1695191528620477cfd00</t>
   </si>
   <si>
     <t>03-030068TC</t>
@@ -536,7 +536,7 @@
     <t>01-010052TC</t>
   </si>
   <si>
-    <t>1b294182deb035c333b2c1fdfcb81713</t>
+    <t>0b8327f1edc9831d15798018c6597512</t>
   </si>
   <si>
     <t>01-010030TP</t>
@@ -581,7 +581,7 @@
     <t>05-050101A</t>
   </si>
   <si>
-    <t>446cd5689bf238428a9870a691bf95d8</t>
+    <t>68aba33c85f15f839937ab7b317c38e7</t>
   </si>
   <si>
     <t>04-040021TM</t>
@@ -614,7 +614,7 @@
     <t>01-010041TC</t>
   </si>
   <si>
-    <t>eb0d0a04fa5b89eaecfbf421c3d8c654</t>
+    <t>b9c3a30747235a94799c8fd975144d13</t>
   </si>
   <si>
     <t>01-010052A</t>
@@ -641,7 +641,7 @@
     <t>05-050102A</t>
   </si>
   <si>
-    <t>4cd5077b6082fb87a81e4364f3a97fc8</t>
+    <t>f06ac3c9f0d3c932494a3a8222e8d12d</t>
   </si>
   <si>
     <t>03-030035TP</t>
@@ -659,7 +659,7 @@
     <t>04-040021TC</t>
   </si>
   <si>
-    <t>48420ca088cfb0b77f018f7e4d7cc8f0</t>
+    <t>2b0d44209a5c2ca87d46b9524af27188</t>
   </si>
   <si>
     <t>04-040010TM</t>
@@ -695,7 +695,7 @@
     <t>01-010030TC</t>
   </si>
   <si>
-    <t>b16bc7b0749f43703e0dc648c43512c1</t>
+    <t>af7afd18e60cd20713b395a54af8134e</t>
   </si>
   <si>
     <t>01-010054TM</t>
@@ -707,7 +707,7 @@
     <t>05-050301TP</t>
   </si>
   <si>
-    <t>ce03f9a65392bb1f4a7723e5ed602b6a</t>
+    <t>44d807560b2d896c6c5311813c2d4c05</t>
   </si>
   <si>
     <t>05-050301TM</t>
@@ -716,13 +716,13 @@
     <t>04-040014TC</t>
   </si>
   <si>
-    <t>28daff3372b07e8a8c0f0b772948767b</t>
+    <t>830272fb9addb937ce2908eabdfcd4c3</t>
   </si>
   <si>
     <t>05-050301TC</t>
   </si>
   <si>
-    <t>2f77ef0d2fe746a94be600df5c842543</t>
+    <t>2e478bf70e14807c221af5a346b4878d</t>
   </si>
   <si>
     <t>01-010054TP</t>
@@ -737,7 +737,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>418bf58892e1570773fd838fd1a3d665</t>
+    <t>c36cfa08576bd03193194588c36f0f45</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -785,7 +785,7 @@
     <t>04-040003TC</t>
   </si>
   <si>
-    <t>86dad47776a536a2722d208725462fe9</t>
+    <t>af9892c91dc441d51d737c6b06f63a75</t>
   </si>
   <si>
     <t>05-050312TC</t>
@@ -812,7 +812,7 @@
     <t>01-010054TC</t>
   </si>
   <si>
-    <t>0ffb287847436932184298721cb34355</t>
+    <t>7e934e39e425ad272b435a07c4f8d377</t>
   </si>
   <si>
     <t>01-110304-11030402A</t>
@@ -884,13 +884,13 @@
     <t>01-010043TC</t>
   </si>
   <si>
-    <t>e7b56bcf0d89e5e16dceb6f97a42f1f9</t>
+    <t>f33b10e34220b882063ece3d497ad1b1</t>
   </si>
   <si>
     <t>05-050007TC</t>
   </si>
   <si>
-    <t>5c1ce96e0672a894c7d1503ae1e2ee33</t>
+    <t>fb53d3cdcd7ea4176b61bbc97045cb54</t>
   </si>
   <si>
     <t>01-110304-11030402TC</t>
@@ -917,25 +917,25 @@
     <t>05-050203TP</t>
   </si>
   <si>
-    <t>6d1c077b514015e5376d940d89c18759</t>
+    <t>087d38d9333308b15402be81293d5fba</t>
   </si>
   <si>
     <t>05-050007TP</t>
   </si>
   <si>
-    <t>15b741bcba61482c8e8891072d1a4395</t>
+    <t>722c8937d4210d50ec047ec1bd8dfb45</t>
   </si>
   <si>
     <t>05-050105TC</t>
   </si>
   <si>
-    <t>59f26dfbf1210f82e8a0cbdec574cd6a</t>
+    <t>3a2a1a04f08eaf35add64f77019a2179</t>
   </si>
   <si>
     <t>05-050308A</t>
   </si>
   <si>
-    <t>36cb197534b28a161a857beea6a427b4</t>
+    <t>2010fc36d9e004ba5ec19162138d97b0</t>
   </si>
   <si>
     <t>05-050203TM</t>
@@ -950,7 +950,7 @@
     <t>01-010078TC</t>
   </si>
   <si>
-    <t>2f205366ab7a50e275334f9659d40d01</t>
+    <t>7fe675d30e938720e15b4adf13fc89da</t>
   </si>
   <si>
     <t>04-040021A</t>
@@ -974,13 +974,13 @@
     <t>01-010032TC</t>
   </si>
   <si>
-    <t>6cb11ea575974fd674255c7ac68bc67e</t>
+    <t>9e8a391204e50f744e4eef730f9b9d73</t>
   </si>
   <si>
     <t>05-050105TP</t>
   </si>
   <si>
-    <t>b7f8f8ba212e6c95206fc0c057751451</t>
+    <t>2e5f33e8f068bf388fe852a333a2f6a7</t>
   </si>
   <si>
     <t>05-050203TC</t>
@@ -1016,7 +1016,7 @@
     <t>05-050303TP</t>
   </si>
   <si>
-    <t>5805d9657f7c365a81b64b0080622806</t>
+    <t>b1ba32eca9138b8cb3789ab4ba6b7d16</t>
   </si>
   <si>
     <t>03-030042TM</t>
@@ -1061,7 +1061,7 @@
     <t>05-050305A</t>
   </si>
   <si>
-    <t>7a973c8cf325fd157a239a8f1467c59d</t>
+    <t>2f86b8c248e288fe052f496cff16c55f</t>
   </si>
   <si>
     <t>04-040001TM</t>
@@ -1106,7 +1106,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>424d1226e64b2fb5df8cf010ef85bec0</t>
+    <t>76194b402ea30878c498724d6f3da001</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>3041c0e03b385af85d993d9797ef8f50</t>
+    <t>26e8df35c47b1349b814821cfaf34b26</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1154,7 +1154,7 @@
     <t>05-050306A</t>
   </si>
   <si>
-    <t>8b1ec063c7706c275a1c0aeea0dff766</t>
+    <t>5d73ea6ec1b6fbdc0b5f536fbd0c8238</t>
   </si>
   <si>
     <t>902-0204-02040102STP</t>
@@ -1169,7 +1169,7 @@
     <t>01-010056TC</t>
   </si>
   <si>
-    <t>1a49785ca7a983cca90a64e4bf74ea5e</t>
+    <t>bddc1b88cdc357d2dced3f4bf74029e2</t>
   </si>
   <si>
     <t>902-0204-02040101ATM</t>
@@ -1223,7 +1223,7 @@
     <t>05-050303A</t>
   </si>
   <si>
-    <t>6c882e6fbacbcb4e6b0573718dc299b6</t>
+    <t>df201de87f8162bb5f86bd3271c79b00</t>
   </si>
   <si>
     <t>05-0709-070910TP</t>
@@ -1235,7 +1235,7 @@
     <t>01-010045TC</t>
   </si>
   <si>
-    <t>161ae6edf106a7bc11dfb812c98f99d1</t>
+    <t>c3672406d5388e4c6350a231bed4cb7e</t>
   </si>
   <si>
     <t>03-030077TC</t>
@@ -1277,7 +1277,7 @@
     <t>05-050009TC</t>
   </si>
   <si>
-    <t>60941dd009ad6aaf73fc845f8e779b79</t>
+    <t>41a2e94e6f73ae06cd1b17d3b32f3465</t>
   </si>
   <si>
     <t>01-010036A</t>
@@ -1307,7 +1307,7 @@
     <t>05-050205TP</t>
   </si>
   <si>
-    <t>66c780f11ef0e907be41cb756ac00af5</t>
+    <t>4f0fae1d6df1031e626607cf5c3ebc73</t>
   </si>
   <si>
     <t>05-050304A</t>
@@ -1319,7 +1319,7 @@
     <t>05-050009TP</t>
   </si>
   <si>
-    <t>92c36c26f5a309ed9c79cab12f216737</t>
+    <t>23c07aea132fcb3bbf89862587005a08</t>
   </si>
   <si>
     <t>05-050205TM</t>
@@ -1409,7 +1409,7 @@
     <t>01-010023TC</t>
   </si>
   <si>
-    <t>7851cdb2ec1c4372dc796e7f313a34f0</t>
+    <t>c48188195dc6175208cfc76710feb755</t>
   </si>
   <si>
     <t>03-02010301-030086A</t>
@@ -1499,7 +1499,7 @@
     <t>01-010058TC</t>
   </si>
   <si>
-    <t>57acc88878f713687f6372ed12a22320</t>
+    <t>eedf595dfb845a52a2d577e9140366b6</t>
   </si>
   <si>
     <t>01-080101-010091TC</t>
@@ -1568,7 +1568,7 @@
     <t>01-010047TC</t>
   </si>
   <si>
-    <t>3e1fd2d2ccd1f1e2bed32ba5728c6491</t>
+    <t>8761ccf1f473e5486764506adec6ddf1</t>
   </si>
   <si>
     <t>01-080101-010112TP</t>
@@ -1616,7 +1616,7 @@
     <t>05-050101TP</t>
   </si>
   <si>
-    <t>6789298f0831a72fc2874037ab900fdf</t>
+    <t>4355077ab94e7998992992bcddcb672d</t>
   </si>
   <si>
     <t>03-030063TC</t>
@@ -1631,7 +1631,7 @@
     <t>05-050201TC</t>
   </si>
   <si>
-    <t>48a29a74bd1d19a8d71958ea4775a844</t>
+    <t>38bfe0c1a3a1a68bac0680e8c08bbdd1</t>
   </si>
   <si>
     <t>03-030061TP</t>
@@ -1724,7 +1724,7 @@
     <t>01-010025TC</t>
   </si>
   <si>
-    <t>5db46bd053c62492630b400c951c4fcd</t>
+    <t>95e1a614cdfbd2a8d2c896661f8ff941</t>
   </si>
   <si>
     <t>915-150011TM</t>
@@ -1748,7 +1748,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>ec31ff71890046b6c689412fc8a5de93</t>
+    <t>e99988527355cbe730e910fcba21b36f</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -1757,7 +1757,7 @@
     <t>01-010049TC</t>
   </si>
   <si>
-    <t>79963f24d68992368b951a0353a5642a</t>
+    <t>c37f9236ae8bf9419cfa7b5180839bf1</t>
   </si>
   <si>
     <t>01-010049TP</t>
@@ -1919,7 +1919,7 @@
     <t>01-010027TC</t>
   </si>
   <si>
-    <t>87e8c430e558ed6fc9241eb747e607aa</t>
+    <t>a5e1c5debee191457ca0a63099855e7c</t>
   </si>
   <si>
     <t>01-010027TP</t>
@@ -1940,7 +1940,7 @@
     <t>05-050005TP</t>
   </si>
   <si>
-    <t>069541344b050b6681eb7d7cc643fe18</t>
+    <t>ba132923527289319bb034912b3eb36a</t>
   </si>
   <si>
     <t>905-9050607-905060702A</t>
@@ -1964,7 +1964,7 @@
     <t>05-050201TP</t>
   </si>
   <si>
-    <t>524c3dd1e30ccfe1fb367287c0f6866e</t>
+    <t>f03c28b2cf4a83870b6dd5ad89866096</t>
   </si>
   <si>
     <t>05-0709-070902TM</t>
@@ -1985,7 +1985,7 @@
     <t>04-040018TC</t>
   </si>
   <si>
-    <t>158f05bbf80516fbeed41b7f46e86a88</t>
+    <t>397b8c6c2654603522232cb990001b09</t>
   </si>
   <si>
     <t>04-040018TM</t>
@@ -2036,7 +2036,7 @@
     <t>02-020001TC</t>
   </si>
   <si>
-    <t>f8a26f15e725de2ffad7fd398e4ebc36</t>
+    <t>a3a6fe55e3f6f9e3d46c8ff4965fd34c</t>
   </si>
   <si>
     <t>01-010016TP</t>
@@ -2102,7 +2102,7 @@
     <t>01-010080TC</t>
   </si>
   <si>
-    <t>400adca321e5daa663f0578481c6845f</t>
+    <t>3c41f82f3e010fe9fe4898bc7db48f97</t>
   </si>
   <si>
     <t>05-0709-070910A</t>
@@ -2168,7 +2168,7 @@
     <t>915-150002TC</t>
   </si>
   <si>
-    <t>4dd7776ba6aa9646b072298ff0fa82c1</t>
+    <t>0aa4cbba2f274acda16f4e3eec9d0ff6</t>
   </si>
   <si>
     <t>02-020001TM</t>
@@ -2261,7 +2261,7 @@
     <t>01-010029TC</t>
   </si>
   <si>
-    <t>a6232cc167e916c3bae255a3aa1b496e</t>
+    <t>01d6fdbf11a886c6db79a70a71ffad9f</t>
   </si>
   <si>
     <t>01-010029TM</t>
@@ -2396,7 +2396,7 @@
     <t>05-050001TC</t>
   </si>
   <si>
-    <t>95faf70c272e0c86f38d79c662cfe83e</t>
+    <t>f7eaf721044041eebecaa083894a45c6</t>
   </si>
   <si>
     <t>05-0709-070954A</t>
@@ -2555,7 +2555,7 @@
     <t>01-010060TC</t>
   </si>
   <si>
-    <t>f9580f601c64e43754e2b01d440a4f65</t>
+    <t>74d9017b58b4d2914dcebf7ec5d73266</t>
   </si>
   <si>
     <t>03-02010301-030093TP</t>
@@ -2615,7 +2615,7 @@
     <t>05-050001TP</t>
   </si>
   <si>
-    <t>0b2c4cfd1491c32d7b87cbd27c329f74</t>
+    <t>0aba477b7b37c51d2efa5e65c5870083</t>
   </si>
   <si>
     <t>03-030039TP</t>
@@ -2699,13 +2699,13 @@
     <t>05-050204A</t>
   </si>
   <si>
-    <t>6824dcbff9b9b18470a696eafad3ed22</t>
+    <t>7c21ebbe20dea263f1ebd2f09f824a70</t>
   </si>
   <si>
     <t>05-050313A</t>
   </si>
   <si>
-    <t>ef1989b9ed4fe94a13257181ff2b5b2a</t>
+    <t>33d0d420a76120a64e95e94e7c546d53</t>
   </si>
   <si>
     <t>902-0204-02040102ATC</t>
@@ -2795,7 +2795,7 @@
     <t>01-010073TC</t>
   </si>
   <si>
-    <t>ce42756ec01c0727aec21745a7bd1769</t>
+    <t>7273dd18ea2d0472e20312f9d9d23ba4</t>
   </si>
   <si>
     <t>901-010202-9010102021TM</t>
@@ -2804,7 +2804,7 @@
     <t>05-050205A</t>
   </si>
   <si>
-    <t>6cac8ff44d664cecbac54fc326f40181</t>
+    <t>58356809d72ffefc470fc0164cf01ff5</t>
   </si>
   <si>
     <t>04-040011TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>09fc7fc3756e43d07691bb5adbe24dc9</t>
+    <t>eb50b670dc742668e3dada6536b130bc</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2837,7 +2837,7 @@
     <t>03-030001TC</t>
   </si>
   <si>
-    <t>89da1243052404e75116934c786c8225</t>
+    <t>f58f65815269c5afaa912035c8625920</t>
   </si>
   <si>
     <t>03-030047TC</t>
@@ -2936,19 +2936,19 @@
     <t>05-050202A</t>
   </si>
   <si>
-    <t>57893c8170a1cc2ba69151ae3cf2baf6</t>
+    <t>05977562b4c05b5d1527002f554fd73a</t>
   </si>
   <si>
     <t>05-050311A</t>
   </si>
   <si>
-    <t>9d2e569c293a312882f4ae50f8ac2487</t>
+    <t>ee0bde4b723d1164531c1d381f0aab89</t>
   </si>
   <si>
     <t>05-050208TP</t>
   </si>
   <si>
-    <t>55e9ed5eed7c904073f06c23be8acf3b</t>
+    <t>aa2c863d3ecbde6df78a75cf91ddb509</t>
   </si>
   <si>
     <t>901-010202-9010102022A</t>
@@ -2975,19 +2975,19 @@
     <t>05-050306TP</t>
   </si>
   <si>
-    <t>bd4fe69c8947ef041f3002f71a088484</t>
+    <t>d05da657f7e7ec85e9ff27cad2a4820b</t>
   </si>
   <si>
     <t>905-9050607-905060701TC</t>
   </si>
   <si>
-    <t>caf0902acd5e4ab007abd4dbb31c1a66</t>
+    <t>a57ceca9b27525da70f92d48f68d5642</t>
   </si>
   <si>
     <t>01-010062TC</t>
   </si>
   <si>
-    <t>28c1e62731b3ff5e91de50f954dcae07</t>
+    <t>07ce20735bf4be24a833e4e0a3178069</t>
   </si>
   <si>
     <t>01-010020A</t>
@@ -3029,13 +3029,13 @@
     <t>05-050009A</t>
   </si>
   <si>
-    <t>16d892eb89e3b8eccd413ed0fdc2e295</t>
+    <t>93e11c66f816abbd324f415218325bc0</t>
   </si>
   <si>
     <t>05-050203A</t>
   </si>
   <si>
-    <t>4ba3200a8ee5e1bd77d51166edc4cea4</t>
+    <t>ed36a7e39502cdb47c4ca66b6eed9d4b</t>
   </si>
   <si>
     <t>01-080101-010087TM</t>
@@ -3080,13 +3080,13 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>3b4e5365c34d2a75f2016c13abd0727b</t>
+    <t>39f4468e10e88b41f2675073ed9de088</t>
   </si>
   <si>
     <t>01-010051TC</t>
   </si>
   <si>
-    <t>af76f2ed1d9e6a7b1e2f4cafa4d6403d</t>
+    <t>af297f7a4f45a52c3c7afab209bea1b1</t>
   </si>
   <si>
     <t>03-02010301-030090TC</t>
@@ -3140,7 +3140,7 @@
     <t>05-050006A</t>
   </si>
   <si>
-    <t>94f5b8ddba84c7717ca6ae7a704cbe5f</t>
+    <t>1f24233dc594be7264afc022937a0800</t>
   </si>
   <si>
     <t>01-080101-010078TM</t>
@@ -3167,7 +3167,7 @@
     <t>01-010040TC</t>
   </si>
   <si>
-    <t>33984657101d7559c4433ab3e9c69b06</t>
+    <t>2f7431be990d665c53b4ff7b709db313</t>
   </si>
   <si>
     <t>01-010064TP</t>
@@ -3212,7 +3212,7 @@
     <t>05-050201A</t>
   </si>
   <si>
-    <t>2f5b356fa3b756c42ddc16fde5069490</t>
+    <t>a80f038d8cfecc0df7f274164f8a60f7</t>
   </si>
   <si>
     <t>04-040020TC</t>
@@ -3230,7 +3230,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>09f3d1a7411ff0ee3ed0fc08be92ca1f</t>
+    <t>81f0c8cd3d187ea52d71d83db99f95fb</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3248,7 +3248,7 @@
     <t>05-050007A</t>
   </si>
   <si>
-    <t>19b5e71c9abcccb9dde06f9fd113f1fa</t>
+    <t>20a1388cf9de6965be77ff07dd97a122</t>
   </si>
   <si>
     <t>03-030036A</t>
@@ -3311,7 +3311,7 @@
     <t>02-020002TC</t>
   </si>
   <si>
-    <t>f867a3e9ecb30848290227f8d455fee5</t>
+    <t>5c5e35aed08a3d086a48f4f171592d65</t>
   </si>
   <si>
     <t>03-030047TP</t>
@@ -3323,7 +3323,7 @@
     <t>05-050004A</t>
   </si>
   <si>
-    <t>2f4b69fbba4eb28d2af56a95aeac2216</t>
+    <t>44242efb22128d3a88796703eab9602e</t>
   </si>
   <si>
     <t>03-030001TP</t>
@@ -3359,7 +3359,7 @@
     <t>05-050308TP</t>
   </si>
   <si>
-    <t>e33003a15fe254e9974c06ed62bd2b9b</t>
+    <t>98b69dd42783217b5cbe88d5d3c103cb</t>
   </si>
   <si>
     <t>03-030035A</t>
@@ -3371,7 +3371,7 @@
     <t>01-010064TC</t>
   </si>
   <si>
-    <t>219884d96e5e2d599fe6aacfce0a7c72</t>
+    <t>0e7967f7ab2da490734524e6ce918ca5</t>
   </si>
   <si>
     <t>01-010064A</t>
@@ -3431,7 +3431,7 @@
     <t>05-050005A</t>
   </si>
   <si>
-    <t>679d6517ecd875770c5ac30ac133f5fc</t>
+    <t>2189bc4d6abee13bad9f542a1a14a829</t>
   </si>
   <si>
     <t>01-080101-010089TM</t>
@@ -3461,7 +3461,7 @@
     <t>01-010053TC</t>
   </si>
   <si>
-    <t>c22701c86202094093123c72a9ea3d4e</t>
+    <t>ce33d570abeee5a9cd940ce31b302fb4</t>
   </si>
   <si>
     <t>02-020002TP</t>
@@ -3542,7 +3542,7 @@
     <t>01-010042TC</t>
   </si>
   <si>
-    <t>922fbfeb06bc04374c9b8582e84c655d</t>
+    <t>1ddc0da42fd673e0682c36473ecc44c1</t>
   </si>
   <si>
     <t>03-030032TC</t>
@@ -3611,7 +3611,7 @@
     <t>05-050204TP</t>
   </si>
   <si>
-    <t>4d04e450dbd4294233557cbf3c065cd9</t>
+    <t>8e692fc544336d1fb0f8b5da2d88fbf6</t>
   </si>
   <si>
     <t>915-150007A</t>
@@ -3632,7 +3632,7 @@
     <t>04-040015TC</t>
   </si>
   <si>
-    <t>9003d4027669b089f69fad61020b5dbb</t>
+    <t>e18167b7efe7103366235ffa0a05980b</t>
   </si>
   <si>
     <t>04-040011A</t>
@@ -3659,7 +3659,7 @@
     <t>01-010031TC</t>
   </si>
   <si>
-    <t>f3734af33378b52b93260ea478c568b3</t>
+    <t>ec2da7937cb92195d14d9fbf9586f1ae</t>
   </si>
   <si>
     <t>03-02010301-030088TP</t>
@@ -3686,7 +3686,7 @@
     <t>05-050302TP</t>
   </si>
   <si>
-    <t>333380440a79efa207e42ccdee6e6a24</t>
+    <t>d86adf49211f901bde4b1d1f6fc31558</t>
   </si>
   <si>
     <t>01-010055TM</t>
@@ -3779,7 +3779,7 @@
     <t>01-010020TC</t>
   </si>
   <si>
-    <t>1d340445f3fed20651d925e12c8777a9</t>
+    <t>6b3966e3d0309afa5c3ba6d1f6f7e28c</t>
   </si>
   <si>
     <t>01-010044TM</t>
@@ -3791,7 +3791,7 @@
     <t>05-050313TP</t>
   </si>
   <si>
-    <t>711b52eb3bff41710ab4da4b34e82eaa</t>
+    <t>612bef7dff576939e9b8a6539bb569bc</t>
   </si>
   <si>
     <t>01-010004A</t>
@@ -3827,7 +3827,7 @@
     <t>05-050313TC</t>
   </si>
   <si>
-    <t>a0434bd934177faeff6d69a08937a7f0</t>
+    <t>65c557c9cf8fe405060f7f6a563c0b59</t>
   </si>
   <si>
     <t>01-010028A</t>
@@ -3842,7 +3842,7 @@
     <t>01-010055TC</t>
   </si>
   <si>
-    <t>06b4f99a0d6d70febcac4b6069121bf0</t>
+    <t>1da53f5aca2c1caad2cd2d83bb8465e6</t>
   </si>
   <si>
     <t>915-150005A</t>
@@ -3881,13 +3881,13 @@
     <t>05-050208A</t>
   </si>
   <si>
-    <t>750f724609df41ec244169e2573685e3</t>
+    <t>4e695cbfd3223686785cfcc63e5dd99b</t>
   </si>
   <si>
     <t>05-050317A</t>
   </si>
   <si>
-    <t>d6efa44b50598db7e91db8daa4b737e1</t>
+    <t>913aa4a2ea682840f52159f3c0a0a804</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -3899,7 +3899,7 @@
     <t>01-010044TC</t>
   </si>
   <si>
-    <t>9278a4a1430b547281cd58135bacac87</t>
+    <t>975d50a5bec35861a8ecd04ad6ccf832</t>
   </si>
   <si>
     <t>03-02010301-030079TP</t>
@@ -3998,7 +3998,7 @@
     <t>01-010079TC</t>
   </si>
   <si>
-    <t>65e90394f770266f23a5fc80aef1f658</t>
+    <t>9abf1aa93f3ff10242f9a86551d6a858</t>
   </si>
   <si>
     <t>05-050206TC</t>
@@ -4070,7 +4070,7 @@
     <t>04-040013TC</t>
   </si>
   <si>
-    <t>5d36b099269766af24b39475fff3e8e3</t>
+    <t>1243fa26e01329027180388dd1b0289d</t>
   </si>
   <si>
     <t>01-010011TP</t>
@@ -4109,7 +4109,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>5369912adaba6ec20b0b0ee581b31e15</t>
+    <t>545cacbf13eb845375ce83083adf4e0c</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -4124,7 +4124,7 @@
     <t>01-010022TC</t>
   </si>
   <si>
-    <t>e9d235c08e4c1c94c33f933f84de5cef</t>
+    <t>a6b99c7eed41a06734d08e737d475ff7</t>
   </si>
   <si>
     <t>01-010049A</t>
@@ -4244,7 +4244,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>42ce0f8056c3dd390f5b7b8147ad97a9</t>
+    <t>d58fc751ffe20b31f4b20d9085871dc5</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -4253,7 +4253,7 @@
     <t>02-020006TC</t>
   </si>
   <si>
-    <t>0f40f04bcc621925417d19dedb02c9eb</t>
+    <t>467f209ca2b5c20d5e613ec01cee52cb</t>
   </si>
   <si>
     <t>05-0709-070921ATC</t>
@@ -4286,7 +4286,7 @@
     <t>01-010057TC</t>
   </si>
   <si>
-    <t>fb9514e813d953806bfa170157b69ea1</t>
+    <t>91dad7cac7dbcc47d8c7b74c86114978</t>
   </si>
   <si>
     <t>05-0709-070905BA</t>
@@ -4316,7 +4316,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>5a982386af55a6d742729e620d1c811f</t>
+    <t>8d45ae5a7d1cc9152872d86dd09672db</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4376,7 +4376,7 @@
     <t>01-010046TC</t>
   </si>
   <si>
-    <t>55122c292562b9a9e9b912dbd618d9af</t>
+    <t>4b282219d57e46615e1c6d9f7eba3a81</t>
   </si>
   <si>
     <t>01-080101-010113TP</t>
@@ -4400,7 +4400,7 @@
     <t>05-050004TC</t>
   </si>
   <si>
-    <t>dd19106b6296b94fbe2beff96f8b6904</t>
+    <t>6fadf3f1addc0f5ba00a643a180d7406</t>
   </si>
   <si>
     <t>04-040019TP</t>
@@ -4433,7 +4433,7 @@
     <t>05-050004TP</t>
   </si>
   <si>
-    <t>a87fa5e1dd60653b4706263526353b54</t>
+    <t>0166105de3083aae37fa0c88250860d5</t>
   </si>
   <si>
     <t>03-030072A</t>
@@ -4457,7 +4457,7 @@
     <t>01-010035TC</t>
   </si>
   <si>
-    <t>535b9101700329efe947e9ed77b67f67</t>
+    <t>2c617b0f9c9cd2780353304415acd131</t>
   </si>
   <si>
     <t>03-02010301-030097A</t>
@@ -4475,7 +4475,7 @@
     <t>05-050102TP</t>
   </si>
   <si>
-    <t>cc857f2f548c99e88ad33c1a942ab4bf</t>
+    <t>0b460618bbe807b3439c9a552f50d8ed</t>
   </si>
   <si>
     <t>03-030062TC</t>
@@ -4499,7 +4499,7 @@
     <t>01-010059TC</t>
   </si>
   <si>
-    <t>febbf4b45684b453483d13f9fa5d9f24</t>
+    <t>e5d1b2d0723df11bf62d826a4fef8bb2</t>
   </si>
   <si>
     <t>01-010059TP</t>
@@ -4571,7 +4571,7 @@
     <t>01-010024TC</t>
   </si>
   <si>
-    <t>e3bec460f39ee5e68962b87012822b80</t>
+    <t>77b5a19feb93b387baaf2223e175b251</t>
   </si>
   <si>
     <t>03-030075TC</t>
@@ -4583,7 +4583,7 @@
     <t>05-050002TC</t>
   </si>
   <si>
-    <t>292ac7fc92e0b9bcb8b8e74b63cdd9a3</t>
+    <t>cc40c7e733531e57fe509499d7cc5eb5</t>
   </si>
   <si>
     <t>03-030075TP</t>
@@ -4601,7 +4601,7 @@
     <t>01-010048TC</t>
   </si>
   <si>
-    <t>92d4fb4c45fdc2f1ceadbf8a59d11320</t>
+    <t>1d86b1da6b671f5a86b4d997ec9bdac4</t>
   </si>
   <si>
     <t>01-010048TP</t>
@@ -4679,7 +4679,7 @@
     <t>01-010037TC</t>
   </si>
   <si>
-    <t>3649d94c57036f9902258b739df13e97</t>
+    <t>b5f488dd71cdbc226bccc5607122d7b4</t>
   </si>
   <si>
     <t>03-90205-0205_006TP</t>
@@ -4721,13 +4721,13 @@
     <t>05-050006TC</t>
   </si>
   <si>
-    <t>b2f1e95cc57ece153fcab2833bd7da1a</t>
+    <t>2530afd01d1f20c8f3f886acd962f92c</t>
   </si>
   <si>
     <t>01-010026TC</t>
   </si>
   <si>
-    <t>f1fa2b661f8f8bf382410faa09bb2d51</t>
+    <t>a9795616dff196cbdab88357545c21e0</t>
   </si>
   <si>
     <t>01-010026TP</t>
@@ -4745,7 +4745,7 @@
     <t>05-050006TP</t>
   </si>
   <si>
-    <t>a2992dd83e22bc7f15c931e5f1ee4853</t>
+    <t>66d052724af6b3c4794988bf0fb92f7f</t>
   </si>
   <si>
     <t>05-050006TM</t>
@@ -4754,7 +4754,7 @@
     <t>05-050104TC</t>
   </si>
   <si>
-    <t>2e91159c4e9e881bcad80bfed883f9c0</t>
+    <t>3d8d915dd15670f42b12f8e683c77ac8</t>
   </si>
   <si>
     <t>03-030060TC</t>
@@ -4772,7 +4772,7 @@
     <t>05-050202TP</t>
   </si>
   <si>
-    <t>baedf182ad6a81af57d78f57524c4106</t>
+    <t>a870064fe7e8a4e6403424cc7fce98b9</t>
   </si>
   <si>
     <t>05-0709-070903TM</t>
@@ -4793,7 +4793,7 @@
     <t>04-040017TC</t>
   </si>
   <si>
-    <t>32299571fb6c160a7fbf6649f1403d62</t>
+    <t>b4ec90c902e7322edd357882b681a10e</t>
   </si>
   <si>
     <t>05-0709-070903TP</t>
@@ -4811,7 +4811,7 @@
     <t>05-050104TM</t>
   </si>
   <si>
-    <t>71ded6a4fe3b064d64c4dadf702fa436</t>
+    <t>cce98ab42191124a1792493f2f90ff09</t>
   </si>
   <si>
     <t>04-040017TP</t>
@@ -4823,7 +4823,7 @@
     <t>05-050104TP</t>
   </si>
   <si>
-    <t>7f3583297e5bf75d0fc5cb0aef60b0a8</t>
+    <t>7c82cd98151ed57d729e7aadd228619a</t>
   </si>
   <si>
     <t>05-050202TC</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>f7ace73729e01af1ea1690b5b3e48612</t>
+    <t>c6ad7b47b2550cf8bda2f1e65676dc31</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4862,7 +4862,7 @@
     <t>915-150012TC</t>
   </si>
   <si>
-    <t>a3b98661bba10de86905304ca5f76fb3</t>
+    <t>f855bb8e68496f2f991e34b25fbb11f5</t>
   </si>
   <si>
     <t>03-02010301-030092A</t>
@@ -4892,7 +4892,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>4766dbefc02fb27e78e178e1f5fdfab7</t>
+    <t>370aeef215fed2ad3cbc5dfb14a31a4a</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -4991,7 +4991,7 @@
     <t>01-010039TC</t>
   </si>
   <si>
-    <t>09a430c663def7edf284235b0d082c8e</t>
+    <t>c6757f11a1c5b578c44dc26987cbc2ca</t>
   </si>
   <si>
     <t>03-030029TC</t>
@@ -5003,13 +5003,13 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>188b27af421fe22a0e14d932b7ee19c6</t>
+    <t>605b9f3512f220f09dd6af9a72c8e40e</t>
   </si>
   <si>
     <t>05-050002A</t>
   </si>
   <si>
-    <t>859448e77e2bc8ddc6531a8347e170c6</t>
+    <t>27e9973bd61c838ee344b1f8528b80f0</t>
   </si>
   <si>
     <t>01-010039TM</t>
@@ -5051,7 +5051,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>09b39441b0843889e708999649d8efb6</t>
+    <t>f61df9d2bfd0790d8760e0d94db684ca</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5438,7 +5438,7 @@
     <t>05-050002TP</t>
   </si>
   <si>
-    <t>a8520a0ba8fb4cc190e727b6f3675bbf</t>
+    <t>6beb1d7067457e82d63450a254c76143</t>
   </si>
   <si>
     <t>05-050002TM</t>
@@ -5486,7 +5486,7 @@
     <t>01-010019TC</t>
   </si>
   <si>
-    <t>7be66c7c33b13ed501cc9342c752ac2d</t>
+    <t>eb6073eca18fe7f49d37c1a3ab31bc1b</t>
   </si>
   <si>
     <t>915-150016TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie mar  3 23:50:08 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5294,7 +5294,7 @@
     <t>05-050001A</t>
   </si>
   <si>
-    <t>275b0dde819612dc7c9f67d79ddafb61</t>
+    <t>0f86d691fe0e305e63b54acceec12cf4</t>
   </si>
   <si>
     <t>01-010006TM</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb mar  4 23:24:48 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -872,7 +872,7 @@
     <t>01-010017A</t>
   </si>
   <si>
-    <t>8c426e7290c4d1f01eeb3fbf2ba62f3e</t>
+    <t>94e3bdce9575af42f713c012e310963c</t>
   </si>
   <si>
     <t>03-030033TC</t>
@@ -2585,7 +2585,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>6f604c66bf55c7354d0b02b41b484b06</t>
+    <t>132cb2ce7322a45f69527701ed8a4d23</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -5468,7 +5468,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
+    <t>49e6a091e08e2fc592046231facaf4a0</t>
   </si>
   <si>
     <t>02-020005A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar mar  7 23:55:00 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -209,7 +209,7 @@
     <t>05-050316TP</t>
   </si>
   <si>
-    <t>472edfaa05e1207d58533aec747cc1a0</t>
+    <t>ed14180819c284197d20ad343158e414</t>
   </si>
   <si>
     <t>915-150018TP</t>
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -737,7 +737,7 @@
     <t>05-050309A</t>
   </si>
   <si>
-    <t>c36cfa08576bd03193194588c36f0f45</t>
+    <t>898c927755a34ac05f8c7723ed95e017</t>
   </si>
   <si>
     <t>04-040003TP</t>
@@ -872,7 +872,7 @@
     <t>01-010017A</t>
   </si>
   <si>
-    <t>94e3bdce9575af42f713c012e310963c</t>
+    <t>8c426e7290c4d1f01eeb3fbf2ba62f3e</t>
   </si>
   <si>
     <t>03-030033TC</t>
@@ -1106,7 +1106,7 @@
     <t>05-050314TP</t>
   </si>
   <si>
-    <t>76194b402ea30878c498724d6f3da001</t>
+    <t>f556688e7c184cea3fbcc1296de65237</t>
   </si>
   <si>
     <t>902-0204-02040102STC</t>
@@ -1145,7 +1145,7 @@
     <t>05-050314TC</t>
   </si>
   <si>
-    <t>26e8df35c47b1349b814821cfaf34b26</t>
+    <t>d0679f82249a3d2a4afbdb723a3c3c29</t>
   </si>
   <si>
     <t>902-0204-02040101ATC</t>
@@ -1748,7 +1748,7 @@
     <t>05-050310TP</t>
   </si>
   <si>
-    <t>e99988527355cbe730e910fcba21b36f</t>
+    <t>abc6a9f439321b777358262fe0c585a3</t>
   </si>
   <si>
     <t>03-030072TM</t>
@@ -2585,7 +2585,7 @@
     <t>03-030063A</t>
   </si>
   <si>
-    <t>132cb2ce7322a45f69527701ed8a4d23</t>
+    <t>6f604c66bf55c7354d0b02b41b484b06</t>
   </si>
   <si>
     <t>05-050001TM</t>
@@ -2816,7 +2816,7 @@
     <t>05-050314A</t>
   </si>
   <si>
-    <t>eb50b670dc742668e3dada6536b130bc</t>
+    <t>6277dbfc0e4fef5f0d55e00c7a814284</t>
   </si>
   <si>
     <t>901-010202-9010102021TP</t>
@@ -2942,7 +2942,7 @@
     <t>05-050311A</t>
   </si>
   <si>
-    <t>ee0bde4b723d1164531c1d381f0aab89</t>
+    <t>78b5cd2da4de5c5320693b5a55be5285</t>
   </si>
   <si>
     <t>05-050208TP</t>
@@ -3080,7 +3080,7 @@
     <t>05-050317TP</t>
   </si>
   <si>
-    <t>39f4468e10e88b41f2675073ed9de088</t>
+    <t>a0e522c2f72add2761f00d3dee8dbdfe</t>
   </si>
   <si>
     <t>01-010051TC</t>
@@ -3230,7 +3230,7 @@
     <t>05-050310A</t>
   </si>
   <si>
-    <t>81f0c8cd3d187ea52d71d83db99f95fb</t>
+    <t>0235701fedac7f47de60cac57b9e0abc</t>
   </si>
   <si>
     <t>915-150008TP</t>
@@ -3887,7 +3887,7 @@
     <t>05-050317A</t>
   </si>
   <si>
-    <t>913aa4a2ea682840f52159f3c0a0a804</t>
+    <t>ca877e39b3cdcbe2ac8b481a7f50baee</t>
   </si>
   <si>
     <t>01-010027A</t>
@@ -4109,7 +4109,7 @@
     <t>05-050315A</t>
   </si>
   <si>
-    <t>545cacbf13eb845375ce83083adf4e0c</t>
+    <t>6d527480c3030876ffbd199c9392d4c6</t>
   </si>
   <si>
     <t>902-0204-02040101STP</t>
@@ -4244,7 +4244,7 @@
     <t>05-050316A</t>
   </si>
   <si>
-    <t>d58fc751ffe20b31f4b20d9085871dc5</t>
+    <t>0a217a8176afd26150f48189e0f5deb4</t>
   </si>
   <si>
     <t>902-0204-02040101BTC</t>
@@ -4316,7 +4316,7 @@
     <t>05-050315TP</t>
   </si>
   <si>
-    <t>8d45ae5a7d1cc9152872d86dd09672db</t>
+    <t>33d02fdb5c950c58dec4942b15e19d93</t>
   </si>
   <si>
     <t>03-030040TP</t>
@@ -4850,7 +4850,7 @@
     <t>05-050311TC</t>
   </si>
   <si>
-    <t>c6ad7b47b2550cf8bda2f1e65676dc31</t>
+    <t>f86ad6e2eb81932138659729531919be</t>
   </si>
   <si>
     <t>04-040014A</t>
@@ -4892,7 +4892,7 @@
     <t>05-050311TP</t>
   </si>
   <si>
-    <t>370aeef215fed2ad3cbc5dfb14a31a4a</t>
+    <t>72886969a8868b29362acc4437302d76</t>
   </si>
   <si>
     <t>01-080101-010081TC</t>
@@ -5003,7 +5003,7 @@
     <t>05-050309TC</t>
   </si>
   <si>
-    <t>605b9f3512f220f09dd6af9a72c8e40e</t>
+    <t>33bb755ed4e50b970d31c18c0233f31c</t>
   </si>
   <si>
     <t>05-050002A</t>
@@ -5051,7 +5051,7 @@
     <t>05-050309TP</t>
   </si>
   <si>
-    <t>f61df9d2bfd0790d8760e0d94db684ca</t>
+    <t>9b657b1f49de90c890f8f5db1c5c7c1b</t>
   </si>
   <si>
     <t>05-050309TM</t>
@@ -5468,7 +5468,7 @@
     <t>03-030052A</t>
   </si>
   <si>
-    <t>49e6a091e08e2fc592046231facaf4a0</t>
+    <t>fd5080f03fc5914f0fe5ee68f0ef06e6</t>
   </si>
   <si>
     <t>02-020005A</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode sáb mar 11 00:09:57 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -257,7 +257,7 @@
     <t>05-0709-070908TC</t>
   </si>
   <si>
-    <t>e7280369bec73f344ac204675f3ed28c</t>
+    <t>b430bc9311c1d50b84788148cae3dc74</t>
   </si>
   <si>
     <t>05-050105A</t>
@@ -338,7 +338,7 @@
     <t>05-0709-070908TM</t>
   </si>
   <si>
-    <t>b09ab385410ab6519f2c5c01b0d8e8d4</t>
+    <t>ff9e9cc58fbd5e02008c7efa8e69326a</t>
   </si>
   <si>
     <t>03-030026A</t>
@@ -356,7 +356,7 @@
     <t>05-0709-070908TP</t>
   </si>
   <si>
-    <t>aec1b3939c8038a5e89e2c291a3f4e97</t>
+    <t>805961b0758545dcaffa68751e5804c3</t>
   </si>
   <si>
     <t>03-030002A</t>
@@ -488,7 +488,7 @@
     <t>05-0709-070952TC</t>
   </si>
   <si>
-    <t>8dddd0fd620bce146d55133f82e739e5</t>
+    <t>af112e30953020cc3a562bbb5664194b</t>
   </si>
   <si>
     <t>01-010041TM</t>
@@ -506,7 +506,7 @@
     <t>05-0709-070952TP</t>
   </si>
   <si>
-    <t>96e9549a1a76078106d55f3b6f03ae51</t>
+    <t>57abc69702aca968e636cd82d11100fb</t>
   </si>
   <si>
     <t>03-030057TP</t>
@@ -518,7 +518,7 @@
     <t>05-0709-070952TM</t>
   </si>
   <si>
-    <t>2e98ae1fbd37482b4bb718204ba65ab6</t>
+    <t>a90a924948cef116497ba896c7a1bc14</t>
   </si>
   <si>
     <t>05-050104A</t>
@@ -779,7 +779,7 @@
     <t>05-0709-070954TC</t>
   </si>
   <si>
-    <t>672e231ce856a7699d969f2f02ad1fe5</t>
+    <t>be5b79cd60655934990838fa8ab74c72</t>
   </si>
   <si>
     <t>04-040003TC</t>
@@ -857,7 +857,7 @@
     <t>05-0709-070954TP</t>
   </si>
   <si>
-    <t>200ccbd2f6a1307fb9201573cfa06429</t>
+    <t>daf139f841c831f917d5de6b476497d5</t>
   </si>
   <si>
     <t>01-080101-010079TM</t>
@@ -1079,7 +1079,7 @@
     <t>05-0709-070906AA</t>
   </si>
   <si>
-    <t>2036bb49d693ba503f6b90238e04c6e8</t>
+    <t>8ea2b10c7927775ae28bcac72567fd1b</t>
   </si>
   <si>
     <t>01-010067TC</t>
@@ -1127,13 +1127,13 @@
     <t>05-0709-070910TC</t>
   </si>
   <si>
-    <t>3b13b77e1ba7650bd966fe990ef71644</t>
+    <t>3929274a6cd70cadf32afc573d91ca5b</t>
   </si>
   <si>
     <t>05-0709-070910TM</t>
   </si>
   <si>
-    <t>ae4025a4e458212368bd492f3e3f1b67</t>
+    <t>10cbe087ef2c2133a16c8f3780b646fb</t>
   </si>
   <si>
     <t>01-010045TP</t>
@@ -1229,7 +1229,7 @@
     <t>05-0709-070910TP</t>
   </si>
   <si>
-    <t>25bb6b8922786406c85e7f4e6793f028</t>
+    <t>a08c3ab3ca6a5c0e3257056440f58a01</t>
   </si>
   <si>
     <t>01-010045TC</t>
@@ -1835,7 +1835,7 @@
     <t>05-0709-070902TC</t>
   </si>
   <si>
-    <t>f7be0b1f684977c506f4fde0fe3e417a</t>
+    <t>4434e58e40eee7046d30b387dc46ae35</t>
   </si>
   <si>
     <t>03-02010301-030097TC</t>
@@ -1958,7 +1958,7 @@
     <t>05-0709-070902TP</t>
   </si>
   <si>
-    <t>066d89d3f1ea5c31ac232654fdea51a1</t>
+    <t>4abc0293f17b15bf72ddbf044ee1e0d4</t>
   </si>
   <si>
     <t>05-050201TP</t>
@@ -1970,7 +1970,7 @@
     <t>05-0709-070902TM</t>
   </si>
   <si>
-    <t>223e194bf733c3a005d4be1af189296e</t>
+    <t>7672b1cb00c29c230961203d1f950819</t>
   </si>
   <si>
     <t>915-150009A</t>
@@ -2015,7 +2015,7 @@
     <t>05-0709-070906ATC</t>
   </si>
   <si>
-    <t>451cdc8e7e60f577abc056f972a86f53</t>
+    <t>ad0afbb4973e433bfca4a9f1ba1faa34</t>
   </si>
   <si>
     <t>915-150013TP</t>
@@ -2066,7 +2066,7 @@
     <t>05-0709-070906ATM</t>
   </si>
   <si>
-    <t>41a860e496fa1c7c4b580ccce6b3de8e</t>
+    <t>877624356de5060abdde8dc79fdcdae7</t>
   </si>
   <si>
     <t>03-030070TC</t>
@@ -2078,7 +2078,7 @@
     <t>05-0709-070906ATP</t>
   </si>
   <si>
-    <t>c423b2fd0c22582aa89570a92b795b16</t>
+    <t>3155a2c696637d528b406714a0774ec2</t>
   </si>
   <si>
     <t>915-150013TC</t>
@@ -2108,7 +2108,7 @@
     <t>05-0709-070910A</t>
   </si>
   <si>
-    <t>95362085d86e2357363fb6a130d4808d</t>
+    <t>96beea3cb870dd02203b50cf7f327a3e</t>
   </si>
   <si>
     <t>01-010074A</t>
@@ -2222,7 +2222,7 @@
     <t>05-0709-070904TC</t>
   </si>
   <si>
-    <t>e9e0c9633698ab6f31af882f3aa87554</t>
+    <t>2496985d2b9f07d12400de7dfc9dbef1</t>
   </si>
   <si>
     <t>01-010073A</t>
@@ -2276,7 +2276,7 @@
     <t>05-0709-070904TM</t>
   </si>
   <si>
-    <t>6e38df94a15d4148e51554dbcd58600c</t>
+    <t>d6ab5069cb0628aca77e51b0d260417e</t>
   </si>
   <si>
     <t>01-010029TP</t>
@@ -2288,7 +2288,7 @@
     <t>05-0709-070904TP</t>
   </si>
   <si>
-    <t>601d6bc103483850ab7140071515f8da</t>
+    <t>4d36a78a3a99de8cba796174b38d7a7d</t>
   </si>
   <si>
     <t>03-030066A</t>
@@ -2306,7 +2306,7 @@
     <t>05-0709-070955A</t>
   </si>
   <si>
-    <t>e987cfc30c2fbcd90de9c06292b04601</t>
+    <t>9c4912532f5a97615efaec192b90c324</t>
   </si>
   <si>
     <t>915-150015TP</t>
@@ -2402,7 +2402,7 @@
     <t>05-0709-070954A</t>
   </si>
   <si>
-    <t>7d5c7dc8f623aebd7e22b44f194c3b80</t>
+    <t>5eeb862964e3ceb1f66a741b7b12eea8</t>
   </si>
   <si>
     <t>01-080101-010086TC</t>
@@ -2525,7 +2525,7 @@
     <t>05-0709-070953A</t>
   </si>
   <si>
-    <t>aeeec4b2d3d6d45258b75168146bf6db</t>
+    <t>7dcf30a05309fbcd1c9381d596d882e6</t>
   </si>
   <si>
     <t>03-030064A</t>
@@ -2573,7 +2573,7 @@
     <t>05-0709-070952A</t>
   </si>
   <si>
-    <t>a89d4798e177098e2141ef2bcb9c67d7</t>
+    <t>319e295bd7b92e35e77450ad471a8d07</t>
   </si>
   <si>
     <t>03-02010301-030088A</t>
@@ -2693,7 +2693,7 @@
     <t>05-0709-070909TC</t>
   </si>
   <si>
-    <t>8f8eae294fa42e1517163b922b5ae8c4</t>
+    <t>38ecc55cb0926db6946287849f723d5a</t>
   </si>
   <si>
     <t>05-050204A</t>
@@ -2825,7 +2825,7 @@
     <t>05-0709-070909TM</t>
   </si>
   <si>
-    <t>7ec6ac3224d80f978a7da37f3286e688</t>
+    <t>8dd219eb165ad5011958194ab64f7c0c</t>
   </si>
   <si>
     <t>01-010009TP</t>
@@ -2849,7 +2849,7 @@
     <t>05-0709-070909TP</t>
   </si>
   <si>
-    <t>6efcb93f76d3f7ed23f6a5d4dd2f147c</t>
+    <t>47afe3afe820bf1c078c14cdf3cf531a</t>
   </si>
   <si>
     <t>04-040011TP</t>
@@ -2969,7 +2969,7 @@
     <t>05-0709-070904A</t>
   </si>
   <si>
-    <t>c9edcfcb1038e192fb210f9a82a62141</t>
+    <t>ddfa692b790555e815bde49df8a53d2a</t>
   </si>
   <si>
     <t>05-050306TP</t>
@@ -3074,7 +3074,7 @@
     <t>05-0709-070903A</t>
   </si>
   <si>
-    <t>8eec6ffcef97e4d2bf963b50dc94cfa8</t>
+    <t>f8519589fd76f19bba31e68f6eb40ed2</t>
   </si>
   <si>
     <t>05-050317TP</t>
@@ -3158,7 +3158,7 @@
     <t>05-0709-070902A</t>
   </si>
   <si>
-    <t>58ccb35a244e1d5a7d9583fbcff414b1</t>
+    <t>4dfb066024eabe43a130e2b3c7e0349b</t>
   </si>
   <si>
     <t>03-030013A</t>
@@ -3260,7 +3260,7 @@
     <t>05-0709-070901A</t>
   </si>
   <si>
-    <t>979f049d9df98d1f708386b326bb16c4</t>
+    <t>c6c8eea7d38e4fc7e73dcc6cc7a1fe1e</t>
   </si>
   <si>
     <t>03-030012A</t>
@@ -3518,7 +3518,7 @@
     <t>05-0709-070955TP</t>
   </si>
   <si>
-    <t>30072928ba18de42643e147d855869dc</t>
+    <t>5cc1a7a0f2846d02a9a72f3dc5c1acdc</t>
   </si>
   <si>
     <t>03-02010301-030090A</t>
@@ -3809,13 +3809,13 @@
     <t>05-0709-070953TC</t>
   </si>
   <si>
-    <t>8bb2da2353fe098265ba073cf6d533f7</t>
+    <t>686b8812b626ecd5f109a6a553719369</t>
   </si>
   <si>
     <t>05-0709-070953TP</t>
   </si>
   <si>
-    <t>c3889a0449e0bab2160be2a250d2f6f2</t>
+    <t>9bc05c596089cc505ad05d044f7230e0</t>
   </si>
   <si>
     <t>03-030056TP</t>
@@ -3989,7 +3989,7 @@
     <t>05-0709-070909A</t>
   </si>
   <si>
-    <t>f64b266e8eaadc4e2e1e01f3f5d9a9e5</t>
+    <t>29f63327be51e85bd32573b50c56a197</t>
   </si>
   <si>
     <t>05-050206TM</t>
@@ -4118,7 +4118,7 @@
     <t>05-0709-070908A</t>
   </si>
   <si>
-    <t>60dd4bf4c2a0a853e9ee671012b01132</t>
+    <t>685dd58e08dbc244b2a664e41ed2f112</t>
   </si>
   <si>
     <t>01-010022TC</t>
@@ -4136,7 +4136,7 @@
     <t>05-0709-070905AA</t>
   </si>
   <si>
-    <t>2499dffb01c68114a99ea19c9dcd1faa</t>
+    <t>e8366321c9227a014c6318f6e28cdb16</t>
   </si>
   <si>
     <t>01-080101-010110TP</t>
@@ -4178,7 +4178,7 @@
     <t>05-0709-070955TC</t>
   </si>
   <si>
-    <t>e593bfc60934c54749f1a9e8804d63dc</t>
+    <t>05a1f39bab6807d2faadb6b63ed41433</t>
   </si>
   <si>
     <t>03-030054TM</t>
@@ -4190,7 +4190,7 @@
     <t>05-0709-070921ATP</t>
   </si>
   <si>
-    <t>4339094c037786953fa88297fefbed6e</t>
+    <t>fefa3adf0e5a9cc74cdce6415b355196</t>
   </si>
   <si>
     <t>01-010024A</t>
@@ -4259,7 +4259,7 @@
     <t>05-0709-070921ATC</t>
   </si>
   <si>
-    <t>c77e688dcb662b21bbe8030648b208a0</t>
+    <t>26c8cc738893d08c147adc1261c7b24d</t>
   </si>
   <si>
     <t>05-050207A</t>
@@ -4334,7 +4334,7 @@
     <t>05-0709-070901TC</t>
   </si>
   <si>
-    <t>269f229c212b2374e74688859011a13d</t>
+    <t>649aabf2bb9d163f7705588cfa3f1b05</t>
   </si>
   <si>
     <t>03-02010301-030096TC</t>
@@ -4346,7 +4346,7 @@
     <t>05-0709-070901TM</t>
   </si>
   <si>
-    <t>7478d81de6f52608ee2450848cb17f24</t>
+    <t>55aafd70336d9978b99cdd6b2d00dad5</t>
   </si>
   <si>
     <t>01-010035TP</t>
@@ -4451,7 +4451,7 @@
     <t>05-0709-070901TP</t>
   </si>
   <si>
-    <t>ec225dcc5f11ea0f240d0239b6d4bc16</t>
+    <t>9f9cb9c8ab207f68722688984ed180b3</t>
   </si>
   <si>
     <t>01-010035TC</t>
@@ -4673,7 +4673,7 @@
     <t>05-0709-070903TC</t>
   </si>
   <si>
-    <t>c1b6ecf546b927cb406f17ac71de9754</t>
+    <t>75de686895a8490d52b1a069749978d4</t>
   </si>
   <si>
     <t>01-010037TC</t>
@@ -4778,7 +4778,7 @@
     <t>05-0709-070903TM</t>
   </si>
   <si>
-    <t>298c528aeda213f18e28ab043ae8fbca</t>
+    <t>0917f648f48fb38719b2c308dff07ffd</t>
   </si>
   <si>
     <t>03-02010301-030093A</t>
@@ -4799,7 +4799,7 @@
     <t>05-0709-070903TP</t>
   </si>
   <si>
-    <t>50ed6d92f70752b191f8846ae1fe2cf9</t>
+    <t>87ee84b8a63480ee7b21fd6fec1cf4d7</t>
   </si>
   <si>
     <t>04-040017TM</t>
@@ -5264,7 +5264,7 @@
     <t>05-0709-070905ATC</t>
   </si>
   <si>
-    <t>32d21c245b8ce615a5ed3d800bb36348</t>
+    <t>41932e19428ef3bc9b4a1deefbb9ac39</t>
   </si>
   <si>
     <t>01-010006TC</t>
@@ -5342,7 +5342,7 @@
     <t>05-0709-070905ATP</t>
   </si>
   <si>
-    <t>3e858897f1ebce7138cacc3416a4c648</t>
+    <t>a97e51a0a4468b402ab7b3bc75adf207</t>
   </si>
   <si>
     <t>03-030018TP</t>
@@ -5396,7 +5396,7 @@
     <t>05-0709-070921AA</t>
   </si>
   <si>
-    <t>80c0ac0afae53c3b9d33dc6442967c45</t>
+    <t>45cf5026c62bc743845e2c79ba3321c6</t>
   </si>
   <si>
     <t>03-02010301-030094TP</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié mar 15 23:53:23 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode jue mar 16 23:51:47 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode vie mar 17 23:56:41 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1241,7 +1241,7 @@
     <t>03-030077TC</t>
   </si>
   <si>
-    <t>8c681427d8a8bdfef77fbf94f81522cf</t>
+    <t>e3cc4013164b376311e716e03c7ed342</t>
   </si>
   <si>
     <t>03-030031TC</t>
@@ -1253,7 +1253,7 @@
     <t>03-030077TM</t>
   </si>
   <si>
-    <t>0e7f38563522c7de665af7e994caed1b</t>
+    <t>00cb4be0fe0038cf76db55e227a3f8ae</t>
   </si>
   <si>
     <t>01-010023TM</t>
@@ -1295,7 +1295,7 @@
     <t>03-030077TP</t>
   </si>
   <si>
-    <t>1ca3db9d241f5bcccd2f63e40c270371</t>
+    <t>e0e2b685807f368bf08dfd6de70529c1</t>
   </si>
   <si>
     <t>01-010023TP</t>
@@ -3530,7 +3530,7 @@
     <t>03-030078TC</t>
   </si>
   <si>
-    <t>81cf198796557ca8b33bd82d4943e53c</t>
+    <t>03915bef5d883f17541998f446868ae5</t>
   </si>
   <si>
     <t>01-010007A</t>
@@ -3560,7 +3560,7 @@
     <t>03-030078TM</t>
   </si>
   <si>
-    <t>f3f83b5eb6fb296e2766341fbb4c0dbd</t>
+    <t>6835a407ec7c7b7cdbe1b3b085ad5b76</t>
   </si>
   <si>
     <t>01-010020TM</t>
@@ -3602,7 +3602,7 @@
     <t>03-030078TP</t>
   </si>
   <si>
-    <t>f36199d34c3f0d11ba28c925d89913d2</t>
+    <t>a2ebb05c9f0f90da0400145edd0c4d67</t>
   </si>
   <si>
     <t>01-110304-11030401TP</t>
@@ -3917,13 +3917,13 @@
     <t>03-030076TC</t>
   </si>
   <si>
-    <t>06d7e7a5cd07f02126e971aba46eabd9</t>
+    <t>e46ecbb6f5f2e7dacb1c576ac9b49f26</t>
   </si>
   <si>
     <t>03-030076TM</t>
   </si>
   <si>
-    <t>39de56a13264c369ba3c863ebba30c8e</t>
+    <t>86e4c30ffff9037486750767e8da2607</t>
   </si>
   <si>
     <t>01-010022TM</t>
@@ -3983,7 +3983,7 @@
     <t>03-030076TP</t>
   </si>
   <si>
-    <t>da57af880c80ea3d4159d755efcc4ca8</t>
+    <t>90990dd39354285ad22b74b681f92c77</t>
   </si>
   <si>
     <t>05-0709-070909A</t>
@@ -4577,7 +4577,7 @@
     <t>03-030075TC</t>
   </si>
   <si>
-    <t>b3798ef9ab5db9680bdc354b51881249</t>
+    <t>f4979590227dbeda95407b443df2103c</t>
   </si>
   <si>
     <t>05-050002TC</t>
@@ -4589,7 +4589,7 @@
     <t>03-030075TP</t>
   </si>
   <si>
-    <t>606f0e6a54262626e109684907854697</t>
+    <t>2f9ccc0ff697f22bcf6481781db33ac2</t>
   </si>
   <si>
     <t>03-030075TM</t>
@@ -5354,7 +5354,7 @@
     <t>03-030078A</t>
   </si>
   <si>
-    <t>83704c9f8b0c1146eaa105f460f4e997</t>
+    <t>3aee87fb09a096d0b3bfed309928ceb7</t>
   </si>
   <si>
     <t>03-02010301-030079A</t>
@@ -5420,7 +5420,7 @@
     <t>03-030077A</t>
   </si>
   <si>
-    <t>fd4ca97cb50e7f86a0dbc343b6cb7e49</t>
+    <t>07843cf8d34b4582f07c7d377afeaddf</t>
   </si>
   <si>
     <t>02-020006A</t>
@@ -5462,7 +5462,7 @@
     <t>03-030076A</t>
   </si>
   <si>
-    <t>c19cc7bc729c576d2518fb6e0d3d8d81</t>
+    <t>9e93ebeda11bc8dc2ec15522f5293143</t>
   </si>
   <si>
     <t>03-030052A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode dom mar 19 23:29:56 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>33f34cf581d8f6ba4abea235324ff213</t>
+    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>8b33d7c797daac5964040351a979ddc0</t>
+    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mar mar 21 00:12:17 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -425,7 +425,7 @@
     <t>03-030049A</t>
   </si>
   <si>
-    <t>3e64bc6cd3ad95b52b13a1b4251093f6</t>
+    <t>33f34cf581d8f6ba4abea235324ff213</t>
   </si>
   <si>
     <t>05-050307TC</t>
@@ -5615,7 +5615,7 @@
     <t>03-030050A</t>
   </si>
   <si>
-    <t>2111c0f12829eeaf4cb870e8a37dab17</t>
+    <t>8b33d7c797daac5964040351a979ddc0</t>
   </si>
   <si>
     <t>01-080101-010081A</t>

</xml_diff>

<commit_message>
Actualización automática hashcode mié mar 22 23:59:35 CET 2023
</commit_message>
<xml_diff>
--- a/data/metadata/hashcode.xlsx
+++ b/data/metadata/hashcode.xlsx
@@ -1520,7 +1520,7 @@
     <t>01-080101-010112TC</t>
   </si>
   <si>
-    <t>cffd45499a810de0f25ac3d2685385f7</t>
+    <t>d006b109bb014545c90f94033680364f</t>
   </si>
   <si>
     <t>01-010036TP</t>
@@ -4595,7 +4595,7 @@
     <t>03-030075TM</t>
   </si>
   <si>
-    <t>e6205dbae3c37da3fd09656e4beab3e7</t>
+    <t>5a8c3f960f6b83a1577d4941d0547bb4</t>
   </si>
   <si>
     <t>01-010048TC</t>

</xml_diff>